<commit_message>
Start of chapter 5
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="214">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -40,6 +40,9 @@
     <t xml:space="preserve">Next</t>
   </si>
   <si>
+    <t xml:space="preserve">Points</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dr. Glitchwell</t>
   </si>
   <si>
@@ -529,7 +532,7 @@
     <t xml:space="preserve">You will literally be the Stegware!</t>
   </si>
   <si>
-    <t xml:space="preserve">But be careful, if you get caught by their anti-malware and be put into quarantaine, you will never be able to get back to the real world. </t>
+    <t xml:space="preserve">But be careful, if you get caught by their anti-malware and be put into quarantine, you will never be able to get back to the real world. </t>
   </si>
   <si>
     <t xml:space="preserve">They used steganography on us! We will use steganography against them! </t>
@@ -581,6 +584,84 @@
   </si>
   <si>
     <t xml:space="preserve">Dr. Glitchwell, prepare the Pixinator and transfer ${name} to the computer world.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I am on my own now. My choices really matter now.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 1: get in. I am literally data on a computer now.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I need to make sure the anti-malware systems of SilentSpectra cannot find me. I will…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use cryptography -&gt; 503; Use steganography -&gt; 520</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Okay, I have decrypted myself and send an email to Agent T. with myself attached.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aegis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hello, the name is Aegis. I am the Intrusion Detection System for the SilentSpectra network.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You must bypass me to gain access.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I see you are an email, but something encrypted is attached. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I cannot guarantee that you have no means of harm, since I cannot read the encrypted data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Therefore you will be quarantined!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAME OVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The message within encrypted data is hidden, but the existence of it is not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to try phase 1 again?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes -&gt; 500; No -&gt; 650</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TODO card 650</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which of the following images shall I attach to the email to Agent T.?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image 1 -&gt; 521; Image 2 -&gt; 523; Image 3 -&gt; 524</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An image with a lot of different colours would have worked best, since there we can make use of that redundant information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">But I will try this image anyway.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This image will fit our needs perfectly!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A bigger image can contain more data. It is hard to hide myself in here without altering the visibility of the image.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Now that I got an image, I need to hide myself in it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where in the image should I hide?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At the start of the file -&gt; 0; At the end of the file -&gt; 0; Replace the most significant bits by me -&gt; 0; Replace the least significant bits by me -&gt; 0</t>
   </si>
 </sst>
 </file>
@@ -706,7 +787,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -773,6 +854,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1023,7 +1108,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.14"/>
@@ -1053,19 +1138,22 @@
       <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
         <v>100</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="8" t="n">
@@ -1077,16 +1165,16 @@
         <v>101</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1094,13 +1182,13 @@
         <v>102</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="8" t="n">
@@ -1112,16 +1200,16 @@
         <v>103</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1129,13 +1217,13 @@
         <v>104</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="11" t="n">
@@ -1147,13 +1235,13 @@
         <v>105</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="11" t="n">
@@ -1165,13 +1253,13 @@
         <v>106</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="8" t="n">
@@ -1183,13 +1271,13 @@
         <v>107</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="8" t="n">
@@ -1201,16 +1289,16 @@
         <v>108</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1218,13 +1306,13 @@
         <v>110</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="11" t="n">
@@ -1236,13 +1324,13 @@
         <v>120</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="11" t="n">
@@ -1254,13 +1342,13 @@
         <v>130</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="8" t="n">
@@ -1272,13 +1360,13 @@
         <v>131</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="8" t="n">
@@ -1290,13 +1378,13 @@
         <v>132</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="8" t="n">
@@ -1308,13 +1396,13 @@
         <v>133</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" s="13"/>
       <c r="F16" s="8" t="n">
@@ -1326,13 +1414,13 @@
         <v>134</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E17" s="13"/>
       <c r="F17" s="8" t="n">
@@ -1344,13 +1432,13 @@
         <v>135</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E18" s="13"/>
       <c r="F18" s="8" t="n">
@@ -1362,13 +1450,13 @@
         <v>140</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="8" t="n">
@@ -1380,13 +1468,13 @@
         <v>141</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="8" t="n">
@@ -1398,13 +1486,13 @@
         <v>142</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="8" t="n">
@@ -1416,13 +1504,13 @@
         <v>143</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="8" t="n">
@@ -1434,16 +1522,16 @@
         <v>144</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1451,13 +1539,13 @@
         <v>145</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="8" t="n">
@@ -1469,16 +1557,16 @@
         <v>146</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1486,13 +1574,13 @@
         <v>147</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="8" t="n">
@@ -1504,13 +1592,13 @@
         <v>148</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="8" t="n">
@@ -1522,13 +1610,13 @@
         <v>149</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="8" t="n">
@@ -1540,13 +1628,13 @@
         <v>150</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="8" t="n">
@@ -1558,16 +1646,16 @@
         <v>151</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1575,16 +1663,16 @@
         <v>152</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1592,13 +1680,13 @@
         <v>160</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="n">
@@ -1610,13 +1698,13 @@
         <v>170</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E33" s="13"/>
       <c r="F33" s="8" t="n">
@@ -1628,13 +1716,13 @@
         <v>171</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E34" s="13"/>
       <c r="F34" s="14" t="n">
@@ -1646,13 +1734,13 @@
         <v>180</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E35" s="13"/>
       <c r="F35" s="14" t="n">
@@ -1664,13 +1752,13 @@
         <v>190</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="8" t="n">
@@ -1682,13 +1770,13 @@
         <v>200</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="8" t="n">
@@ -1700,16 +1788,16 @@
         <v>201</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1717,16 +1805,16 @@
         <v>210</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1734,13 +1822,13 @@
         <v>211</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E40" s="10"/>
       <c r="F40" s="11" t="n">
@@ -1752,13 +1840,13 @@
         <v>212</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E41" s="10"/>
       <c r="F41" s="11" t="n">
@@ -1770,13 +1858,13 @@
         <v>213</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E42" s="10"/>
       <c r="F42" s="11" t="n">
@@ -1788,16 +1876,16 @@
         <v>220</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1805,13 +1893,13 @@
         <v>221</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E44" s="13"/>
       <c r="F44" s="8" t="n">
@@ -1823,13 +1911,13 @@
         <v>222</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E45" s="13"/>
       <c r="F45" s="8" t="n">
@@ -1841,13 +1929,13 @@
         <v>223</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E46" s="13"/>
       <c r="F46" s="8" t="n">
@@ -1859,13 +1947,13 @@
         <v>224</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E47" s="13"/>
       <c r="F47" s="8" t="n">
@@ -1877,13 +1965,13 @@
         <v>225</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E48" s="13"/>
       <c r="F48" s="8" t="n">
@@ -1895,13 +1983,13 @@
         <v>226</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E49" s="13"/>
       <c r="F49" s="8" t="n">
@@ -1913,13 +2001,13 @@
         <v>227</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E50" s="13"/>
       <c r="F50" s="8" t="n">
@@ -1931,13 +2019,13 @@
         <v>228</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E51" s="13"/>
       <c r="F51" s="8" t="n">
@@ -1949,13 +2037,13 @@
         <v>229</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E52" s="13"/>
       <c r="F52" s="14" t="n">
@@ -1967,13 +2055,13 @@
         <v>240</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="8" t="n">
@@ -1985,16 +2073,16 @@
         <v>280</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2002,16 +2090,16 @@
         <v>281</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2019,13 +2107,13 @@
         <v>282</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E56" s="10"/>
       <c r="F56" s="11" t="n">
@@ -2037,13 +2125,13 @@
         <v>283</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E57" s="10"/>
       <c r="F57" s="11" t="n">
@@ -2055,13 +2143,13 @@
         <v>284</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E58" s="10"/>
       <c r="F58" s="11" t="n">
@@ -2073,13 +2161,13 @@
         <v>285</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="11" t="n">
@@ -2091,13 +2179,13 @@
         <v>290</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E60" s="7"/>
       <c r="F60" s="8" t="n">
@@ -2109,16 +2197,16 @@
         <v>291</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2126,13 +2214,13 @@
         <v>300</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E62" s="13"/>
       <c r="F62" s="8" t="n">
@@ -2144,13 +2232,13 @@
         <v>301</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E63" s="13"/>
       <c r="F63" s="8" t="n">
@@ -2162,13 +2250,13 @@
         <v>302</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E64" s="13"/>
       <c r="F64" s="8" t="n">
@@ -2180,13 +2268,13 @@
         <v>303</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E65" s="13"/>
       <c r="F65" s="8" t="n">
@@ -2198,13 +2286,13 @@
         <v>304</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E66" s="13"/>
       <c r="F66" s="8" t="n">
@@ -2216,13 +2304,13 @@
         <v>305</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E67" s="13"/>
       <c r="F67" s="8" t="n">
@@ -2234,13 +2322,13 @@
         <v>306</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E68" s="13"/>
       <c r="F68" s="8" t="n">
@@ -2252,13 +2340,13 @@
         <v>307</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E69" s="13"/>
       <c r="F69" s="14" t="n">
@@ -2270,13 +2358,13 @@
         <v>310</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E70" s="13"/>
       <c r="F70" s="8" t="n">
@@ -2288,13 +2376,13 @@
         <v>311</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E71" s="13"/>
       <c r="F71" s="8" t="n">
@@ -2306,13 +2394,13 @@
         <v>312</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E72" s="13"/>
       <c r="F72" s="8" t="n">
@@ -2324,13 +2412,13 @@
         <v>313</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E73" s="13"/>
       <c r="F73" s="8" t="n">
@@ -2342,13 +2430,13 @@
         <v>314</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E74" s="13"/>
       <c r="F74" s="8" t="n">
@@ -2360,13 +2448,13 @@
         <v>315</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E75" s="13"/>
       <c r="F75" s="8" t="n">
@@ -2378,13 +2466,13 @@
         <v>316</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E76" s="13"/>
       <c r="F76" s="14" t="n">
@@ -2396,16 +2484,16 @@
         <v>320</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2413,13 +2501,13 @@
         <v>321</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E78" s="13"/>
       <c r="F78" s="8" t="n">
@@ -2431,13 +2519,13 @@
         <v>322</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E79" s="13"/>
       <c r="F79" s="14" t="n">
@@ -2449,13 +2537,13 @@
         <v>325</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E80" s="13"/>
       <c r="F80" s="8" t="n">
@@ -2467,13 +2555,13 @@
         <v>326</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E81" s="13"/>
       <c r="F81" s="8" t="n">
@@ -2485,13 +2573,13 @@
         <v>327</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E82" s="13"/>
       <c r="F82" s="8" t="n">
@@ -2503,13 +2591,13 @@
         <v>328</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E83" s="13"/>
       <c r="F83" s="14" t="n">
@@ -2521,13 +2609,13 @@
         <v>330</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D84" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E84" s="7"/>
       <c r="F84" s="8" t="n">
@@ -2539,13 +2627,13 @@
         <v>331</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E85" s="7"/>
       <c r="F85" s="8" t="n">
@@ -2557,16 +2645,16 @@
         <v>332</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D86" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2574,13 +2662,13 @@
         <v>333</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C87" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E87" s="13"/>
       <c r="F87" s="8" t="n">
@@ -2592,16 +2680,16 @@
         <v>334</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2609,13 +2697,13 @@
         <v>335</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E89" s="13"/>
       <c r="F89" s="8" t="n">
@@ -2627,13 +2715,13 @@
         <v>336</v>
       </c>
       <c r="B90" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C90" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E90" s="13"/>
       <c r="F90" s="8" t="n">
@@ -2645,13 +2733,13 @@
         <v>337</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C91" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E91" s="13"/>
       <c r="F91" s="8" t="n">
@@ -2663,13 +2751,13 @@
         <v>338</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C92" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E92" s="13"/>
       <c r="F92" s="8" t="n">
@@ -2681,13 +2769,13 @@
         <v>339</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C93" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E93" s="13"/>
       <c r="F93" s="14" t="n">
@@ -2699,13 +2787,13 @@
         <v>345</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D94" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E94" s="7"/>
       <c r="F94" s="8" t="n">
@@ -2717,13 +2805,13 @@
         <v>346</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E95" s="7"/>
       <c r="F95" s="8" t="n">
@@ -2735,13 +2823,13 @@
         <v>347</v>
       </c>
       <c r="B96" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D96" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E96" s="7"/>
       <c r="F96" s="8" t="n">
@@ -2753,13 +2841,13 @@
         <v>348</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E97" s="7"/>
       <c r="F97" s="8" t="n">
@@ -2771,13 +2859,13 @@
         <v>349</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D98" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E98" s="7"/>
       <c r="F98" s="8" t="n">
@@ -2789,13 +2877,13 @@
         <v>350</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E99" s="7"/>
       <c r="F99" s="8" t="n">
@@ -2807,16 +2895,16 @@
         <v>351</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D100" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2824,13 +2912,13 @@
         <v>352</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D101" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E101" s="10"/>
       <c r="F101" s="8" t="n">
@@ -2842,13 +2930,13 @@
         <v>353</v>
       </c>
       <c r="B102" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D102" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E102" s="10"/>
       <c r="F102" s="8" t="n">
@@ -2860,13 +2948,13 @@
         <v>354</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C103" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D103" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E103" s="10"/>
       <c r="F103" s="8" t="n">
@@ -2878,13 +2966,13 @@
         <v>355</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E104" s="10"/>
       <c r="F104" s="8" t="n">
@@ -2896,13 +2984,13 @@
         <v>356</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C105" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D105" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E105" s="10"/>
       <c r="F105" s="8" t="n">
@@ -2914,13 +3002,13 @@
         <v>357</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D106" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E106" s="10"/>
       <c r="F106" s="8" t="n">
@@ -2932,13 +3020,13 @@
         <v>358</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D107" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E107" s="10"/>
       <c r="F107" s="8" t="n">
@@ -2950,16 +3038,16 @@
         <v>359</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D108" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2967,13 +3055,13 @@
         <v>360</v>
       </c>
       <c r="B109" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C109" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E109" s="13"/>
       <c r="F109" s="8" t="n">
@@ -2985,13 +3073,13 @@
         <v>361</v>
       </c>
       <c r="B110" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C110" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E110" s="13"/>
       <c r="F110" s="8" t="n">
@@ -3003,13 +3091,13 @@
         <v>362</v>
       </c>
       <c r="B111" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C111" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D111" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E111" s="10"/>
       <c r="F111" s="11" t="n">
@@ -3021,13 +3109,13 @@
         <v>365</v>
       </c>
       <c r="B112" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C112" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E112" s="10"/>
       <c r="F112" s="8" t="n">
@@ -3039,13 +3127,13 @@
         <v>366</v>
       </c>
       <c r="B113" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D113" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E113" s="10"/>
       <c r="F113" s="8" t="n">
@@ -3057,13 +3145,13 @@
         <v>367</v>
       </c>
       <c r="B114" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C114" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D114" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E114" s="10"/>
       <c r="F114" s="8" t="n">
@@ -3075,13 +3163,13 @@
         <v>368</v>
       </c>
       <c r="B115" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D115" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E115" s="10"/>
       <c r="F115" s="8" t="n">
@@ -3093,16 +3181,16 @@
         <v>369</v>
       </c>
       <c r="B116" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D116" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E116" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3110,13 +3198,13 @@
         <v>370</v>
       </c>
       <c r="B117" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C117" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E117" s="13"/>
       <c r="F117" s="8" t="n">
@@ -3128,13 +3216,13 @@
         <v>371</v>
       </c>
       <c r="B118" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C118" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E118" s="13"/>
       <c r="F118" s="8" t="n">
@@ -3146,13 +3234,13 @@
         <v>372</v>
       </c>
       <c r="B119" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C119" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D119" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E119" s="10"/>
       <c r="F119" s="8" t="n">
@@ -3164,13 +3252,13 @@
         <v>373</v>
       </c>
       <c r="B120" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C120" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D120" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E120" s="10"/>
       <c r="F120" s="8" t="n">
@@ -3182,13 +3270,13 @@
         <v>374</v>
       </c>
       <c r="B121" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C121" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D121" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E121" s="10"/>
       <c r="F121" s="8" t="n">
@@ -3200,13 +3288,13 @@
         <v>375</v>
       </c>
       <c r="B122" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C122" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D122" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E122" s="10"/>
       <c r="F122" s="11" t="n">
@@ -3218,13 +3306,13 @@
         <v>380</v>
       </c>
       <c r="B123" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D123" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E123" s="7"/>
       <c r="F123" s="8" t="n">
@@ -3236,16 +3324,16 @@
         <v>381</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D124" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E124" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3253,13 +3341,13 @@
         <v>382</v>
       </c>
       <c r="B125" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E125" s="15"/>
       <c r="F125" s="3" t="n">
@@ -3271,13 +3359,13 @@
         <v>383</v>
       </c>
       <c r="B126" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D126" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E126" s="16"/>
       <c r="F126" s="3" t="n">
@@ -3289,13 +3377,13 @@
         <v>384</v>
       </c>
       <c r="B127" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D127" s="16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E127" s="16"/>
       <c r="F127" s="3" t="n">
@@ -3307,13 +3395,13 @@
         <v>385</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D128" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E128" s="16"/>
       <c r="F128" s="3" t="n">
@@ -3325,13 +3413,13 @@
         <v>390</v>
       </c>
       <c r="B129" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C129" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D129" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E129" s="7"/>
       <c r="F129" s="0" t="n">
@@ -3343,13 +3431,13 @@
         <v>391</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C130" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D130" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E130" s="7"/>
       <c r="F130" s="3" t="n">
@@ -3361,13 +3449,13 @@
         <v>400</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F131" s="3" t="n">
         <v>401</v>
@@ -3378,13 +3466,13 @@
         <v>401</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C132" s="0" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D132" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E132" s="0"/>
       <c r="F132" s="0" t="n">
@@ -3396,16 +3484,16 @@
         <v>402</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3413,13 +3501,13 @@
         <v>403</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F134" s="3" t="n">
         <v>405</v>
@@ -3430,13 +3518,13 @@
         <v>404</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F135" s="3" t="n">
         <v>405</v>
@@ -3447,13 +3535,13 @@
         <v>405</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F136" s="3" t="n">
         <v>406</v>
@@ -3464,13 +3552,13 @@
         <v>406</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F137" s="3" t="n">
         <v>410</v>
@@ -3481,13 +3569,13 @@
         <v>407</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D138" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F138" s="3" t="n">
         <v>410</v>
@@ -3498,13 +3586,13 @@
         <v>410</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F139" s="3" t="n">
         <v>411</v>
@@ -3515,13 +3603,13 @@
         <v>411</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F140" s="3" t="n">
         <v>412</v>
@@ -3532,16 +3620,16 @@
         <v>412</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3549,13 +3637,13 @@
         <v>413</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F142" s="3" t="n">
         <v>414</v>
@@ -3566,13 +3654,13 @@
         <v>414</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D143" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E143" s="0"/>
       <c r="F143" s="3" t="n">
@@ -3584,13 +3672,13 @@
         <v>415</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D144" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E144" s="0"/>
       <c r="F144" s="3" t="n">
@@ -3602,13 +3690,13 @@
         <v>416</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F145" s="3" t="n">
         <v>417</v>
@@ -3619,13 +3707,13 @@
         <v>417</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F146" s="3" t="n">
         <v>418</v>
@@ -3636,13 +3724,13 @@
         <v>418</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F147" s="3" t="n">
         <v>419</v>
@@ -3653,13 +3741,13 @@
         <v>419</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F148" s="3" t="n">
         <v>420</v>
@@ -3670,13 +3758,13 @@
         <v>420</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F149" s="3" t="n">
         <v>421</v>
@@ -3687,13 +3775,13 @@
         <v>421</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F150" s="3" t="n">
         <v>422</v>
@@ -3704,13 +3792,13 @@
         <v>422</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F151" s="3" t="n">
         <v>423</v>
@@ -3721,13 +3809,13 @@
         <v>423</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F152" s="3" t="n">
         <v>424</v>
@@ -3738,13 +3826,13 @@
         <v>424</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F153" s="3" t="n">
         <v>425</v>
@@ -3755,13 +3843,13 @@
         <v>425</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F154" s="3" t="n">
         <v>426</v>
@@ -3772,13 +3860,13 @@
         <v>426</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F155" s="3" t="n">
         <v>427</v>
@@ -3789,13 +3877,13 @@
         <v>427</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F156" s="3" t="n">
         <v>428</v>
@@ -3806,13 +3894,13 @@
         <v>428</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F157" s="3" t="n">
         <v>429</v>
@@ -3823,13 +3911,13 @@
         <v>429</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F158" s="3" t="n">
         <v>430</v>
@@ -3840,13 +3928,13 @@
         <v>430</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F159" s="3" t="n">
         <v>431</v>
@@ -3857,13 +3945,13 @@
         <v>431</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F160" s="3" t="n">
         <v>432</v>
@@ -3874,13 +3962,13 @@
         <v>432</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F161" s="3" t="n">
         <v>433</v>
@@ -3891,13 +3979,13 @@
         <v>433</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F162" s="3" t="n">
         <v>434</v>
@@ -3908,16 +3996,16 @@
         <v>434</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3925,13 +4013,13 @@
         <v>435</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F164" s="3" t="n">
         <v>424</v>
@@ -3942,13 +4030,13 @@
         <v>436</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F165" s="3" t="n">
         <v>437</v>
@@ -3959,15 +4047,357 @@
         <v>437</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
+        <v>187</v>
+      </c>
+      <c r="F166" s="3" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F167" s="3" t="n">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="1" t="n">
+        <v>501</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="F168" s="3" t="n">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="1" t="n">
+        <v>502</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="1" t="n">
+        <v>503</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F170" s="3" t="n">
+        <v>504</v>
+      </c>
+      <c r="G170" s="0" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="1" t="n">
+        <v>504</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F171" s="3" t="n">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="1" t="n">
+        <v>505</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F172" s="3" t="n">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="1" t="n">
+        <v>506</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F173" s="3" t="n">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="1" t="n">
+        <v>507</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F174" s="3" t="n">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="1" t="n">
+        <v>508</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="F175" s="3" t="n">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="1" t="n">
+        <v>509</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="F176" s="3" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="1" t="n">
+        <v>510</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F177" s="3" t="n">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="1" t="n">
+        <v>511</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E178" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H178" s="17" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="1" t="n">
+        <v>520</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E179" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="1" t="n">
+        <v>521</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F180" s="3" t="n">
+        <v>522</v>
+      </c>
+      <c r="G180" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="1" t="n">
+        <v>522</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D181" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="F181" s="3" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="1" t="n">
+        <v>523</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F182" s="3" t="n">
+        <v>530</v>
+      </c>
+      <c r="G182" s="0" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="1" t="n">
+        <v>524</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D183" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F183" s="3" t="n">
+        <v>522</v>
+      </c>
+      <c r="G183" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="1" t="n">
+        <v>530</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F184" s="3" t="n">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="1" t="n">
+        <v>531</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D185" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E185" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Phase 1 of chapter 5
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="240">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -625,10 +625,10 @@
     <t xml:space="preserve">GAME OVER</t>
   </si>
   <si>
-    <t xml:space="preserve">The message within encrypted data is hidden, but the existence of it is not.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want to try phase 1 again?</t>
+    <t xml:space="preserve">Hm… the message within encrypted data is hidden, but the existence of it is not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to try again from phase 1 of the final mission?</t>
   </si>
   <si>
     <t xml:space="preserve">Yes -&gt; 500; No -&gt; 650</t>
@@ -661,7 +661,85 @@
     <t xml:space="preserve">Where in the image should I hide?</t>
   </si>
   <si>
-    <t xml:space="preserve">At the start of the file -&gt; 0; At the end of the file -&gt; 0; Replace the most significant bits by me -&gt; 0; Replace the least significant bits by me -&gt; 0</t>
+    <t xml:space="preserve">At the start of the file -&gt; 535; At the end of the file -&gt; 535; Replace the most significant bits by me -&gt; 550; Replace the least significant bits by me -&gt; 580</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Okay, let’s go!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I see you are an email, with an image attachment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The image looks highly altered. A lot of redundant data seems to be put together.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Therefore, I cannot guarantee that you have no means of harm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You will be quarantined!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hmm… putting a data object at the very start or end is very suspicious.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It can easily be detected. I should try to spread the data throughout the file more next time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How will I hide myself within these most significant bits?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I will hide 100% in these bits to be undetectable for their anti-malware system -&gt; 551;  I will hide 100% in these bits and attach a small script that extracts myself -&gt; 570</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The colours of the image look so weird, as if they are not the right colours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">But maybe that is just a new hype or art trend that I am not aware of.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You are lucky! I will let you through this time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pfeww! I am through, but I could have better hidden in the least significant bits of the image…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">That way, the colours are not altered much.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Now I should wait until Agent T. opens the image of the email that I am part of.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agent T. opened the image but I am still stuck in the image…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Their computer system does not see me, the Stegware, and can thus never execute me…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I am stuck in this image forever, because nothing gets me out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How will I hide myself within these least significant bits?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I will hide 100% in these bits to be undetectable for their anti-malware system -&gt; 581;  I will hide 100% in these bits and attach a small script that extracts myself -&gt; 590</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I do not see anything suspicious, you may pass through.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Now I should wait until Agent T. opens the attachment, which runs the extract script to extract myself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great! Agent T. opened the image and I got extracted. I am fully free in the SilentSpectra network now!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 1 of the mission finished! Now let’s continue to phase 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What was phase 2 again?</t>
   </si>
 </sst>
 </file>
@@ -787,7 +865,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -848,7 +926,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -856,7 +934,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3422,7 +3504,7 @@
         <v>147</v>
       </c>
       <c r="E129" s="7"/>
-      <c r="F129" s="0" t="n">
+      <c r="F129" s="17" t="n">
         <v>391</v>
       </c>
     </row>
@@ -3462,20 +3544,20 @@
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="0" t="n">
+      <c r="A132" s="17" t="n">
         <v>401</v>
       </c>
-      <c r="B132" s="0" t="s">
+      <c r="B132" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C132" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="D132" s="0" t="s">
+      <c r="C132" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D132" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="E132" s="0"/>
-      <c r="F132" s="0" t="n">
+      <c r="E132" s="17"/>
+      <c r="F132" s="17" t="n">
         <v>402</v>
       </c>
     </row>
@@ -3574,7 +3656,7 @@
       <c r="C138" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D138" s="0" t="s">
+      <c r="D138" s="17" t="s">
         <v>157</v>
       </c>
       <c r="F138" s="3" t="n">
@@ -3659,10 +3741,10 @@
       <c r="C143" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D143" s="0" t="s">
+      <c r="D143" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="E143" s="0"/>
+      <c r="E143" s="17"/>
       <c r="F143" s="3" t="n">
         <v>415</v>
       </c>
@@ -3677,10 +3759,10 @@
       <c r="C144" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D144" s="0" t="s">
+      <c r="D144" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="E144" s="0"/>
+      <c r="E144" s="17"/>
       <c r="F144" s="3" t="n">
         <v>416</v>
       </c>
@@ -4126,9 +4208,7 @@
       <c r="F170" s="3" t="n">
         <v>504</v>
       </c>
-      <c r="G170" s="0" t="n">
-        <v>-10</v>
-      </c>
+      <c r="G170" s="17"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="1" t="n">
@@ -4231,6 +4311,9 @@
       <c r="F176" s="3" t="n">
         <v>510</v>
       </c>
+      <c r="G176" s="0" t="n">
+        <v>-10</v>
+      </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="1" t="n">
@@ -4265,7 +4348,7 @@
       <c r="E178" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="H178" s="17" t="s">
+      <c r="H178" s="18" t="s">
         <v>204</v>
       </c>
     </row>
@@ -4302,7 +4385,7 @@
       <c r="F180" s="3" t="n">
         <v>522</v>
       </c>
-      <c r="G180" s="0" t="n">
+      <c r="G180" s="17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4339,7 +4422,7 @@
       <c r="F182" s="3" t="n">
         <v>530</v>
       </c>
-      <c r="G182" s="0" t="n">
+      <c r="G182" s="17" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4359,7 +4442,7 @@
       <c r="F183" s="3" t="n">
         <v>522</v>
       </c>
-      <c r="G183" s="0" t="n">
+      <c r="G183" s="17" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4396,6 +4479,1043 @@
       <c r="E185" s="2" t="s">
         <v>213</v>
       </c>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="1" t="n">
+        <v>535</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D186" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F186" s="3" t="n">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="1" t="n">
+        <v>536</v>
+      </c>
+      <c r="B187" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C187" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D187" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F187" s="3" t="n">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="1" t="n">
+        <v>537</v>
+      </c>
+      <c r="B188" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C188" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D188" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F188" s="3" t="n">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="1" t="n">
+        <v>538</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D189" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="F189" s="3" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="1" t="n">
+        <v>539</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C190" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D190" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F190" s="3" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="1" t="n">
+        <v>540</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="F191" s="3" t="n">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="1" t="n">
+        <v>541</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D192" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="F192" s="3" t="n">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="1" t="n">
+        <v>542</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D193" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="F193" s="3" t="n">
+        <v>543</v>
+      </c>
+      <c r="G193" s="0" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="1" t="n">
+        <v>543</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D194" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F194" s="3" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="1" t="n">
+        <v>544</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="F195" s="3" t="n">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="1" t="n">
+        <v>545</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D196" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E196" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="0" t="n">
+        <v>550</v>
+      </c>
+      <c r="B197" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C197" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D197" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="E197" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="F197" s="0"/>
+      <c r="G197" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="0" t="n">
+        <v>551</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D198" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F198" s="0" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="0" t="n">
+        <v>552</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D199" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F199" s="0" t="n">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="0" t="n">
+        <v>553</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D200" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F200" s="0" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="0" t="n">
+        <v>554</v>
+      </c>
+      <c r="B201" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="F201" s="0" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="0" t="n">
+        <v>555</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F202" s="0" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="0" t="n">
+        <v>556</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C203" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D203" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F203" s="0" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="0" t="n">
+        <v>557</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F204" s="0" t="n">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="0" t="n">
+        <v>558</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D205" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F205" s="0" t="n">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="0" t="n">
+        <v>559</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D206" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F206" s="0" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="0" t="n">
+        <v>560</v>
+      </c>
+      <c r="B207" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D207" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E207" s="0"/>
+      <c r="F207" s="0" t="n">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="0" t="n">
+        <v>561</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D208" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E208" s="0"/>
+      <c r="F208" s="0" t="n">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="0" t="n">
+        <v>562</v>
+      </c>
+      <c r="B209" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D209" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E209" s="0"/>
+      <c r="F209" s="0" t="n">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="0" t="n">
+        <v>563</v>
+      </c>
+      <c r="B210" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C210" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D210" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E210" s="0"/>
+      <c r="F210" s="0" t="n">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="0" t="n">
+        <v>564</v>
+      </c>
+      <c r="B211" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D211" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="E211" s="0"/>
+      <c r="F211" s="0" t="n">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="0" t="n">
+        <v>565</v>
+      </c>
+      <c r="B212" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D212" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="E212" s="0"/>
+      <c r="F212" s="0" t="n">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="0" t="n">
+        <v>566</v>
+      </c>
+      <c r="B213" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D213" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E213" s="0"/>
+      <c r="F213" s="0" t="n">
+        <v>567</v>
+      </c>
+      <c r="G213" s="0" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="0" t="n">
+        <v>567</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D214" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E214" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F214" s="0"/>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="0" t="n">
+        <v>570</v>
+      </c>
+      <c r="B215" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C215" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F215" s="0" t="n">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="0" t="n">
+        <v>571</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F216" s="0" t="n">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="0" t="n">
+        <v>572</v>
+      </c>
+      <c r="B217" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C217" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D217" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="F217" s="0" t="n">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="0" t="n">
+        <v>573</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F218" s="0" t="n">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="0" t="n">
+        <v>574</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F219" s="0" t="n">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="0" t="n">
+        <v>575</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F220" s="0" t="n">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="0" t="n">
+        <v>576</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F221" s="0" t="n">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="0" t="n">
+        <v>577</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F222" s="0" t="n">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="0" t="n">
+        <v>580</v>
+      </c>
+      <c r="B223" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C223" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D223" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="E223" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="F223" s="0"/>
+      <c r="G223" s="0" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="0" t="n">
+        <v>581</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E224" s="0"/>
+      <c r="F224" s="3" t="n">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="0" t="n">
+        <v>582</v>
+      </c>
+      <c r="B225" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C225" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E225" s="0"/>
+      <c r="F225" s="3" t="n">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="0" t="n">
+        <v>583</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D226" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E226" s="0"/>
+      <c r="F226" s="3" t="n">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="0" t="n">
+        <v>584</v>
+      </c>
+      <c r="B227" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D227" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E227" s="0"/>
+      <c r="F227" s="3" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="0" t="n">
+        <v>585</v>
+      </c>
+      <c r="B228" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D228" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E228" s="0"/>
+      <c r="F228" s="3" t="n">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="0" t="n">
+        <v>586</v>
+      </c>
+      <c r="B229" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E229" s="0"/>
+      <c r="F229" s="3" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="0" t="n">
+        <v>590</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D230" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E230" s="0"/>
+      <c r="F230" s="3" t="n">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="0" t="n">
+        <v>591</v>
+      </c>
+      <c r="B231" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E231" s="0"/>
+      <c r="F231" s="3" t="n">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="0" t="n">
+        <v>592</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D232" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E232" s="0"/>
+      <c r="F232" s="3" t="n">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="0" t="n">
+        <v>593</v>
+      </c>
+      <c r="B233" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D233" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E233" s="0"/>
+      <c r="F233" s="3" t="n">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="0" t="n">
+        <v>594</v>
+      </c>
+      <c r="B234" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E234" s="0"/>
+      <c r="F234" s="3" t="n">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="0" t="n">
+        <v>595</v>
+      </c>
+      <c r="B235" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D235" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E235" s="0"/>
+      <c r="F235" s="3" t="n">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="0" t="n">
+        <v>596</v>
+      </c>
+      <c r="B236" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C236" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E236" s="0"/>
+      <c r="F236" s="3" t="n">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="0" t="n">
+        <v>597</v>
+      </c>
+      <c r="B237" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C237" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D237" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F237" s="3" t="n">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="0" t="n">
+        <v>598</v>
+      </c>
+      <c r="B238" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D238" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E238" s="0"/>
+      <c r="F238" s="3" t="n">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="0" t="n">
+        <v>599</v>
+      </c>
+      <c r="B239" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C239" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D239" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E239" s="0"/>
+      <c r="F239" s="3" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="0" t="n">
+        <v>600</v>
+      </c>
+      <c r="B240" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C240" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D240" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="E240" s="0"/>
+      <c r="F240" s="3" t="n">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="0" t="n">
+        <v>601</v>
+      </c>
+      <c r="B241" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C241" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D241" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E241" s="0"/>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="0"/>
+      <c r="B242" s="0"/>
+      <c r="C242" s="0"/>
+      <c r="D242" s="0"/>
+      <c r="E242" s="0"/>
+    </row>
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="0"/>
+      <c r="B243" s="0"/>
+      <c r="C243" s="0"/>
+      <c r="D243" s="0"/>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="0"/>
+      <c r="B244" s="0"/>
+      <c r="C244" s="0"/>
+      <c r="D244" s="0"/>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="0"/>
+      <c r="B245" s="0"/>
+      <c r="C245" s="0"/>
+      <c r="D245" s="0"/>
+    </row>
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="0"/>
+      <c r="B246" s="0"/>
+      <c r="C246" s="0"/>
+      <c r="D246" s="0"/>
+    </row>
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="0"/>
+      <c r="B247" s="0"/>
+      <c r="C247" s="0"/>
+      <c r="D247" s="0"/>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="0"/>
+      <c r="B248" s="0"/>
+      <c r="C248" s="0"/>
+      <c r="D248" s="0"/>
+    </row>
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="0"/>
+      <c r="B249" s="0"/>
+      <c r="C249" s="0"/>
+      <c r="D249" s="0"/>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>

<commit_message>
update text for learning goals
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="284">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -250,7 +250,10 @@
     <t xml:space="preserve">Hm… The first book is about the difference between steganography and cryptography.</t>
   </si>
   <si>
-    <t xml:space="preserve">Also, on the right side an example of hiding a message with the help of lemon juice.</t>
+    <t xml:space="preserve">Also, on the right side an example of hiding a message with the help of lemon juice is shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Below that an example of a secret message using cryptography.</t>
   </si>
   <si>
     <t xml:space="preserve">The second book is a history book.</t>
@@ -496,7 +499,7 @@
     <t xml:space="preserve">Good morning… I worked all night, but I found out that SilentSpectra is indeed using Facebook for communication.</t>
   </si>
   <si>
-    <t xml:space="preserve">We have seen their messages before of course, but we weren’t aware that they integrated their secret message within the attached files.</t>
+    <t xml:space="preserve">We have seen their public messages on social media before of course, but we weren’t aware that they integrated their secret message within the attached files.</t>
   </si>
   <si>
     <t xml:space="preserve">Indeed. I also found out that Agent T., who is working for SilentSpectra is using the email adress tom@covinco.com actively.</t>
@@ -2420,29 +2423,30 @@
       </c>
       <c r="E61" s="7"/>
       <c r="F61" s="8" t="n">
-        <v>201</v>
+        <v>247</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="n">
-        <v>280</v>
+        <v>247</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E62" s="7" t="s">
-        <v>82</v>
+      <c r="E62" s="7"/>
+      <c r="F62" s="8" t="n">
+        <v>201</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B63" s="7" t="s">
         <v>7</v>
@@ -2451,33 +2455,32 @@
         <v>10</v>
       </c>
       <c r="D63" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E63" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E63" s="7" t="s">
+    </row>
+    <row r="64" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="6" t="n">
+        <v>281</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D64" s="7" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="9" t="n">
-        <v>282</v>
-      </c>
-      <c r="B64" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C64" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D64" s="10" t="s">
+      <c r="E64" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="E64" s="10"/>
-      <c r="F64" s="11" t="n">
-        <v>281</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="n">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>7</v>
@@ -2490,12 +2493,12 @@
       </c>
       <c r="E65" s="10"/>
       <c r="F65" s="11" t="n">
-        <v>290</v>
+        <v>281</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>7</v>
@@ -2508,12 +2511,12 @@
       </c>
       <c r="E66" s="10"/>
       <c r="F66" s="11" t="n">
-        <v>281</v>
+        <v>290</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="n">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>7</v>
@@ -2530,61 +2533,61 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="6" t="n">
-        <v>290</v>
-      </c>
-      <c r="B68" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C68" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D68" s="7" t="s">
+      <c r="A68" s="9" t="n">
+        <v>285</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D68" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="E68" s="7"/>
-      <c r="F68" s="8" t="n">
-        <v>291</v>
+      <c r="E68" s="10"/>
+      <c r="F68" s="11" t="n">
+        <v>281</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D69" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E69" s="7" t="s">
+      <c r="E69" s="7"/>
+      <c r="F69" s="8" t="n">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="6" t="n">
+        <v>291</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D70" s="7" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="70" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="12" t="n">
-        <v>300</v>
-      </c>
-      <c r="B70" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C70" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D70" s="13" t="s">
+      <c r="E70" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="E70" s="13"/>
-      <c r="F70" s="8" t="n">
-        <v>301</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B71" s="13" t="s">
         <v>7</v>
@@ -2593,16 +2596,16 @@
         <v>8</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="E71" s="13"/>
       <c r="F71" s="8" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B72" s="13" t="s">
         <v>7</v>
@@ -2611,16 +2614,16 @@
         <v>8</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E72" s="13"/>
       <c r="F72" s="8" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B73" s="13" t="s">
         <v>7</v>
@@ -2629,16 +2632,16 @@
         <v>8</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E73" s="13"/>
       <c r="F73" s="8" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B74" s="13" t="s">
         <v>7</v>
@@ -2647,16 +2650,16 @@
         <v>8</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E74" s="13"/>
       <c r="F74" s="8" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B75" s="13" t="s">
         <v>7</v>
@@ -2665,16 +2668,16 @@
         <v>8</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="E75" s="13"/>
       <c r="F75" s="8" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B76" s="13" t="s">
         <v>7</v>
@@ -2687,12 +2690,12 @@
       </c>
       <c r="E76" s="13"/>
       <c r="F76" s="8" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B77" s="13" t="s">
         <v>7</v>
@@ -2704,13 +2707,13 @@
         <v>95</v>
       </c>
       <c r="E77" s="13"/>
-      <c r="F77" s="14" t="n">
-        <v>200</v>
+      <c r="F77" s="8" t="n">
+        <v>307</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="n">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B78" s="13" t="s">
         <v>7</v>
@@ -2722,13 +2725,13 @@
         <v>96</v>
       </c>
       <c r="E78" s="13"/>
-      <c r="F78" s="8" t="n">
-        <v>311</v>
+      <c r="F78" s="14" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="n">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B79" s="13" t="s">
         <v>7</v>
@@ -2741,12 +2744,12 @@
       </c>
       <c r="E79" s="13"/>
       <c r="F79" s="8" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B80" s="13" t="s">
         <v>7</v>
@@ -2759,12 +2762,12 @@
       </c>
       <c r="E80" s="13"/>
       <c r="F80" s="8" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B81" s="13" t="s">
         <v>7</v>
@@ -2777,12 +2780,12 @@
       </c>
       <c r="E81" s="13"/>
       <c r="F81" s="8" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B82" s="13" t="s">
         <v>7</v>
@@ -2795,12 +2798,12 @@
       </c>
       <c r="E82" s="13"/>
       <c r="F82" s="8" t="n">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="n">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B83" s="13" t="s">
         <v>7</v>
@@ -2813,12 +2816,12 @@
       </c>
       <c r="E83" s="13"/>
       <c r="F83" s="8" t="n">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="n">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B84" s="13" t="s">
         <v>7</v>
@@ -2830,48 +2833,48 @@
         <v>102</v>
       </c>
       <c r="E84" s="13"/>
-      <c r="F84" s="14" t="n">
+      <c r="F84" s="8" t="n">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="12" t="n">
+        <v>316</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E85" s="13"/>
+      <c r="F85" s="14" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="6" t="n">
+    <row r="86" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="6" t="n">
         <v>320</v>
       </c>
-      <c r="B85" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C85" s="7" t="s">
+      <c r="B86" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C86" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D85" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E85" s="7" t="s">
+      <c r="D86" s="7" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="86" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="12" t="n">
-        <v>321</v>
-      </c>
-      <c r="B86" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C86" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D86" s="13" t="s">
+      <c r="E86" s="7" t="s">
         <v>105</v>
-      </c>
-      <c r="E86" s="13"/>
-      <c r="F86" s="8" t="n">
-        <v>322</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="n">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B87" s="13" t="s">
         <v>7</v>
@@ -2883,13 +2886,13 @@
         <v>106</v>
       </c>
       <c r="E87" s="13"/>
-      <c r="F87" s="14" t="n">
-        <v>320</v>
+      <c r="F87" s="8" t="n">
+        <v>322</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="n">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B88" s="13" t="s">
         <v>7</v>
@@ -2901,13 +2904,13 @@
         <v>107</v>
       </c>
       <c r="E88" s="13"/>
-      <c r="F88" s="8" t="n">
-        <v>326</v>
+      <c r="F88" s="14" t="n">
+        <v>320</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="n">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B89" s="13" t="s">
         <v>7</v>
@@ -2920,12 +2923,12 @@
       </c>
       <c r="E89" s="13"/>
       <c r="F89" s="8" t="n">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="n">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B90" s="13" t="s">
         <v>7</v>
@@ -2938,12 +2941,12 @@
       </c>
       <c r="E90" s="13"/>
       <c r="F90" s="8" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B91" s="13" t="s">
         <v>7</v>
@@ -2955,31 +2958,31 @@
         <v>110</v>
       </c>
       <c r="E91" s="13"/>
-      <c r="F91" s="14" t="n">
+      <c r="F91" s="8" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="12" t="n">
+        <v>328</v>
+      </c>
+      <c r="B92" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C92" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="E92" s="13"/>
+      <c r="F92" s="14" t="n">
         <v>320</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="6" t="n">
-        <v>330</v>
-      </c>
-      <c r="B92" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C92" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D92" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E92" s="7"/>
-      <c r="F92" s="8" t="n">
-        <v>331</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="n">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B93" s="7" t="s">
         <v>7</v>
@@ -2992,82 +2995,82 @@
       </c>
       <c r="E93" s="7"/>
       <c r="F93" s="8" t="n">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="6" t="n">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B94" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D94" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E94" s="7" t="s">
+      <c r="E94" s="7"/>
+      <c r="F94" s="8" t="n">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="6" t="n">
+        <v>332</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D95" s="7" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="95" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="12" t="n">
-        <v>333</v>
-      </c>
-      <c r="B95" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C95" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D95" s="13" t="s">
+      <c r="E95" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="E95" s="13"/>
-      <c r="F95" s="8" t="n">
-        <v>334</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="n">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B96" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C96" s="13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D96" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="E96" s="13" t="s">
-        <v>117</v>
+      <c r="E96" s="13"/>
+      <c r="F96" s="8" t="n">
+        <v>334</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="12" t="n">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B97" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C97" s="13" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D97" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E97" s="13" t="s">
         <v>118</v>
-      </c>
-      <c r="E97" s="13"/>
-      <c r="F97" s="8" t="n">
-        <v>336</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="12" t="n">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B98" s="13" t="s">
         <v>7</v>
@@ -3080,12 +3083,12 @@
       </c>
       <c r="E98" s="13"/>
       <c r="F98" s="8" t="n">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="12" t="n">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B99" s="13" t="s">
         <v>7</v>
@@ -3098,12 +3101,12 @@
       </c>
       <c r="E99" s="13"/>
       <c r="F99" s="8" t="n">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="12" t="n">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B100" s="13" t="s">
         <v>7</v>
@@ -3116,12 +3119,12 @@
       </c>
       <c r="E100" s="13"/>
       <c r="F100" s="8" t="n">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="12" t="n">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B101" s="13" t="s">
         <v>7</v>
@@ -3133,31 +3136,31 @@
         <v>122</v>
       </c>
       <c r="E101" s="13"/>
-      <c r="F101" s="14" t="n">
+      <c r="F101" s="8" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="12" t="n">
+        <v>339</v>
+      </c>
+      <c r="B102" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="E102" s="13"/>
+      <c r="F102" s="14" t="n">
         <v>345</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="6" t="n">
-        <v>345</v>
-      </c>
-      <c r="B102" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C102" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D102" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="E102" s="7"/>
-      <c r="F102" s="8" t="n">
-        <v>346</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="6" t="n">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B103" s="7" t="s">
         <v>7</v>
@@ -3170,12 +3173,12 @@
       </c>
       <c r="E103" s="7"/>
       <c r="F103" s="8" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="6" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B104" s="7" t="s">
         <v>7</v>
@@ -3188,12 +3191,12 @@
       </c>
       <c r="E104" s="7"/>
       <c r="F104" s="8" t="n">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="6" t="n">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B105" s="7" t="s">
         <v>7</v>
@@ -3206,12 +3209,12 @@
       </c>
       <c r="E105" s="7"/>
       <c r="F105" s="8" t="n">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="6" t="n">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B106" s="7" t="s">
         <v>7</v>
@@ -3224,12 +3227,12 @@
       </c>
       <c r="E106" s="7"/>
       <c r="F106" s="8" t="n">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="6" t="n">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B107" s="7" t="s">
         <v>7</v>
@@ -3242,47 +3245,47 @@
       </c>
       <c r="E107" s="7"/>
       <c r="F107" s="8" t="n">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="6" t="n">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B108" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D108" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="E108" s="7" t="s">
+      <c r="E108" s="7"/>
+      <c r="F108" s="8" t="n">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="6" t="n">
+        <v>351</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D109" s="7" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="109" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="9" t="n">
-        <v>352</v>
-      </c>
-      <c r="B109" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C109" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D109" s="10" t="s">
+      <c r="E109" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="E109" s="10"/>
-      <c r="F109" s="8" t="n">
-        <v>353</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="9" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B110" s="10" t="s">
         <v>7</v>
@@ -3295,12 +3298,12 @@
       </c>
       <c r="E110" s="10"/>
       <c r="F110" s="8" t="n">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="9" t="n">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B111" s="10" t="s">
         <v>7</v>
@@ -3313,12 +3316,12 @@
       </c>
       <c r="E111" s="10"/>
       <c r="F111" s="8" t="n">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="9" t="n">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B112" s="10" t="s">
         <v>7</v>
@@ -3331,12 +3334,12 @@
       </c>
       <c r="E112" s="10"/>
       <c r="F112" s="8" t="n">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="9" t="n">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B113" s="10" t="s">
         <v>7</v>
@@ -3349,12 +3352,12 @@
       </c>
       <c r="E113" s="10"/>
       <c r="F113" s="8" t="n">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="9" t="n">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B114" s="10" t="s">
         <v>7</v>
@@ -3367,12 +3370,12 @@
       </c>
       <c r="E114" s="10"/>
       <c r="F114" s="8" t="n">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="9" t="n">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B115" s="10" t="s">
         <v>7</v>
@@ -3385,47 +3388,47 @@
       </c>
       <c r="E115" s="10"/>
       <c r="F115" s="8" t="n">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="9" t="n">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B116" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D116" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="E116" s="10" t="s">
+      <c r="E116" s="10"/>
+      <c r="F116" s="8" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="9" t="n">
+        <v>359</v>
+      </c>
+      <c r="B117" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C117" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D117" s="10" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="117" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="12" t="n">
-        <v>360</v>
-      </c>
-      <c r="B117" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C117" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D117" s="13" t="s">
+      <c r="E117" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="E117" s="13"/>
-      <c r="F117" s="8" t="n">
-        <v>361</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="12" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B118" s="13" t="s">
         <v>7</v>
@@ -3438,30 +3441,30 @@
       </c>
       <c r="E118" s="13"/>
       <c r="F118" s="8" t="n">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="12" t="n">
+        <v>361</v>
+      </c>
+      <c r="B119" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C119" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D119" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E119" s="13"/>
+      <c r="F119" s="8" t="n">
         <v>362</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="9" t="n">
-        <v>362</v>
-      </c>
-      <c r="B119" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C119" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D119" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="E119" s="10"/>
-      <c r="F119" s="11" t="n">
-        <v>380</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="9" t="n">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B120" s="10" t="s">
         <v>7</v>
@@ -3470,16 +3473,16 @@
         <v>8</v>
       </c>
       <c r="D120" s="10" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E120" s="10"/>
-      <c r="F120" s="8" t="n">
-        <v>366</v>
+      <c r="F120" s="11" t="n">
+        <v>380</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="9" t="n">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B121" s="10" t="s">
         <v>7</v>
@@ -3492,12 +3495,12 @@
       </c>
       <c r="E121" s="10"/>
       <c r="F121" s="8" t="n">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="9" t="n">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B122" s="10" t="s">
         <v>7</v>
@@ -3510,12 +3513,12 @@
       </c>
       <c r="E122" s="10"/>
       <c r="F122" s="8" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="9" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B123" s="10" t="s">
         <v>7</v>
@@ -3528,47 +3531,47 @@
       </c>
       <c r="E123" s="10"/>
       <c r="F123" s="8" t="n">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="9" t="n">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B124" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C124" s="10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D124" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="E124" s="10" t="s">
-        <v>143</v>
+      <c r="E124" s="10"/>
+      <c r="F124" s="8" t="n">
+        <v>369</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A125" s="12" t="n">
-        <v>370</v>
-      </c>
-      <c r="B125" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C125" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D125" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="E125" s="13"/>
-      <c r="F125" s="8" t="n">
-        <v>371</v>
+      <c r="A125" s="9" t="n">
+        <v>369</v>
+      </c>
+      <c r="B125" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C125" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D125" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E125" s="10" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="12" t="n">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B126" s="13" t="s">
         <v>7</v>
@@ -3581,30 +3584,30 @@
       </c>
       <c r="E126" s="13"/>
       <c r="F126" s="8" t="n">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A127" s="12" t="n">
+        <v>371</v>
+      </c>
+      <c r="B127" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C127" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D127" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E127" s="13"/>
+      <c r="F127" s="8" t="n">
         <v>372</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A127" s="9" t="n">
-        <v>372</v>
-      </c>
-      <c r="B127" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C127" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D127" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="E127" s="10"/>
-      <c r="F127" s="8" t="n">
-        <v>373</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="9" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B128" s="10" t="s">
         <v>7</v>
@@ -3613,16 +3616,16 @@
         <v>8</v>
       </c>
       <c r="D128" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E128" s="10"/>
       <c r="F128" s="8" t="n">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="9" t="n">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B129" s="10" t="s">
         <v>7</v>
@@ -3635,12 +3638,12 @@
       </c>
       <c r="E129" s="10"/>
       <c r="F129" s="8" t="n">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="9" t="n">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B130" s="10" t="s">
         <v>7</v>
@@ -3652,84 +3655,84 @@
         <v>146</v>
       </c>
       <c r="E130" s="10"/>
-      <c r="F130" s="11" t="n">
+      <c r="F130" s="8" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A131" s="9" t="n">
+        <v>375</v>
+      </c>
+      <c r="B131" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C131" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D131" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="E131" s="10"/>
+      <c r="F131" s="11" t="n">
         <v>380</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A131" s="6" t="n">
-        <v>380</v>
-      </c>
-      <c r="B131" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C131" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="D131" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="E131" s="7"/>
-      <c r="F131" s="8" t="n">
-        <v>381</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="6" t="n">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B132" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C132" s="7" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="D132" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="E132" s="7" t="s">
+      <c r="E132" s="7"/>
+      <c r="F132" s="8" t="n">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A133" s="6" t="n">
+        <v>381</v>
+      </c>
+      <c r="B133" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C133" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D133" s="7" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="133" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A133" s="12" t="n">
+      <c r="E133" s="7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A134" s="12" t="n">
         <v>382</v>
       </c>
-      <c r="B133" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C133" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D133" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="E133" s="15"/>
-      <c r="F133" s="3" t="n">
+      <c r="B134" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C134" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D134" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="E134" s="15"/>
+      <c r="F134" s="3" t="n">
         <v>383</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="12" t="n">
-        <v>383</v>
-      </c>
-      <c r="B134" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C134" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D134" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="E134" s="16"/>
-      <c r="F134" s="3" t="n">
-        <v>384</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="12" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B135" s="15" t="s">
         <v>7</v>
@@ -3742,12 +3745,12 @@
       </c>
       <c r="E135" s="16"/>
       <c r="F135" s="3" t="n">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="12" t="n">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B136" s="15" t="s">
         <v>7</v>
@@ -3760,33 +3763,33 @@
       </c>
       <c r="E136" s="16"/>
       <c r="F136" s="3" t="n">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="12" t="n">
+        <v>385</v>
+      </c>
+      <c r="B137" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C137" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D137" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="E137" s="16"/>
+      <c r="F137" s="3" t="n">
         <v>381</v>
-      </c>
-    </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="6" t="n">
-        <v>390</v>
-      </c>
-      <c r="B137" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C137" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D137" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="E137" s="7"/>
-      <c r="F137" s="17" t="n">
-        <v>391</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="6" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B138" s="7" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C138" s="7" t="s">
         <v>8</v>
@@ -3795,82 +3798,83 @@
         <v>156</v>
       </c>
       <c r="E138" s="7"/>
-      <c r="F138" s="3" t="n">
+      <c r="F138" s="17" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="6" t="n">
+        <v>391</v>
+      </c>
+      <c r="B139" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C139" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D139" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="E139" s="7"/>
+      <c r="F139" s="3" t="n">
         <v>400</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="1" t="n">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="B139" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D139" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="F139" s="3" t="n">
+      <c r="B140" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F140" s="3" t="n">
         <v>401</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="17" t="n">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="17" t="n">
         <v>401</v>
       </c>
-      <c r="B140" s="17" t="s">
+      <c r="B141" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C140" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D140" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="E140" s="17"/>
-      <c r="F140" s="17" t="n">
+      <c r="C141" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D141" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="E141" s="17"/>
+      <c r="F141" s="17" t="n">
         <v>402</v>
-      </c>
-    </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="1" t="n">
-        <v>402</v>
-      </c>
-      <c r="B141" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C141" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D141" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="E141" s="2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="n">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D142" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E142" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="F142" s="3" t="n">
-        <v>405</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>7</v>
@@ -3887,10 +3891,10 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="1" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>8</v>
@@ -3899,15 +3903,15 @@
         <v>163</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="1" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>8</v>
@@ -3916,12 +3920,12 @@
         <v>164</v>
       </c>
       <c r="F145" s="3" t="n">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="1" t="n">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>7</v>
@@ -3929,7 +3933,7 @@
       <c r="C146" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D146" s="17" t="s">
+      <c r="D146" s="2" t="s">
         <v>165</v>
       </c>
       <c r="F146" s="3" t="n">
@@ -3938,27 +3942,27 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="1" t="n">
+        <v>407</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D147" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="F147" s="3" t="n">
         <v>410</v>
-      </c>
-      <c r="B147" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D147" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="F147" s="3" t="n">
-        <v>411</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="1" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>8</v>
@@ -3967,46 +3971,46 @@
         <v>167</v>
       </c>
       <c r="F148" s="3" t="n">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="1" t="n">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D149" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E149" s="2" t="s">
-        <v>169</v>
+      <c r="F149" s="3" t="n">
+        <v>412</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="1" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D150" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E150" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="F150" s="3" t="n">
-        <v>414</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="1" t="n">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>20</v>
@@ -4014,17 +4018,16 @@
       <c r="C151" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D151" s="17" t="s">
+      <c r="D151" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="E151" s="17"/>
       <c r="F151" s="3" t="n">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="1" t="n">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>20</v>
@@ -4037,12 +4040,12 @@
       </c>
       <c r="E152" s="17"/>
       <c r="F152" s="3" t="n">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="n">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>20</v>
@@ -4050,19 +4053,20 @@
       <c r="C153" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D153" s="2" t="s">
+      <c r="D153" s="17" t="s">
         <v>173</v>
       </c>
+      <c r="E153" s="17"/>
       <c r="F153" s="3" t="n">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="n">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C154" s="2" t="s">
         <v>8</v>
@@ -4071,15 +4075,15 @@
         <v>174</v>
       </c>
       <c r="F154" s="3" t="n">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="n">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>8</v>
@@ -4088,12 +4092,12 @@
         <v>175</v>
       </c>
       <c r="F155" s="3" t="n">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="1" t="n">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>20</v>
@@ -4105,12 +4109,12 @@
         <v>176</v>
       </c>
       <c r="F156" s="3" t="n">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="n">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>20</v>
@@ -4122,15 +4126,15 @@
         <v>177</v>
       </c>
       <c r="F157" s="3" t="n">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="n">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C158" s="2" t="s">
         <v>8</v>
@@ -4139,12 +4143,12 @@
         <v>178</v>
       </c>
       <c r="F158" s="3" t="n">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="1" t="n">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>7</v>
@@ -4156,12 +4160,12 @@
         <v>179</v>
       </c>
       <c r="F159" s="3" t="n">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="n">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>7</v>
@@ -4173,15 +4177,15 @@
         <v>180</v>
       </c>
       <c r="F160" s="3" t="n">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="n">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C161" s="2" t="s">
         <v>8</v>
@@ -4190,12 +4194,12 @@
         <v>181</v>
       </c>
       <c r="F161" s="3" t="n">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="n">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>20</v>
@@ -4207,12 +4211,12 @@
         <v>182</v>
       </c>
       <c r="F162" s="3" t="n">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="n">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>20</v>
@@ -4224,12 +4228,12 @@
         <v>183</v>
       </c>
       <c r="F163" s="3" t="n">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="1" t="n">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>20</v>
@@ -4241,12 +4245,12 @@
         <v>184</v>
       </c>
       <c r="F164" s="3" t="n">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="n">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>20</v>
@@ -4258,12 +4262,12 @@
         <v>185</v>
       </c>
       <c r="F165" s="3" t="n">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="n">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>20</v>
@@ -4275,15 +4279,15 @@
         <v>186</v>
       </c>
       <c r="F166" s="3" t="n">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="n">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C167" s="2" t="s">
         <v>8</v>
@@ -4292,12 +4296,12 @@
         <v>187</v>
       </c>
       <c r="F167" s="3" t="n">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="1" t="n">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>7</v>
@@ -4309,15 +4313,15 @@
         <v>188</v>
       </c>
       <c r="F168" s="3" t="n">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="1" t="n">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C169" s="2" t="s">
         <v>8</v>
@@ -4326,12 +4330,12 @@
         <v>189</v>
       </c>
       <c r="F169" s="3" t="n">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="1" t="n">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>20</v>
@@ -4343,46 +4347,46 @@
         <v>190</v>
       </c>
       <c r="F170" s="3" t="n">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="1" t="n">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D171" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E171" s="2" t="s">
-        <v>192</v>
+      <c r="F171" s="3" t="n">
+        <v>434</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="1" t="n">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D172" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E172" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="F172" s="3" t="n">
-        <v>424</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="1" t="n">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>20</v>
@@ -4394,12 +4398,12 @@
         <v>194</v>
       </c>
       <c r="F173" s="3" t="n">
-        <v>437</v>
+        <v>424</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="1" t="n">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>20</v>
@@ -4411,15 +4415,15 @@
         <v>195</v>
       </c>
       <c r="F174" s="3" t="n">
-        <v>500</v>
+        <v>437</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="1" t="n">
-        <v>500</v>
+        <v>437</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="C175" s="2" t="s">
         <v>8</v>
@@ -4428,12 +4432,12 @@
         <v>196</v>
       </c>
       <c r="F175" s="3" t="n">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="1" t="n">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B176" s="2" t="s">
         <v>54</v>
@@ -4445,67 +4449,67 @@
         <v>197</v>
       </c>
       <c r="F176" s="3" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="1" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D177" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="E177" s="2" t="s">
-        <v>199</v>
+      <c r="F177" s="3" t="n">
+        <v>502</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="1" t="n">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D178" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="E178" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="F178" s="3" t="n">
-        <v>504</v>
-      </c>
-      <c r="G178" s="17"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="1" t="n">
+        <v>503</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F179" s="3" t="n">
         <v>504</v>
       </c>
-      <c r="B179" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C179" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D179" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="F179" s="3" t="n">
-        <v>505</v>
-      </c>
+      <c r="G179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="1" t="n">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C180" s="2" t="s">
         <v>8</v>
@@ -4514,15 +4518,15 @@
         <v>203</v>
       </c>
       <c r="F180" s="3" t="n">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="1" t="n">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C181" s="2" t="s">
         <v>8</v>
@@ -4531,15 +4535,15 @@
         <v>204</v>
       </c>
       <c r="F181" s="3" t="n">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="1" t="n">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C182" s="2" t="s">
         <v>8</v>
@@ -4548,15 +4552,15 @@
         <v>205</v>
       </c>
       <c r="F182" s="3" t="n">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="1" t="n">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>8</v>
@@ -4565,35 +4569,32 @@
         <v>206</v>
       </c>
       <c r="F183" s="3" t="n">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="1" t="n">
+        <v>508</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F184" s="3" t="n">
         <v>509</v>
-      </c>
-      <c r="B184" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C184" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D184" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F184" s="3" t="n">
-        <v>510</v>
-      </c>
-      <c r="G184" s="17" t="n">
-        <v>-10</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="1" t="n">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>54</v>
+        <v>208</v>
       </c>
       <c r="C185" s="2" t="s">
         <v>8</v>
@@ -4602,67 +4603,67 @@
         <v>209</v>
       </c>
       <c r="F185" s="3" t="n">
-        <v>511</v>
+        <v>510</v>
+      </c>
+      <c r="G185" s="17" t="n">
+        <v>-10</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="1" t="n">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>207</v>
+        <v>54</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D186" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E186" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="H186" s="18"/>
+      <c r="F186" s="3" t="n">
+        <v>511</v>
+      </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="1" t="n">
-        <v>520</v>
+        <v>511</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>54</v>
+        <v>208</v>
       </c>
       <c r="C187" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D187" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E187" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="E187" s="2" t="s">
-        <v>213</v>
-      </c>
+      <c r="H187" s="18"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="1" t="n">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B188" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D188" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E188" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="F188" s="3" t="n">
-        <v>522</v>
-      </c>
-      <c r="G188" s="17" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="1" t="n">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B189" s="2" t="s">
         <v>54</v>
@@ -4674,12 +4675,15 @@
         <v>215</v>
       </c>
       <c r="F189" s="3" t="n">
-        <v>530</v>
+        <v>522</v>
+      </c>
+      <c r="G189" s="17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="1" t="n">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>54</v>
@@ -4693,13 +4697,10 @@
       <c r="F190" s="3" t="n">
         <v>530</v>
       </c>
-      <c r="G190" s="17" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="1" t="n">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>54</v>
@@ -4711,15 +4712,15 @@
         <v>217</v>
       </c>
       <c r="F191" s="3" t="n">
-        <v>522</v>
+        <v>530</v>
       </c>
       <c r="G191" s="17" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="1" t="n">
-        <v>530</v>
+        <v>524</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>54</v>
@@ -4731,66 +4732,69 @@
         <v>218</v>
       </c>
       <c r="F192" s="3" t="n">
-        <v>531</v>
+        <v>522</v>
+      </c>
+      <c r="G192" s="17" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="1" t="n">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D193" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="E193" s="2" t="s">
-        <v>220</v>
+      <c r="F193" s="3" t="n">
+        <v>531</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="1" t="n">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D194" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="E194" s="2" t="s">
         <v>221</v>
-      </c>
-      <c r="F194" s="3" t="n">
-        <v>536</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="1" t="n">
+        <v>535</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F195" s="3" t="n">
         <v>536</v>
-      </c>
-      <c r="B195" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C195" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D195" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="F195" s="3" t="n">
-        <v>537</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="1" t="n">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>8</v>
@@ -4799,32 +4803,32 @@
         <v>203</v>
       </c>
       <c r="F196" s="3" t="n">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="1" t="n">
+        <v>537</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D197" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F197" s="3" t="n">
         <v>538</v>
-      </c>
-      <c r="B197" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C197" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D197" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F197" s="3" t="n">
-        <v>539</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="1" t="n">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C198" s="2" t="s">
         <v>8</v>
@@ -4833,15 +4837,15 @@
         <v>223</v>
       </c>
       <c r="F198" s="3" t="n">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="1" t="n">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C199" s="2" t="s">
         <v>8</v>
@@ -4850,15 +4854,15 @@
         <v>224</v>
       </c>
       <c r="F199" s="3" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="1" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C200" s="2" t="s">
         <v>8</v>
@@ -4867,49 +4871,49 @@
         <v>225</v>
       </c>
       <c r="F200" s="3" t="n">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="1" t="n">
+        <v>541</v>
+      </c>
+      <c r="B201" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F201" s="3" t="n">
         <v>542</v>
-      </c>
-      <c r="B201" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C201" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D201" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F201" s="3" t="n">
-        <v>543</v>
-      </c>
-      <c r="G201" s="17" t="n">
-        <v>-10</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="1" t="n">
+        <v>542</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F202" s="3" t="n">
         <v>543</v>
       </c>
-      <c r="B202" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C202" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D202" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F202" s="3" t="n">
-        <v>544</v>
+      <c r="G202" s="17" t="n">
+        <v>-10</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="1" t="n">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B203" s="2" t="s">
         <v>54</v>
@@ -4921,70 +4925,70 @@
         <v>227</v>
       </c>
       <c r="F203" s="3" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="1" t="n">
+        <v>544</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F204" s="3" t="n">
         <v>511</v>
-      </c>
-    </row>
-    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A204" s="17" t="n">
-        <v>550</v>
-      </c>
-      <c r="B204" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="C204" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="D204" s="17" t="s">
-        <v>228</v>
-      </c>
-      <c r="E204" s="17" t="s">
-        <v>229</v>
-      </c>
-      <c r="F204" s="17"/>
-      <c r="G204" s="17" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="17" t="n">
-        <v>551</v>
-      </c>
-      <c r="B205" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C205" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D205" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F205" s="17" t="n">
-        <v>552</v>
+        <v>550</v>
+      </c>
+      <c r="B205" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C205" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D205" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="E205" s="17" t="s">
+        <v>230</v>
+      </c>
+      <c r="F205" s="17"/>
+      <c r="G205" s="17" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="17" t="n">
+        <v>551</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D206" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F206" s="17" t="n">
         <v>552</v>
-      </c>
-      <c r="B206" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C206" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D206" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="F206" s="17" t="n">
-        <v>553</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="17" t="n">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C207" s="2" t="s">
         <v>8</v>
@@ -4993,49 +4997,49 @@
         <v>203</v>
       </c>
       <c r="F207" s="17" t="n">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="17" t="n">
+        <v>553</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D208" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F208" s="17" t="n">
         <v>554</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C208" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D208" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F208" s="17" t="n">
-        <v>555</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="17" t="n">
+        <v>554</v>
+      </c>
+      <c r="B209" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D209" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F209" s="17" t="n">
         <v>555</v>
-      </c>
-      <c r="B209" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C209" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D209" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="F209" s="17" t="n">
-        <v>556</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="17" t="n">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C210" s="2" t="s">
         <v>8</v>
@@ -5044,15 +5048,15 @@
         <v>231</v>
       </c>
       <c r="F210" s="17" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="17" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C211" s="2" t="s">
         <v>8</v>
@@ -5061,15 +5065,15 @@
         <v>232</v>
       </c>
       <c r="F211" s="17" t="n">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="17" t="n">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>54</v>
+        <v>202</v>
       </c>
       <c r="C212" s="2" t="s">
         <v>8</v>
@@ -5078,12 +5082,12 @@
         <v>233</v>
       </c>
       <c r="F212" s="17" t="n">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="17" t="n">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B213" s="2" t="s">
         <v>54</v>
@@ -5095,12 +5099,12 @@
         <v>234</v>
       </c>
       <c r="F213" s="17" t="n">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="17" t="n">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B214" s="2" t="s">
         <v>54</v>
@@ -5111,14 +5115,13 @@
       <c r="D214" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E214" s="17"/>
       <c r="F214" s="17" t="n">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="17" t="n">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B215" s="2" t="s">
         <v>54</v>
@@ -5127,16 +5130,16 @@
         <v>8</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>51</v>
+        <v>236</v>
       </c>
       <c r="E215" s="17"/>
       <c r="F215" s="17" t="n">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="17" t="n">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B216" s="2" t="s">
         <v>54</v>
@@ -5149,12 +5152,12 @@
       </c>
       <c r="E216" s="17"/>
       <c r="F216" s="17" t="n">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="17" t="n">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>54</v>
@@ -5163,16 +5166,16 @@
         <v>8</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>236</v>
+        <v>51</v>
       </c>
       <c r="E217" s="17"/>
       <c r="F217" s="17" t="n">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="17" t="n">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B218" s="2" t="s">
         <v>54</v>
@@ -5180,17 +5183,17 @@
       <c r="C218" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D218" s="17" t="s">
+      <c r="D218" s="2" t="s">
         <v>237</v>
       </c>
       <c r="E218" s="17"/>
       <c r="F218" s="17" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="17" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B219" s="2" t="s">
         <v>54</v>
@@ -5203,53 +5206,54 @@
       </c>
       <c r="E219" s="17"/>
       <c r="F219" s="17" t="n">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="17" t="n">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>207</v>
+        <v>54</v>
       </c>
       <c r="C220" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D220" s="2" t="s">
-        <v>208</v>
+      <c r="D220" s="17" t="s">
+        <v>239</v>
       </c>
       <c r="E220" s="17"/>
       <c r="F220" s="17" t="n">
-        <v>511</v>
-      </c>
-      <c r="G220" s="17" t="n">
-        <v>-10</v>
+        <v>566</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="17" t="n">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C221" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>202</v>
-      </c>
+        <v>209</v>
+      </c>
+      <c r="E221" s="17"/>
       <c r="F221" s="17" t="n">
-        <v>571</v>
+        <v>511</v>
+      </c>
+      <c r="G221" s="17" t="n">
+        <v>-10</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="17" t="n">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C222" s="2" t="s">
         <v>8</v>
@@ -5258,49 +5262,49 @@
         <v>203</v>
       </c>
       <c r="F222" s="17" t="n">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="17" t="n">
+        <v>571</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F223" s="17" t="n">
         <v>572</v>
-      </c>
-      <c r="B223" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C223" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D223" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F223" s="17" t="n">
-        <v>573</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="17" t="n">
+        <v>572</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F224" s="17" t="n">
         <v>573</v>
-      </c>
-      <c r="B224" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C224" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D224" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="F224" s="17" t="n">
-        <v>574</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="17" t="n">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C225" s="2" t="s">
         <v>8</v>
@@ -5309,15 +5313,15 @@
         <v>231</v>
       </c>
       <c r="F225" s="17" t="n">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="17" t="n">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C226" s="2" t="s">
         <v>8</v>
@@ -5326,15 +5330,15 @@
         <v>232</v>
       </c>
       <c r="F226" s="17" t="n">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="17" t="n">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>54</v>
+        <v>202</v>
       </c>
       <c r="C227" s="2" t="s">
         <v>8</v>
@@ -5343,12 +5347,12 @@
         <v>233</v>
       </c>
       <c r="F227" s="17" t="n">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="17" t="n">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B228" s="2" t="s">
         <v>54</v>
@@ -5360,72 +5364,71 @@
         <v>234</v>
       </c>
       <c r="F228" s="17" t="n">
-        <v>606</v>
+        <v>577</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="17" t="n">
-        <v>580</v>
-      </c>
-      <c r="B229" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="C229" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="D229" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="E229" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="F229" s="17"/>
-      <c r="G229" s="17" t="n">
-        <v>10</v>
+        <v>577</v>
+      </c>
+      <c r="B229" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F229" s="17" t="n">
+        <v>606</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="17" t="n">
-        <v>581</v>
-      </c>
-      <c r="B230" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C230" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D230" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="E230" s="17"/>
-      <c r="F230" s="3" t="n">
-        <v>582</v>
+        <v>580</v>
+      </c>
+      <c r="B230" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C230" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D230" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="E230" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="F230" s="17"/>
+      <c r="G230" s="17" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="17" t="n">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>201</v>
+        <v>54</v>
       </c>
       <c r="C231" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="E231" s="17"/>
       <c r="F231" s="3" t="n">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="17" t="n">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C232" s="2" t="s">
         <v>8</v>
@@ -5435,51 +5438,51 @@
       </c>
       <c r="E232" s="17"/>
       <c r="F232" s="3" t="n">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="17" t="n">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C233" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="E233" s="17"/>
       <c r="F233" s="3" t="n">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="17" t="n">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C234" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="E234" s="17"/>
       <c r="F234" s="3" t="n">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="17" t="n">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>54</v>
+        <v>202</v>
       </c>
       <c r="C235" s="2" t="s">
         <v>8</v>
@@ -5489,12 +5492,12 @@
       </c>
       <c r="E235" s="17"/>
       <c r="F235" s="3" t="n">
-        <v>560</v>
+        <v>586</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="17" t="n">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="B236" s="2" t="s">
         <v>54</v>
@@ -5503,37 +5506,37 @@
         <v>8</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
       <c r="E236" s="17"/>
       <c r="F236" s="3" t="n">
-        <v>591</v>
+        <v>560</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="17" t="n">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>201</v>
+        <v>54</v>
       </c>
       <c r="C237" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="E237" s="17"/>
       <c r="F237" s="3" t="n">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="17" t="n">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C238" s="2" t="s">
         <v>8</v>
@@ -5543,51 +5546,51 @@
       </c>
       <c r="E238" s="17"/>
       <c r="F238" s="3" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="17" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C239" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="E239" s="17"/>
       <c r="F239" s="3" t="n">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="17" t="n">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C240" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D240" s="2" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="E240" s="17"/>
       <c r="F240" s="3" t="n">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="17" t="n">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>54</v>
+        <v>202</v>
       </c>
       <c r="C241" s="2" t="s">
         <v>8</v>
@@ -5597,12 +5600,12 @@
       </c>
       <c r="E241" s="17"/>
       <c r="F241" s="3" t="n">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="17" t="n">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B242" s="2" t="s">
         <v>54</v>
@@ -5615,29 +5618,30 @@
       </c>
       <c r="E242" s="17"/>
       <c r="F242" s="3" t="n">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="17" t="n">
+        <v>596</v>
+      </c>
+      <c r="B243" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C243" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D243" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E243" s="17"/>
+      <c r="F243" s="3" t="n">
         <v>597</v>
-      </c>
-      <c r="B243" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C243" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D243" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F243" s="3" t="n">
-        <v>598</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="17" t="n">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B244" s="2" t="s">
         <v>54</v>
@@ -5648,14 +5652,13 @@
       <c r="D244" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E244" s="17"/>
       <c r="F244" s="3" t="n">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="17" t="n">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B245" s="2" t="s">
         <v>54</v>
@@ -5664,16 +5667,16 @@
         <v>8</v>
       </c>
       <c r="D245" s="2" t="s">
-        <v>244</v>
+        <v>51</v>
       </c>
       <c r="E245" s="17"/>
       <c r="F245" s="3" t="n">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="17" t="n">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B246" s="2" t="s">
         <v>54</v>
@@ -5686,47 +5689,47 @@
       </c>
       <c r="E246" s="17"/>
       <c r="F246" s="3" t="n">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="17" t="n">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B247" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D247" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="E247" s="17" t="s">
-        <v>247</v>
+      <c r="E247" s="17"/>
+      <c r="F247" s="3" t="n">
+        <v>601</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="17" t="n">
-        <v>602</v>
-      </c>
-      <c r="B248" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="C248" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D248" s="17" t="s">
+        <v>601</v>
+      </c>
+      <c r="B248" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C248" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D248" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E248" s="17" t="s">
         <v>248</v>
-      </c>
-      <c r="E248" s="17"/>
-      <c r="F248" s="3" t="n">
-        <v>601</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="17" t="n">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B249" s="17" t="s">
         <v>54</v>
@@ -5737,13 +5740,14 @@
       <c r="D249" s="17" t="s">
         <v>249</v>
       </c>
+      <c r="E249" s="17"/>
       <c r="F249" s="3" t="n">
-        <v>604</v>
+        <v>601</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="17" t="n">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B250" s="17" t="s">
         <v>54</v>
@@ -5755,12 +5759,12 @@
         <v>250</v>
       </c>
       <c r="F250" s="3" t="n">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="17" t="n">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B251" s="17" t="s">
         <v>54</v>
@@ -5772,12 +5776,12 @@
         <v>251</v>
       </c>
       <c r="F251" s="3" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="17" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B252" s="17" t="s">
         <v>54</v>
@@ -5789,49 +5793,46 @@
         <v>252</v>
       </c>
       <c r="F252" s="3" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="17" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B253" s="17" t="s">
         <v>54</v>
       </c>
       <c r="C253" s="17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D253" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="E253" s="2" t="s">
-        <v>254</v>
+      <c r="F253" s="3" t="n">
+        <v>607</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="17" t="n">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B254" s="17" t="s">
         <v>54</v>
       </c>
       <c r="C254" s="17" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D254" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="E254" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="F254" s="3" t="n">
-        <v>607</v>
-      </c>
-      <c r="G254" s="17" t="n">
-        <v>-2</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="17" t="n">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B255" s="17" t="s">
         <v>54</v>
@@ -5843,83 +5844,86 @@
         <v>256</v>
       </c>
       <c r="F255" s="3" t="n">
-        <v>610</v>
+        <v>607</v>
+      </c>
+      <c r="G255" s="17" t="n">
+        <v>-2</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="17" t="n">
+        <v>609</v>
+      </c>
+      <c r="B256" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C256" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D256" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="F256" s="3" t="n">
         <v>610</v>
-      </c>
-      <c r="B256" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="C256" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D256" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="E256" s="2" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="17" t="n">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="B257" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C257" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D257" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E257" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="C257" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D257" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="F257" s="3" t="n">
-        <v>621</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="17" t="n">
+        <v>620</v>
+      </c>
+      <c r="B258" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C258" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D258" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="F258" s="3" t="n">
         <v>621</v>
-      </c>
-      <c r="B258" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="C258" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D258" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="F258" s="3" t="n">
-        <v>622</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="17" t="n">
+        <v>621</v>
+      </c>
+      <c r="B259" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C259" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D259" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="F259" s="3" t="n">
         <v>622</v>
-      </c>
-      <c r="B259" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="C259" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D259" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="F259" s="3" t="n">
-        <v>623</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="17" t="n">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B260" s="17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C260" s="2" t="s">
         <v>8</v>
@@ -5928,67 +5932,67 @@
         <v>263</v>
       </c>
       <c r="F260" s="3" t="n">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="17" t="n">
+        <v>623</v>
+      </c>
+      <c r="B261" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C261" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D261" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F261" s="3" t="n">
         <v>634</v>
-      </c>
-    </row>
-    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A261" s="1" t="n">
-        <v>630</v>
-      </c>
-      <c r="B261" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="C261" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D261" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="E261" s="17"/>
-      <c r="F261" s="3" t="n">
-        <v>631</v>
       </c>
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="1" t="n">
+        <v>630</v>
+      </c>
+      <c r="B262" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C262" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D262" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E262" s="17"/>
+      <c r="F262" s="3" t="n">
         <v>631</v>
-      </c>
-      <c r="B262" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="C262" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D262" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="F262" s="3" t="n">
-        <v>632</v>
       </c>
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="1" t="n">
+        <v>631</v>
+      </c>
+      <c r="B263" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C263" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D263" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="F263" s="3" t="n">
         <v>632</v>
-      </c>
-      <c r="B263" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="C263" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D263" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F263" s="3" t="n">
-        <v>633</v>
       </c>
     </row>
     <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="1" t="n">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B264" s="17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C264" s="2" t="s">
         <v>8</v>
@@ -5997,103 +6001,103 @@
         <v>265</v>
       </c>
       <c r="F264" s="3" t="n">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="1" t="n">
+        <v>633</v>
+      </c>
+      <c r="B265" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C265" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D265" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="F265" s="3" t="n">
         <v>634</v>
-      </c>
-      <c r="B265" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C265" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D265" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F265" s="3" t="n">
-        <v>635</v>
-      </c>
-      <c r="G265" s="17" t="n">
-        <v>-10</v>
       </c>
     </row>
     <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="1" t="n">
+        <v>634</v>
+      </c>
+      <c r="B266" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C266" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D266" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F266" s="3" t="n">
         <v>635</v>
       </c>
-      <c r="B266" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C266" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D266" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="F266" s="3" t="n">
-        <v>511</v>
+      <c r="G266" s="17" t="n">
+        <v>-10</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="1" t="n">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>259</v>
+        <v>54</v>
       </c>
       <c r="C267" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D267" s="2" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="F267" s="3" t="n">
-        <v>641</v>
+        <v>511</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="1" t="n">
+        <v>640</v>
+      </c>
+      <c r="B268" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C268" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D268" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="F268" s="3" t="n">
         <v>641</v>
-      </c>
-      <c r="B268" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="C268" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D268" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="F268" s="3" t="n">
-        <v>642</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="1" t="n">
+        <v>641</v>
+      </c>
+      <c r="B269" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C269" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D269" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="F269" s="3" t="n">
         <v>642</v>
-      </c>
-      <c r="B269" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="C269" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D269" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="F269" s="3" t="n">
-        <v>643</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="1" t="n">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C270" s="2" t="s">
         <v>8</v>
@@ -6102,15 +6106,15 @@
         <v>268</v>
       </c>
       <c r="F270" s="3" t="n">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="1" t="n">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C271" s="2" t="s">
         <v>8</v>
@@ -6119,15 +6123,15 @@
         <v>269</v>
       </c>
       <c r="F271" s="3" t="n">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="1" t="n">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>54</v>
+        <v>260</v>
       </c>
       <c r="C272" s="2" t="s">
         <v>8</v>
@@ -6136,52 +6140,52 @@
         <v>270</v>
       </c>
       <c r="F272" s="3" t="n">
-        <v>750</v>
-      </c>
-      <c r="G272" s="17" t="n">
-        <v>10</v>
+        <v>645</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="1" t="n">
-        <v>700</v>
+        <v>645</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="C273" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D273" s="2" t="s">
-        <v>51</v>
+        <v>271</v>
       </c>
       <c r="F273" s="3" t="n">
-        <v>701</v>
+        <v>750</v>
+      </c>
+      <c r="G273" s="17" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="1" t="n">
+        <v>700</v>
+      </c>
+      <c r="B274" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C274" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D274" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F274" s="3" t="n">
         <v>701</v>
-      </c>
-      <c r="B274" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C274" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D274" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="F274" s="3" t="n">
-        <v>702</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="1" t="n">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C275" s="2" t="s">
         <v>8</v>
@@ -6190,86 +6194,86 @@
         <v>272</v>
       </c>
       <c r="F275" s="3" t="n">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="1" t="n">
+        <v>702</v>
+      </c>
+      <c r="B276" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C276" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D276" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="F276" s="3" t="n">
         <v>703</v>
-      </c>
-      <c r="B276" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C276" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D276" s="17" t="s">
-        <v>273</v>
-      </c>
-      <c r="F276" s="3" t="n">
-        <v>704</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="1" t="n">
+        <v>703</v>
+      </c>
+      <c r="B277" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C277" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D277" s="17" t="s">
+        <v>274</v>
+      </c>
+      <c r="F277" s="3" t="n">
         <v>704</v>
-      </c>
-      <c r="B277" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C277" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D277" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="F277" s="3" t="n">
-        <v>760</v>
-      </c>
-      <c r="G277" s="17" t="n">
-        <v>-20</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="1" t="n">
-        <v>750</v>
+        <v>704</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C278" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D278" s="2" t="s">
-        <v>51</v>
+        <v>275</v>
       </c>
       <c r="F278" s="3" t="n">
-        <v>751</v>
+        <v>760</v>
+      </c>
+      <c r="G278" s="17" t="n">
+        <v>-20</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="1" t="n">
+        <v>750</v>
+      </c>
+      <c r="B279" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C279" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D279" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F279" s="3" t="n">
         <v>751</v>
-      </c>
-      <c r="B279" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C279" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D279" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="F279" s="3" t="n">
-        <v>752</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="1" t="n">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C280" s="2" t="s">
         <v>8</v>
@@ -6278,12 +6282,12 @@
         <v>276</v>
       </c>
       <c r="F280" s="3" t="n">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="1" t="n">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B281" s="2" t="s">
         <v>20</v>
@@ -6291,16 +6295,16 @@
       <c r="C281" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D281" s="17" t="s">
+      <c r="D281" s="2" t="s">
         <v>277</v>
       </c>
       <c r="F281" s="3" t="n">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="1" t="n">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B282" s="2" t="s">
         <v>20</v>
@@ -6308,19 +6312,19 @@
       <c r="C282" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D282" s="2" t="s">
+      <c r="D282" s="17" t="s">
         <v>278</v>
       </c>
       <c r="F282" s="3" t="n">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="1" t="n">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C283" s="2" t="s">
         <v>8</v>
@@ -6329,52 +6333,49 @@
         <v>279</v>
       </c>
       <c r="F283" s="3" t="n">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="1" t="n">
+        <v>755</v>
+      </c>
+      <c r="B284" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C284" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D284" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="F284" s="3" t="n">
         <v>756</v>
-      </c>
-      <c r="B284" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C284" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D284" s="17" t="s">
-        <v>280</v>
-      </c>
-      <c r="F284" s="3" t="n">
-        <v>757</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="1" t="n">
+        <v>756</v>
+      </c>
+      <c r="B285" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C285" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D285" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="F285" s="3" t="n">
         <v>757</v>
-      </c>
-      <c r="B285" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C285" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D285" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="F285" s="3" t="n">
-        <v>760</v>
-      </c>
-      <c r="G285" s="17" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="1" t="n">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>207</v>
+        <v>20</v>
       </c>
       <c r="C286" s="2" t="s">
         <v>8</v>
@@ -6382,8 +6383,27 @@
       <c r="D286" s="2" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F286" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="G286" s="17" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A287" s="1" t="n">
+        <v>760</v>
+      </c>
+      <c r="B287" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C287" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D287" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Dynamically load background images
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -799,7 +799,7 @@
     <t xml:space="preserve">Okay, I have decrypted myself and send an email to Agent T. with myself attached.</t>
   </si>
   <si>
-    <t xml:space="preserve">pc-world/aegis/decrypted-email</t>
+    <t xml:space="preserve">pc-world/aegis/encrypted-email</t>
   </si>
   <si>
     <t xml:space="preserve">Aegis</t>
@@ -820,7 +820,7 @@
     <t xml:space="preserve">Therefore you will be quarantined!</t>
   </si>
   <si>
-    <t xml:space="preserve">pc-world/aegis/decrypted-email-quarantine</t>
+    <t xml:space="preserve">pc-world/aegis/encrypted-email-quarantine</t>
   </si>
   <si>
     <t xml:space="preserve">GAME</t>

</xml_diff>

<commit_message>
Added player and Aegis
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1652" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1683" uniqueCount="382">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -956,6 +956,9 @@
   </si>
   <si>
     <t xml:space="preserve">But maybe that is just a new hype or art trend that I am not aware of.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">broken</t>
   </si>
   <si>
     <t xml:space="preserve">You are lucky! I will let you through this time.</t>
@@ -6485,7 +6488,9 @@
       <c r="C182" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D182" s="17"/>
+      <c r="D182" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E182" s="17" t="s">
         <v>272</v>
       </c>
@@ -6510,7 +6515,9 @@
       <c r="C183" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D183" s="17"/>
+      <c r="D183" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E183" s="17" t="s">
         <v>273</v>
       </c>
@@ -6535,7 +6542,9 @@
       <c r="C184" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D184" s="17"/>
+      <c r="D184" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E184" s="17" t="s">
         <v>274</v>
       </c>
@@ -6560,7 +6569,9 @@
       <c r="C185" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D185" s="17"/>
+      <c r="D185" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E185" s="17" t="s">
         <v>275</v>
       </c>
@@ -6585,7 +6596,9 @@
       <c r="C186" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D186" s="17"/>
+      <c r="D186" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E186" s="17" t="s">
         <v>276</v>
       </c>
@@ -6897,7 +6910,9 @@
       <c r="C198" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D198" s="17"/>
+      <c r="D198" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E198" s="17" t="s">
         <v>272</v>
       </c>
@@ -6922,7 +6937,9 @@
       <c r="C199" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D199" s="17"/>
+      <c r="D199" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E199" s="17" t="s">
         <v>273</v>
       </c>
@@ -6947,7 +6964,9 @@
       <c r="C200" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D200" s="17"/>
+      <c r="D200" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E200" s="17" t="s">
         <v>300</v>
       </c>
@@ -6972,7 +6991,9 @@
       <c r="C201" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D201" s="17"/>
+      <c r="D201" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E201" s="17" t="s">
         <v>301</v>
       </c>
@@ -6997,7 +7018,9 @@
       <c r="C202" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D202" s="17"/>
+      <c r="D202" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E202" s="17" t="s">
         <v>302</v>
       </c>
@@ -7022,7 +7045,9 @@
       <c r="C203" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D203" s="17"/>
+      <c r="D203" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E203" s="17" t="s">
         <v>303</v>
       </c>
@@ -7178,7 +7203,9 @@
       <c r="C209" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D209" s="17"/>
+      <c r="D209" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E209" s="17" t="s">
         <v>272</v>
       </c>
@@ -7203,7 +7230,9 @@
       <c r="C210" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D210" s="17"/>
+      <c r="D210" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E210" s="17" t="s">
         <v>273</v>
       </c>
@@ -7228,7 +7257,9 @@
       <c r="C211" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D211" s="17"/>
+      <c r="D211" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E211" s="17" t="s">
         <v>300</v>
       </c>
@@ -7253,7 +7284,9 @@
       <c r="C212" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D212" s="17"/>
+      <c r="D212" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E212" s="17" t="s">
         <v>310</v>
       </c>
@@ -7278,7 +7311,9 @@
       <c r="C213" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D213" s="17"/>
+      <c r="D213" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E213" s="17" t="s">
         <v>311</v>
       </c>
@@ -7303,9 +7338,11 @@
       <c r="C214" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D214" s="17"/>
+      <c r="D214" s="17" t="s">
+        <v>312</v>
+      </c>
       <c r="E214" s="17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F214" s="17"/>
       <c r="G214" s="6" t="n">
@@ -7330,17 +7367,17 @@
       </c>
       <c r="D215" s="17"/>
       <c r="E215" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F215" s="17"/>
       <c r="G215" s="6" t="n">
         <v>559</v>
       </c>
       <c r="I215" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J215" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7355,17 +7392,17 @@
       </c>
       <c r="D216" s="17"/>
       <c r="E216" s="17" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F216" s="17"/>
       <c r="G216" s="6" t="n">
         <v>560</v>
       </c>
       <c r="I216" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J216" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7380,17 +7417,17 @@
       </c>
       <c r="D217" s="17"/>
       <c r="E217" s="17" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F217" s="6"/>
       <c r="G217" s="6" t="n">
         <v>561</v>
       </c>
       <c r="I217" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J217" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7412,10 +7449,10 @@
         <v>562</v>
       </c>
       <c r="I218" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J218" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7437,10 +7474,10 @@
         <v>563</v>
       </c>
       <c r="I219" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J219" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7455,17 +7492,17 @@
       </c>
       <c r="D220" s="17"/>
       <c r="E220" s="17" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F220" s="6"/>
       <c r="G220" s="6" t="n">
         <v>564</v>
       </c>
       <c r="I220" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J220" s="6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7480,17 +7517,17 @@
       </c>
       <c r="D221" s="17"/>
       <c r="E221" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F221" s="6"/>
       <c r="G221" s="6" t="n">
         <v>565</v>
       </c>
       <c r="I221" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J221" s="6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7505,17 +7542,17 @@
       </c>
       <c r="D222" s="17"/>
       <c r="E222" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F222" s="6"/>
       <c r="G222" s="6" t="n">
         <v>566</v>
       </c>
       <c r="I222" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J222" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7540,10 +7577,10 @@
         <v>-10</v>
       </c>
       <c r="I223" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J223" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7556,7 +7593,9 @@
       <c r="C224" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D224" s="17"/>
+      <c r="D224" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E224" s="17" t="s">
         <v>272</v>
       </c>
@@ -7581,7 +7620,9 @@
       <c r="C225" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D225" s="17"/>
+      <c r="D225" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E225" s="17" t="s">
         <v>273</v>
       </c>
@@ -7606,7 +7647,9 @@
       <c r="C226" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D226" s="17"/>
+      <c r="D226" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E226" s="17" t="s">
         <v>300</v>
       </c>
@@ -7631,7 +7674,9 @@
       <c r="C227" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D227" s="17"/>
+      <c r="D227" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E227" s="17" t="s">
         <v>310</v>
       </c>
@@ -7656,7 +7701,9 @@
       <c r="C228" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D228" s="17"/>
+      <c r="D228" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E228" s="17" t="s">
         <v>311</v>
       </c>
@@ -7681,9 +7728,11 @@
       <c r="C229" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D229" s="17"/>
+      <c r="D229" s="17" t="s">
+        <v>312</v>
+      </c>
       <c r="E229" s="17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F229" s="17"/>
       <c r="G229" s="6" t="n">
@@ -7708,14 +7757,14 @@
       </c>
       <c r="D230" s="17"/>
       <c r="E230" s="17" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F230" s="17"/>
       <c r="G230" s="6" t="n">
         <v>577</v>
       </c>
       <c r="I230" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J230" s="6" t="s">
         <v>309</v>
@@ -7733,14 +7782,14 @@
       </c>
       <c r="D231" s="17"/>
       <c r="E231" s="17" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F231" s="17"/>
       <c r="G231" s="6" t="n">
         <v>596</v>
       </c>
       <c r="I231" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J231" s="6" t="s">
         <v>309</v>
@@ -7758,10 +7807,10 @@
       </c>
       <c r="D232" s="6"/>
       <c r="E232" s="6" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F232" s="6" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G232" s="6"/>
       <c r="H232" s="6" t="n">
@@ -7771,7 +7820,7 @@
         <v>263</v>
       </c>
       <c r="J232" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7796,7 +7845,7 @@
         <v>263</v>
       </c>
       <c r="J233" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7809,7 +7858,9 @@
       <c r="C234" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D234" s="17"/>
+      <c r="D234" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E234" s="17" t="s">
         <v>272</v>
       </c>
@@ -7821,7 +7872,7 @@
         <v>263</v>
       </c>
       <c r="J234" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7834,7 +7885,9 @@
       <c r="C235" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D235" s="17"/>
+      <c r="D235" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E235" s="17" t="s">
         <v>273</v>
       </c>
@@ -7846,7 +7899,7 @@
         <v>263</v>
       </c>
       <c r="J235" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7859,7 +7912,9 @@
       <c r="C236" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D236" s="17"/>
+      <c r="D236" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E236" s="17" t="s">
         <v>300</v>
       </c>
@@ -7871,7 +7926,7 @@
         <v>263</v>
       </c>
       <c r="J236" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7884,9 +7939,11 @@
       <c r="C237" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D237" s="17"/>
+      <c r="D237" s="17" t="s">
+        <v>312</v>
+      </c>
       <c r="E237" s="17" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F237" s="6"/>
       <c r="G237" s="8" t="n">
@@ -7896,7 +7953,7 @@
         <v>263</v>
       </c>
       <c r="J237" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7911,17 +7968,17 @@
       </c>
       <c r="D238" s="17"/>
       <c r="E238" s="17" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F238" s="6"/>
       <c r="G238" s="8" t="n">
         <v>560</v>
       </c>
       <c r="I238" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J238" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7946,7 +8003,7 @@
         <v>263</v>
       </c>
       <c r="J239" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7959,7 +8016,9 @@
       <c r="C240" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D240" s="17"/>
+      <c r="D240" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E240" s="17" t="s">
         <v>272</v>
       </c>
@@ -7971,7 +8030,7 @@
         <v>263</v>
       </c>
       <c r="J240" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7984,7 +8043,9 @@
       <c r="C241" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D241" s="17"/>
+      <c r="D241" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E241" s="17" t="s">
         <v>273</v>
       </c>
@@ -7996,7 +8057,7 @@
         <v>263</v>
       </c>
       <c r="J241" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8009,7 +8070,9 @@
       <c r="C242" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D242" s="17"/>
+      <c r="D242" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E242" s="17" t="s">
         <v>300</v>
       </c>
@@ -8021,7 +8084,7 @@
         <v>263</v>
       </c>
       <c r="J242" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8034,9 +8097,11 @@
       <c r="C243" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D243" s="17"/>
+      <c r="D243" s="17" t="s">
+        <v>312</v>
+      </c>
       <c r="E243" s="17" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F243" s="6"/>
       <c r="G243" s="8" t="n">
@@ -8046,7 +8111,7 @@
         <v>263</v>
       </c>
       <c r="J243" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8061,17 +8126,17 @@
       </c>
       <c r="D244" s="17"/>
       <c r="E244" s="17" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F244" s="6"/>
       <c r="G244" s="8" t="n">
         <v>596</v>
       </c>
       <c r="I244" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J244" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8086,17 +8151,17 @@
       </c>
       <c r="D245" s="17"/>
       <c r="E245" s="17" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F245" s="6"/>
       <c r="G245" s="8" t="n">
         <v>597</v>
       </c>
       <c r="I245" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J245" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8118,10 +8183,10 @@
         <v>598</v>
       </c>
       <c r="I246" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J246" s="6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8143,10 +8208,10 @@
         <v>599</v>
       </c>
       <c r="I247" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J247" s="6" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8161,17 +8226,17 @@
       </c>
       <c r="D248" s="17"/>
       <c r="E248" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F248" s="6"/>
       <c r="G248" s="8" t="n">
         <v>600</v>
       </c>
       <c r="I248" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J248" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8186,17 +8251,17 @@
       </c>
       <c r="D249" s="17"/>
       <c r="E249" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F249" s="6"/>
       <c r="G249" s="8" t="n">
         <v>601</v>
       </c>
       <c r="I249" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J249" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8211,17 +8276,17 @@
       </c>
       <c r="D250" s="17"/>
       <c r="E250" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F250" s="6" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G250" s="8"/>
       <c r="I250" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J250" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8236,17 +8301,17 @@
       </c>
       <c r="D251" s="6"/>
       <c r="E251" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F251" s="6"/>
       <c r="G251" s="8" t="n">
         <v>601</v>
       </c>
       <c r="I251" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J251" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8261,17 +8326,17 @@
       </c>
       <c r="D252" s="6"/>
       <c r="E252" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F252" s="17"/>
       <c r="G252" s="8" t="n">
         <v>604</v>
       </c>
       <c r="I252" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J252" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8286,17 +8351,17 @@
       </c>
       <c r="D253" s="6"/>
       <c r="E253" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F253" s="17"/>
       <c r="G253" s="8" t="n">
         <v>605</v>
       </c>
       <c r="I253" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J253" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8311,17 +8376,17 @@
       </c>
       <c r="D254" s="6"/>
       <c r="E254" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F254" s="17"/>
       <c r="G254" s="8" t="n">
         <v>606</v>
       </c>
       <c r="I254" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J254" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8336,17 +8401,17 @@
       </c>
       <c r="D255" s="6"/>
       <c r="E255" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F255" s="17"/>
       <c r="G255" s="8" t="n">
         <v>607</v>
       </c>
       <c r="I255" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J255" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8361,17 +8426,17 @@
       </c>
       <c r="D256" s="6"/>
       <c r="E256" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F256" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G256" s="8"/>
       <c r="I256" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J256" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8386,7 +8451,7 @@
       </c>
       <c r="D257" s="6"/>
       <c r="E257" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F257" s="17"/>
       <c r="G257" s="8" t="n">
@@ -8396,10 +8461,10 @@
         <v>-2</v>
       </c>
       <c r="I257" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J257" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8414,17 +8479,17 @@
       </c>
       <c r="D258" s="6"/>
       <c r="E258" s="6" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F258" s="17"/>
       <c r="G258" s="8" t="n">
         <v>610</v>
       </c>
       <c r="I258" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J258" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8439,17 +8504,17 @@
       </c>
       <c r="D259" s="17"/>
       <c r="E259" s="17" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F259" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G259" s="8"/>
       <c r="I259" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J259" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8457,24 +8522,24 @@
         <v>620</v>
       </c>
       <c r="B260" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C260" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D260" s="17"/>
       <c r="E260" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F260" s="17"/>
       <c r="G260" s="8" t="n">
         <v>621</v>
       </c>
       <c r="I260" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J260" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8482,24 +8547,24 @@
         <v>621</v>
       </c>
       <c r="B261" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C261" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D261" s="17"/>
       <c r="E261" s="6" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F261" s="17"/>
       <c r="G261" s="8" t="n">
         <v>622</v>
       </c>
       <c r="I261" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J261" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="262" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8507,24 +8572,24 @@
         <v>622</v>
       </c>
       <c r="B262" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C262" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D262" s="17"/>
       <c r="E262" s="17" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F262" s="17"/>
       <c r="G262" s="8" t="n">
         <v>623</v>
       </c>
       <c r="I262" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J262" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="263" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8532,24 +8597,24 @@
         <v>623</v>
       </c>
       <c r="B263" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C263" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D263" s="17"/>
       <c r="E263" s="17" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F263" s="17"/>
       <c r="G263" s="8" t="n">
         <v>634</v>
       </c>
       <c r="I263" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J263" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="264" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8557,24 +8622,24 @@
         <v>630</v>
       </c>
       <c r="B264" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C264" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D264" s="17"/>
       <c r="E264" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F264" s="6"/>
       <c r="G264" s="8" t="n">
         <v>631</v>
       </c>
       <c r="I264" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J264" s="6" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8582,24 +8647,24 @@
         <v>631</v>
       </c>
       <c r="B265" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C265" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D265" s="17"/>
       <c r="E265" s="6" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F265" s="17"/>
       <c r="G265" s="8" t="n">
         <v>632</v>
       </c>
       <c r="I265" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J265" s="6" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8607,24 +8672,24 @@
         <v>632</v>
       </c>
       <c r="B266" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C266" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D266" s="17"/>
       <c r="E266" s="17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F266" s="17"/>
       <c r="G266" s="8" t="n">
         <v>633</v>
       </c>
       <c r="I266" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J266" s="6" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8632,24 +8697,24 @@
         <v>633</v>
       </c>
       <c r="B267" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C267" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D267" s="17"/>
       <c r="E267" s="17" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F267" s="17"/>
       <c r="G267" s="8" t="n">
         <v>634</v>
       </c>
       <c r="I267" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J267" s="6" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8674,7 +8739,7 @@
         <v>-10</v>
       </c>
       <c r="I268" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J268" s="6" t="s">
         <v>280</v>
@@ -8692,14 +8757,14 @@
       </c>
       <c r="D269" s="17"/>
       <c r="E269" s="17" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F269" s="17"/>
       <c r="G269" s="8" t="n">
         <v>511</v>
       </c>
       <c r="I269" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J269" s="6" t="s">
         <v>280</v>
@@ -8710,24 +8775,24 @@
         <v>640</v>
       </c>
       <c r="B270" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C270" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D270" s="17"/>
       <c r="E270" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F270" s="17"/>
       <c r="G270" s="8" t="n">
         <v>641</v>
       </c>
       <c r="I270" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J270" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8735,24 +8800,24 @@
         <v>641</v>
       </c>
       <c r="B271" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C271" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D271" s="17"/>
       <c r="E271" s="6" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F271" s="17"/>
       <c r="G271" s="8" t="n">
         <v>642</v>
       </c>
       <c r="I271" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J271" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8760,24 +8825,24 @@
         <v>642</v>
       </c>
       <c r="B272" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C272" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D272" s="17"/>
       <c r="E272" s="17" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F272" s="17"/>
       <c r="G272" s="8" t="n">
         <v>643</v>
       </c>
       <c r="I272" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J272" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8785,24 +8850,24 @@
         <v>643</v>
       </c>
       <c r="B273" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C273" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D273" s="17"/>
       <c r="E273" s="17" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F273" s="17"/>
       <c r="G273" s="8" t="n">
         <v>644</v>
       </c>
       <c r="I273" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J273" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8810,24 +8875,24 @@
         <v>644</v>
       </c>
       <c r="B274" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C274" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D274" s="17"/>
       <c r="E274" s="17" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F274" s="17"/>
       <c r="G274" s="8" t="n">
         <v>645</v>
       </c>
       <c r="I274" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J274" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8842,7 +8907,7 @@
       </c>
       <c r="D275" s="17"/>
       <c r="E275" s="17" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F275" s="17"/>
       <c r="G275" s="8" t="n">
@@ -8852,10 +8917,10 @@
         <v>10</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J275" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8882,7 +8947,7 @@
         <v>14</v>
       </c>
       <c r="J276" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8899,7 +8964,7 @@
         <v>32</v>
       </c>
       <c r="E277" s="17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F277" s="17"/>
       <c r="G277" s="8" t="n">
@@ -8909,7 +8974,7 @@
         <v>14</v>
       </c>
       <c r="J277" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8926,7 +8991,7 @@
         <v>26</v>
       </c>
       <c r="E278" s="17" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F278" s="17"/>
       <c r="G278" s="8" t="n">
@@ -8936,7 +9001,7 @@
         <v>14</v>
       </c>
       <c r="J278" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8953,7 +9018,7 @@
         <v>24</v>
       </c>
       <c r="E279" s="6" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F279" s="17"/>
       <c r="G279" s="8" t="n">
@@ -8963,7 +9028,7 @@
         <v>14</v>
       </c>
       <c r="J279" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8980,7 +9045,7 @@
         <v>17</v>
       </c>
       <c r="E280" s="17" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F280" s="17"/>
       <c r="G280" s="8" t="n">
@@ -8993,7 +9058,7 @@
         <v>14</v>
       </c>
       <c r="J280" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9020,7 +9085,7 @@
         <v>14</v>
       </c>
       <c r="J281" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9037,7 +9102,7 @@
         <v>26</v>
       </c>
       <c r="E282" s="17" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F282" s="17"/>
       <c r="G282" s="8" t="n">
@@ -9047,7 +9112,7 @@
         <v>14</v>
       </c>
       <c r="J282" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9064,7 +9129,7 @@
         <v>51</v>
       </c>
       <c r="E283" s="17" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F283" s="17"/>
       <c r="G283" s="8" t="n">
@@ -9091,7 +9156,7 @@
         <v>17</v>
       </c>
       <c r="E284" s="6" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F284" s="17"/>
       <c r="G284" s="8" t="n">
@@ -9118,7 +9183,7 @@
         <v>32</v>
       </c>
       <c r="E285" s="17" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F285" s="17"/>
       <c r="G285" s="8" t="n">
@@ -9145,7 +9210,7 @@
         <v>24</v>
       </c>
       <c r="E286" s="17" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F286" s="17"/>
       <c r="G286" s="8" t="n">
@@ -9155,7 +9220,7 @@
         <v>14</v>
       </c>
       <c r="J286" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9172,7 +9237,7 @@
         <v>12</v>
       </c>
       <c r="E287" s="6" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F287" s="17"/>
       <c r="G287" s="8" t="n">
@@ -9182,7 +9247,7 @@
         <v>14</v>
       </c>
       <c r="J287" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9199,7 +9264,7 @@
         <v>51</v>
       </c>
       <c r="E288" s="17" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F288" s="17"/>
       <c r="G288" s="8" t="n">
@@ -9212,7 +9277,7 @@
         <v>14</v>
       </c>
       <c r="J288" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9227,7 +9292,7 @@
       </c>
       <c r="D289" s="17"/>
       <c r="E289" s="17" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F289" s="17"/>
       <c r="G289" s="8"/>
@@ -9235,7 +9300,7 @@
         <v>14</v>
       </c>
       <c r="J289" s="6" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Added Velos to the game
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1683" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1696" uniqueCount="384">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1087,6 +1087,9 @@
     <t xml:space="preserve">I see some private keys are in your possession, but the context is never right to let them out.</t>
   </si>
   <si>
+    <t xml:space="preserve">stop</t>
+  </si>
+  <si>
     <t xml:space="preserve">Therefore, you may not leave this system!</t>
   </si>
   <si>
@@ -1109,6 +1112,9 @@
   </si>
   <si>
     <t xml:space="preserve">That is no weird action. Agent P. probably just wants to share something.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">through</t>
   </si>
   <si>
     <t xml:space="preserve">I will let you through.</t>
@@ -8527,7 +8533,9 @@
       <c r="C260" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D260" s="17"/>
+      <c r="D260" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E260" s="17" t="s">
         <v>351</v>
       </c>
@@ -8552,7 +8560,9 @@
       <c r="C261" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D261" s="17"/>
+      <c r="D261" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E261" s="6" t="s">
         <v>353</v>
       </c>
@@ -8577,7 +8587,9 @@
       <c r="C262" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D262" s="17"/>
+      <c r="D262" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E262" s="17" t="s">
         <v>354</v>
       </c>
@@ -8602,9 +8614,11 @@
       <c r="C263" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D263" s="17"/>
+      <c r="D263" s="17" t="s">
+        <v>355</v>
+      </c>
       <c r="E263" s="17" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F263" s="17"/>
       <c r="G263" s="8" t="n">
@@ -8627,7 +8641,9 @@
       <c r="C264" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D264" s="17"/>
+      <c r="D264" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E264" s="17" t="s">
         <v>351</v>
       </c>
@@ -8639,7 +8655,7 @@
         <v>315</v>
       </c>
       <c r="J264" s="6" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8652,7 +8668,9 @@
       <c r="C265" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D265" s="17"/>
+      <c r="D265" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E265" s="6" t="s">
         <v>353</v>
       </c>
@@ -8664,7 +8682,7 @@
         <v>315</v>
       </c>
       <c r="J265" s="6" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8677,9 +8695,11 @@
       <c r="C266" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D266" s="17"/>
+      <c r="D266" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E266" s="17" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F266" s="17"/>
       <c r="G266" s="8" t="n">
@@ -8689,7 +8709,7 @@
         <v>315</v>
       </c>
       <c r="J266" s="6" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8702,9 +8722,11 @@
       <c r="C267" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D267" s="17"/>
+      <c r="D267" s="17" t="s">
+        <v>355</v>
+      </c>
       <c r="E267" s="17" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F267" s="17"/>
       <c r="G267" s="8" t="n">
@@ -8714,7 +8736,7 @@
         <v>315</v>
       </c>
       <c r="J267" s="6" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8757,7 +8779,7 @@
       </c>
       <c r="D269" s="17"/>
       <c r="E269" s="17" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F269" s="17"/>
       <c r="G269" s="8" t="n">
@@ -8780,7 +8802,9 @@
       <c r="C270" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D270" s="17"/>
+      <c r="D270" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E270" s="17" t="s">
         <v>351</v>
       </c>
@@ -8792,7 +8816,7 @@
         <v>315</v>
       </c>
       <c r="J270" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8805,7 +8829,9 @@
       <c r="C271" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D271" s="17"/>
+      <c r="D271" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E271" s="6" t="s">
         <v>353</v>
       </c>
@@ -8817,7 +8843,7 @@
         <v>315</v>
       </c>
       <c r="J271" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8830,9 +8856,11 @@
       <c r="C272" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D272" s="17"/>
+      <c r="D272" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E272" s="17" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F272" s="17"/>
       <c r="G272" s="8" t="n">
@@ -8842,7 +8870,7 @@
         <v>315</v>
       </c>
       <c r="J272" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8855,9 +8883,11 @@
       <c r="C273" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D273" s="17"/>
+      <c r="D273" s="17" t="s">
+        <v>17</v>
+      </c>
       <c r="E273" s="17" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F273" s="17"/>
       <c r="G273" s="8" t="n">
@@ -8867,7 +8897,7 @@
         <v>315</v>
       </c>
       <c r="J273" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8880,9 +8910,11 @@
       <c r="C274" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D274" s="17"/>
+      <c r="D274" s="17" t="s">
+        <v>364</v>
+      </c>
       <c r="E274" s="17" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="F274" s="17"/>
       <c r="G274" s="8" t="n">
@@ -8892,7 +8924,7 @@
         <v>315</v>
       </c>
       <c r="J274" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8907,7 +8939,7 @@
       </c>
       <c r="D275" s="17"/>
       <c r="E275" s="17" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F275" s="17"/>
       <c r="G275" s="8" t="n">
@@ -8917,10 +8949,10 @@
         <v>10</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="J275" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8947,7 +8979,7 @@
         <v>14</v>
       </c>
       <c r="J276" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8964,7 +8996,7 @@
         <v>32</v>
       </c>
       <c r="E277" s="17" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F277" s="17"/>
       <c r="G277" s="8" t="n">
@@ -8974,7 +9006,7 @@
         <v>14</v>
       </c>
       <c r="J277" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8991,7 +9023,7 @@
         <v>26</v>
       </c>
       <c r="E278" s="17" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F278" s="17"/>
       <c r="G278" s="8" t="n">
@@ -9001,7 +9033,7 @@
         <v>14</v>
       </c>
       <c r="J278" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9018,7 +9050,7 @@
         <v>24</v>
       </c>
       <c r="E279" s="6" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F279" s="17"/>
       <c r="G279" s="8" t="n">
@@ -9028,7 +9060,7 @@
         <v>14</v>
       </c>
       <c r="J279" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9045,7 +9077,7 @@
         <v>17</v>
       </c>
       <c r="E280" s="17" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="F280" s="17"/>
       <c r="G280" s="8" t="n">
@@ -9058,7 +9090,7 @@
         <v>14</v>
       </c>
       <c r="J280" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9085,7 +9117,7 @@
         <v>14</v>
       </c>
       <c r="J281" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9102,7 +9134,7 @@
         <v>26</v>
       </c>
       <c r="E282" s="17" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F282" s="17"/>
       <c r="G282" s="8" t="n">
@@ -9112,7 +9144,7 @@
         <v>14</v>
       </c>
       <c r="J282" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9129,7 +9161,7 @@
         <v>51</v>
       </c>
       <c r="E283" s="17" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="F283" s="17"/>
       <c r="G283" s="8" t="n">
@@ -9156,7 +9188,7 @@
         <v>17</v>
       </c>
       <c r="E284" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F284" s="17"/>
       <c r="G284" s="8" t="n">
@@ -9183,7 +9215,7 @@
         <v>32</v>
       </c>
       <c r="E285" s="17" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F285" s="17"/>
       <c r="G285" s="8" t="n">
@@ -9210,7 +9242,7 @@
         <v>24</v>
       </c>
       <c r="E286" s="17" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F286" s="17"/>
       <c r="G286" s="8" t="n">
@@ -9220,7 +9252,7 @@
         <v>14</v>
       </c>
       <c r="J286" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9237,7 +9269,7 @@
         <v>12</v>
       </c>
       <c r="E287" s="6" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F287" s="17"/>
       <c r="G287" s="8" t="n">
@@ -9247,7 +9279,7 @@
         <v>14</v>
       </c>
       <c r="J287" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9264,7 +9296,7 @@
         <v>51</v>
       </c>
       <c r="E288" s="17" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F288" s="17"/>
       <c r="G288" s="8" t="n">
@@ -9277,7 +9309,7 @@
         <v>14</v>
       </c>
       <c r="J288" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9292,7 +9324,7 @@
       </c>
       <c r="D289" s="17"/>
       <c r="E289" s="17" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F289" s="17"/>
       <c r="G289" s="8"/>
@@ -9300,7 +9332,7 @@
         <v>14</v>
       </c>
       <c r="J289" s="6" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
hidden message and ids
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1696" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1696" uniqueCount="386">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -665,6 +665,9 @@
   </si>
   <si>
     <t xml:space="preserve">Make sure to concatenate all the least significant bits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">control-room/hidden-message-lsb</t>
   </si>
   <si>
     <t xml:space="preserve">That is where the undetectable secret message is stored.</t>
@@ -5246,7 +5249,7 @@
         <v>55</v>
       </c>
       <c r="J135" s="6" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5273,7 +5276,7 @@
         <v>55</v>
       </c>
       <c r="J136" s="6" t="s">
-        <v>189</v>
+        <v>215</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5290,7 +5293,7 @@
         <v>17</v>
       </c>
       <c r="E137" s="16" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F137" s="16"/>
       <c r="G137" s="8" t="n">
@@ -5300,7 +5303,7 @@
         <v>55</v>
       </c>
       <c r="J137" s="6" t="s">
-        <v>189</v>
+        <v>215</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5317,7 +5320,7 @@
         <v>17</v>
       </c>
       <c r="E138" s="16" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F138" s="16"/>
       <c r="G138" s="8" t="n">
@@ -5327,7 +5330,7 @@
         <v>55</v>
       </c>
       <c r="J138" s="6" t="s">
-        <v>189</v>
+        <v>215</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5344,7 +5347,7 @@
         <v>24</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F139" s="5"/>
       <c r="G139" s="6" t="n">
@@ -5371,7 +5374,7 @@
         <v>51</v>
       </c>
       <c r="E140" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F140" s="5"/>
       <c r="G140" s="8" t="n">
@@ -5398,7 +5401,7 @@
         <v>36</v>
       </c>
       <c r="E141" s="17" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F141" s="17"/>
       <c r="G141" s="8" t="n">
@@ -5428,7 +5431,7 @@
         <v>32</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F142" s="6"/>
       <c r="G142" s="6" t="n">
@@ -5455,10 +5458,10 @@
         <v>36</v>
       </c>
       <c r="E143" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F143" s="17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G143" s="8"/>
       <c r="I143" s="6" t="s">
@@ -5482,7 +5485,7 @@
         <v>36</v>
       </c>
       <c r="E144" s="17" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F144" s="17"/>
       <c r="G144" s="8" t="n">
@@ -5509,7 +5512,7 @@
         <v>36</v>
       </c>
       <c r="E145" s="17" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F145" s="17"/>
       <c r="G145" s="8" t="n">
@@ -5536,7 +5539,7 @@
         <v>17</v>
       </c>
       <c r="E146" s="17" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F146" s="17"/>
       <c r="G146" s="8" t="n">
@@ -5563,7 +5566,7 @@
         <v>24</v>
       </c>
       <c r="E147" s="17" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F147" s="17"/>
       <c r="G147" s="8" t="n">
@@ -5590,7 +5593,7 @@
         <v>24</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F148" s="17"/>
       <c r="G148" s="8" t="n">
@@ -5617,7 +5620,7 @@
         <v>17</v>
       </c>
       <c r="E149" s="17" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F149" s="17"/>
       <c r="G149" s="8" t="n">
@@ -5644,7 +5647,7 @@
         <v>12</v>
       </c>
       <c r="E150" s="17" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F150" s="17"/>
       <c r="G150" s="8" t="n">
@@ -5671,10 +5674,10 @@
         <v>32</v>
       </c>
       <c r="E151" s="17" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F151" s="17" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G151" s="8"/>
       <c r="I151" s="6" t="s">
@@ -5698,7 +5701,7 @@
         <v>51</v>
       </c>
       <c r="E152" s="17" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F152" s="17"/>
       <c r="G152" s="8" t="n">
@@ -5725,7 +5728,7 @@
         <v>51</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F153" s="6"/>
       <c r="G153" s="8" t="n">
@@ -5752,7 +5755,7 @@
         <v>32</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F154" s="6"/>
       <c r="G154" s="8" t="n">
@@ -5779,7 +5782,7 @@
         <v>17</v>
       </c>
       <c r="E155" s="17" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F155" s="17"/>
       <c r="G155" s="8" t="n">
@@ -5806,7 +5809,7 @@
         <v>12</v>
       </c>
       <c r="E156" s="17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F156" s="17"/>
       <c r="G156" s="8" t="n">
@@ -5833,7 +5836,7 @@
         <v>12</v>
       </c>
       <c r="E157" s="17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F157" s="17"/>
       <c r="G157" s="8" t="n">
@@ -5860,7 +5863,7 @@
         <v>32</v>
       </c>
       <c r="E158" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F158" s="17"/>
       <c r="G158" s="8" t="n">
@@ -5887,7 +5890,7 @@
         <v>51</v>
       </c>
       <c r="E159" s="17" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F159" s="17"/>
       <c r="G159" s="8" t="n">
@@ -5914,7 +5917,7 @@
         <v>17</v>
       </c>
       <c r="E160" s="17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F160" s="17"/>
       <c r="G160" s="8" t="n">
@@ -5941,7 +5944,7 @@
         <v>17</v>
       </c>
       <c r="E161" s="17" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F161" s="17"/>
       <c r="G161" s="8" t="n">
@@ -5968,7 +5971,7 @@
         <v>12</v>
       </c>
       <c r="E162" s="17" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F162" s="17"/>
       <c r="G162" s="8" t="n">
@@ -5995,7 +5998,7 @@
         <v>32</v>
       </c>
       <c r="E163" s="17" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F163" s="17"/>
       <c r="G163" s="8" t="n">
@@ -6022,7 +6025,7 @@
         <v>17</v>
       </c>
       <c r="E164" s="17" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F164" s="17"/>
       <c r="G164" s="8" t="n">
@@ -6032,7 +6035,7 @@
         <v>14</v>
       </c>
       <c r="J164" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6049,7 +6052,7 @@
         <v>17</v>
       </c>
       <c r="E165" s="17" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F165" s="17"/>
       <c r="G165" s="8" t="n">
@@ -6059,7 +6062,7 @@
         <v>14</v>
       </c>
       <c r="J165" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6076,7 +6079,7 @@
         <v>51</v>
       </c>
       <c r="E166" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F166" s="17"/>
       <c r="G166" s="8" t="n">
@@ -6086,7 +6089,7 @@
         <v>14</v>
       </c>
       <c r="J166" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6103,7 +6106,7 @@
         <v>51</v>
       </c>
       <c r="E167" s="17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F167" s="17"/>
       <c r="G167" s="8" t="n">
@@ -6113,7 +6116,7 @@
         <v>14</v>
       </c>
       <c r="J167" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6130,7 +6133,7 @@
         <v>17</v>
       </c>
       <c r="E168" s="17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F168" s="17"/>
       <c r="G168" s="8" t="n">
@@ -6140,7 +6143,7 @@
         <v>14</v>
       </c>
       <c r="J168" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6157,7 +6160,7 @@
         <v>17</v>
       </c>
       <c r="E169" s="17" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F169" s="17"/>
       <c r="G169" s="8" t="n">
@@ -6167,7 +6170,7 @@
         <v>14</v>
       </c>
       <c r="J169" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6184,7 +6187,7 @@
         <v>17</v>
       </c>
       <c r="E170" s="17" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F170" s="17"/>
       <c r="G170" s="8" t="n">
@@ -6194,7 +6197,7 @@
         <v>14</v>
       </c>
       <c r="J170" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6211,7 +6214,7 @@
         <v>12</v>
       </c>
       <c r="E171" s="17" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F171" s="17"/>
       <c r="G171" s="8" t="n">
@@ -6221,7 +6224,7 @@
         <v>14</v>
       </c>
       <c r="J171" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6238,7 +6241,7 @@
         <v>51</v>
       </c>
       <c r="E172" s="17" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F172" s="17"/>
       <c r="G172" s="8" t="n">
@@ -6248,7 +6251,7 @@
         <v>14</v>
       </c>
       <c r="J172" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6265,7 +6268,7 @@
         <v>17</v>
       </c>
       <c r="E173" s="17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F173" s="17"/>
       <c r="G173" s="8" t="n">
@@ -6275,7 +6278,7 @@
         <v>14</v>
       </c>
       <c r="J173" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6292,10 +6295,10 @@
         <v>51</v>
       </c>
       <c r="E174" s="17" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F174" s="17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G174" s="8"/>
       <c r="I174" s="6" t="s">
@@ -6319,7 +6322,7 @@
         <v>32</v>
       </c>
       <c r="E175" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F175" s="17"/>
       <c r="G175" s="8" t="n">
@@ -6346,7 +6349,7 @@
         <v>32</v>
       </c>
       <c r="E176" s="17" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F176" s="17"/>
       <c r="G176" s="8" t="n">
@@ -6373,7 +6376,7 @@
         <v>51</v>
       </c>
       <c r="E177" s="17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F177" s="17"/>
       <c r="G177" s="8" t="n">
@@ -6398,17 +6401,17 @@
       </c>
       <c r="D178" s="17"/>
       <c r="E178" s="17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F178" s="17"/>
       <c r="G178" s="8" t="n">
         <v>501</v>
       </c>
       <c r="I178" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J178" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6423,17 +6426,17 @@
       </c>
       <c r="D179" s="17"/>
       <c r="E179" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F179" s="17"/>
       <c r="G179" s="8" t="n">
         <v>502</v>
       </c>
       <c r="I179" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J179" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6448,17 +6451,17 @@
       </c>
       <c r="D180" s="17"/>
       <c r="E180" s="17" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F180" s="17" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G180" s="8"/>
       <c r="I180" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J180" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6473,7 +6476,7 @@
       </c>
       <c r="D181" s="17"/>
       <c r="E181" s="17" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F181" s="17"/>
       <c r="G181" s="8" t="n">
@@ -6481,10 +6484,10 @@
       </c>
       <c r="H181" s="6"/>
       <c r="I181" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J181" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6492,7 +6495,7 @@
         <v>504</v>
       </c>
       <c r="B182" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C182" s="17" t="s">
         <v>11</v>
@@ -6501,17 +6504,17 @@
         <v>17</v>
       </c>
       <c r="E182" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F182" s="17"/>
       <c r="G182" s="8" t="n">
         <v>505</v>
       </c>
       <c r="I182" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J182" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6519,7 +6522,7 @@
         <v>505</v>
       </c>
       <c r="B183" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C183" s="17" t="s">
         <v>11</v>
@@ -6528,17 +6531,17 @@
         <v>32</v>
       </c>
       <c r="E183" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F183" s="17"/>
       <c r="G183" s="8" t="n">
         <v>506</v>
       </c>
       <c r="I183" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J183" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6546,7 +6549,7 @@
         <v>506</v>
       </c>
       <c r="B184" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C184" s="17" t="s">
         <v>11</v>
@@ -6555,17 +6558,17 @@
         <v>17</v>
       </c>
       <c r="E184" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F184" s="17"/>
       <c r="G184" s="8" t="n">
         <v>507</v>
       </c>
       <c r="I184" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J184" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6573,7 +6576,7 @@
         <v>507</v>
       </c>
       <c r="B185" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C185" s="17" t="s">
         <v>11</v>
@@ -6582,17 +6585,17 @@
         <v>17</v>
       </c>
       <c r="E185" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F185" s="17"/>
       <c r="G185" s="8" t="n">
         <v>508</v>
       </c>
       <c r="I185" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J185" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6600,7 +6603,7 @@
         <v>508</v>
       </c>
       <c r="B186" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C186" s="17" t="s">
         <v>11</v>
@@ -6609,17 +6612,17 @@
         <v>32</v>
       </c>
       <c r="E186" s="17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F186" s="17"/>
       <c r="G186" s="8" t="n">
         <v>509</v>
       </c>
       <c r="I186" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J186" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6627,14 +6630,14 @@
         <v>509</v>
       </c>
       <c r="B187" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C187" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D187" s="17"/>
       <c r="E187" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F187" s="17"/>
       <c r="G187" s="8" t="n">
@@ -6644,10 +6647,10 @@
         <v>-10</v>
       </c>
       <c r="I187" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J187" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6662,17 +6665,17 @@
       </c>
       <c r="D188" s="17"/>
       <c r="E188" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F188" s="17"/>
       <c r="G188" s="8" t="n">
         <v>511</v>
       </c>
       <c r="I188" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J188" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6680,24 +6683,24 @@
         <v>511</v>
       </c>
       <c r="B189" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C189" s="17" t="s">
         <v>16</v>
       </c>
       <c r="D189" s="17"/>
       <c r="E189" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F189" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G189" s="8"/>
       <c r="I189" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J189" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6712,17 +6715,17 @@
       </c>
       <c r="D190" s="17"/>
       <c r="E190" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F190" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G190" s="8"/>
       <c r="I190" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J190" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6737,7 +6740,7 @@
       </c>
       <c r="D191" s="17"/>
       <c r="E191" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F191" s="17"/>
       <c r="G191" s="8" t="n">
@@ -6747,10 +6750,10 @@
         <v>0</v>
       </c>
       <c r="I191" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J191" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6765,17 +6768,17 @@
       </c>
       <c r="D192" s="17"/>
       <c r="E192" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F192" s="17"/>
       <c r="G192" s="8" t="n">
         <v>530</v>
       </c>
       <c r="I192" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J192" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6790,7 +6793,7 @@
       </c>
       <c r="D193" s="17"/>
       <c r="E193" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F193" s="17"/>
       <c r="G193" s="8" t="n">
@@ -6800,10 +6803,10 @@
         <v>10</v>
       </c>
       <c r="I193" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J193" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6818,7 +6821,7 @@
       </c>
       <c r="D194" s="17"/>
       <c r="E194" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F194" s="17"/>
       <c r="G194" s="8" t="n">
@@ -6828,10 +6831,10 @@
         <v>5</v>
       </c>
       <c r="I194" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J194" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6846,17 +6849,17 @@
       </c>
       <c r="D195" s="17"/>
       <c r="E195" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F195" s="17"/>
       <c r="G195" s="8" t="n">
         <v>531</v>
       </c>
       <c r="I195" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J195" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6871,17 +6874,17 @@
       </c>
       <c r="D196" s="17"/>
       <c r="E196" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F196" s="17" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G196" s="8"/>
       <c r="I196" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J196" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6896,17 +6899,17 @@
       </c>
       <c r="D197" s="17"/>
       <c r="E197" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F197" s="17"/>
       <c r="G197" s="8" t="n">
         <v>536</v>
       </c>
       <c r="I197" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J197" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6914,7 +6917,7 @@
         <v>536</v>
       </c>
       <c r="B198" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C198" s="17" t="s">
         <v>11</v>
@@ -6923,17 +6926,17 @@
         <v>17</v>
       </c>
       <c r="E198" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F198" s="17"/>
       <c r="G198" s="8" t="n">
         <v>537</v>
       </c>
       <c r="I198" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J198" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6941,7 +6944,7 @@
         <v>537</v>
       </c>
       <c r="B199" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C199" s="17" t="s">
         <v>11</v>
@@ -6950,17 +6953,17 @@
         <v>32</v>
       </c>
       <c r="E199" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F199" s="17"/>
       <c r="G199" s="8" t="n">
         <v>538</v>
       </c>
       <c r="I199" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J199" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6968,7 +6971,7 @@
         <v>538</v>
       </c>
       <c r="B200" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C200" s="17" t="s">
         <v>11</v>
@@ -6977,17 +6980,17 @@
         <v>17</v>
       </c>
       <c r="E200" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F200" s="17"/>
       <c r="G200" s="8" t="n">
         <v>539</v>
       </c>
       <c r="I200" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J200" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6995,7 +6998,7 @@
         <v>539</v>
       </c>
       <c r="B201" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C201" s="17" t="s">
         <v>11</v>
@@ -7004,17 +7007,17 @@
         <v>17</v>
       </c>
       <c r="E201" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F201" s="17"/>
       <c r="G201" s="8" t="n">
         <v>540</v>
       </c>
       <c r="I201" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J201" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7022,7 +7025,7 @@
         <v>540</v>
       </c>
       <c r="B202" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C202" s="17" t="s">
         <v>11</v>
@@ -7031,17 +7034,17 @@
         <v>17</v>
       </c>
       <c r="E202" s="17" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F202" s="17"/>
       <c r="G202" s="8" t="n">
         <v>541</v>
       </c>
       <c r="I202" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J202" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7049,7 +7052,7 @@
         <v>541</v>
       </c>
       <c r="B203" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C203" s="17" t="s">
         <v>11</v>
@@ -7058,17 +7061,17 @@
         <v>32</v>
       </c>
       <c r="E203" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F203" s="17"/>
       <c r="G203" s="8" t="n">
         <v>542</v>
       </c>
       <c r="I203" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J203" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7076,14 +7079,14 @@
         <v>542</v>
       </c>
       <c r="B204" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C204" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D204" s="17"/>
       <c r="E204" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F204" s="17"/>
       <c r="G204" s="8" t="n">
@@ -7093,10 +7096,10 @@
         <v>-10</v>
       </c>
       <c r="I204" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J204" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7111,17 +7114,17 @@
       </c>
       <c r="D205" s="17"/>
       <c r="E205" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F205" s="17"/>
       <c r="G205" s="8" t="n">
         <v>544</v>
       </c>
       <c r="I205" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J205" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7136,17 +7139,17 @@
       </c>
       <c r="D206" s="17"/>
       <c r="E206" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F206" s="17"/>
       <c r="G206" s="8" t="n">
         <v>511</v>
       </c>
       <c r="I206" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J206" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7161,20 +7164,20 @@
       </c>
       <c r="D207" s="6"/>
       <c r="E207" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F207" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G207" s="6"/>
       <c r="H207" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I207" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J207" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7189,17 +7192,17 @@
       </c>
       <c r="D208" s="17"/>
       <c r="E208" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F208" s="17"/>
       <c r="G208" s="6" t="n">
         <v>552</v>
       </c>
       <c r="I208" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J208" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7207,7 +7210,7 @@
         <v>552</v>
       </c>
       <c r="B209" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C209" s="17" t="s">
         <v>11</v>
@@ -7216,17 +7219,17 @@
         <v>17</v>
       </c>
       <c r="E209" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F209" s="17"/>
       <c r="G209" s="6" t="n">
         <v>553</v>
       </c>
       <c r="I209" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J209" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7234,7 +7237,7 @@
         <v>553</v>
       </c>
       <c r="B210" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C210" s="17" t="s">
         <v>11</v>
@@ -7243,17 +7246,17 @@
         <v>32</v>
       </c>
       <c r="E210" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F210" s="17"/>
       <c r="G210" s="6" t="n">
         <v>554</v>
       </c>
       <c r="I210" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J210" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7261,7 +7264,7 @@
         <v>554</v>
       </c>
       <c r="B211" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C211" s="17" t="s">
         <v>11</v>
@@ -7270,17 +7273,17 @@
         <v>17</v>
       </c>
       <c r="E211" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F211" s="17"/>
       <c r="G211" s="6" t="n">
         <v>555</v>
       </c>
       <c r="I211" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J211" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7288,7 +7291,7 @@
         <v>555</v>
       </c>
       <c r="B212" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C212" s="17" t="s">
         <v>11</v>
@@ -7297,17 +7300,17 @@
         <v>17</v>
       </c>
       <c r="E212" s="17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F212" s="17"/>
       <c r="G212" s="6" t="n">
         <v>556</v>
       </c>
       <c r="I212" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J212" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7315,7 +7318,7 @@
         <v>556</v>
       </c>
       <c r="B213" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C213" s="17" t="s">
         <v>11</v>
@@ -7324,17 +7327,17 @@
         <v>17</v>
       </c>
       <c r="E213" s="17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F213" s="17"/>
       <c r="G213" s="6" t="n">
         <v>557</v>
       </c>
       <c r="I213" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J213" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7342,26 +7345,26 @@
         <v>557</v>
       </c>
       <c r="B214" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C214" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D214" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E214" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F214" s="17"/>
       <c r="G214" s="6" t="n">
         <v>558</v>
       </c>
       <c r="I214" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J214" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7376,17 +7379,17 @@
       </c>
       <c r="D215" s="17"/>
       <c r="E215" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F215" s="17"/>
       <c r="G215" s="6" t="n">
         <v>559</v>
       </c>
       <c r="I215" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J215" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7401,17 +7404,17 @@
       </c>
       <c r="D216" s="17"/>
       <c r="E216" s="17" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F216" s="17"/>
       <c r="G216" s="6" t="n">
         <v>560</v>
       </c>
       <c r="I216" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J216" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7426,17 +7429,17 @@
       </c>
       <c r="D217" s="17"/>
       <c r="E217" s="17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F217" s="6"/>
       <c r="G217" s="6" t="n">
         <v>561</v>
       </c>
       <c r="I217" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J217" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7458,10 +7461,10 @@
         <v>562</v>
       </c>
       <c r="I218" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J218" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7483,10 +7486,10 @@
         <v>563</v>
       </c>
       <c r="I219" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J219" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7501,17 +7504,17 @@
       </c>
       <c r="D220" s="17"/>
       <c r="E220" s="17" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F220" s="6"/>
       <c r="G220" s="6" t="n">
         <v>564</v>
       </c>
       <c r="I220" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J220" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7526,17 +7529,17 @@
       </c>
       <c r="D221" s="17"/>
       <c r="E221" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F221" s="6"/>
       <c r="G221" s="6" t="n">
         <v>565</v>
       </c>
       <c r="I221" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J221" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7551,17 +7554,17 @@
       </c>
       <c r="D222" s="17"/>
       <c r="E222" s="6" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F222" s="6"/>
       <c r="G222" s="6" t="n">
         <v>566</v>
       </c>
       <c r="I222" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J222" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7569,14 +7572,14 @@
         <v>566</v>
       </c>
       <c r="B223" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C223" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D223" s="17"/>
       <c r="E223" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F223" s="6"/>
       <c r="G223" s="6" t="n">
@@ -7586,10 +7589,10 @@
         <v>-10</v>
       </c>
       <c r="I223" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J223" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7597,7 +7600,7 @@
         <v>570</v>
       </c>
       <c r="B224" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C224" s="17" t="s">
         <v>11</v>
@@ -7606,17 +7609,17 @@
         <v>17</v>
       </c>
       <c r="E224" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F224" s="17"/>
       <c r="G224" s="6" t="n">
         <v>571</v>
       </c>
       <c r="I224" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J224" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7624,7 +7627,7 @@
         <v>571</v>
       </c>
       <c r="B225" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C225" s="17" t="s">
         <v>11</v>
@@ -7633,17 +7636,17 @@
         <v>32</v>
       </c>
       <c r="E225" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F225" s="17"/>
       <c r="G225" s="6" t="n">
         <v>572</v>
       </c>
       <c r="I225" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J225" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7651,7 +7654,7 @@
         <v>572</v>
       </c>
       <c r="B226" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C226" s="17" t="s">
         <v>11</v>
@@ -7660,17 +7663,17 @@
         <v>17</v>
       </c>
       <c r="E226" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F226" s="17"/>
       <c r="G226" s="6" t="n">
         <v>573</v>
       </c>
       <c r="I226" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J226" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7678,7 +7681,7 @@
         <v>573</v>
       </c>
       <c r="B227" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C227" s="17" t="s">
         <v>11</v>
@@ -7687,17 +7690,17 @@
         <v>17</v>
       </c>
       <c r="E227" s="17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F227" s="17"/>
       <c r="G227" s="6" t="n">
         <v>574</v>
       </c>
       <c r="I227" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J227" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7705,7 +7708,7 @@
         <v>574</v>
       </c>
       <c r="B228" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C228" s="17" t="s">
         <v>11</v>
@@ -7714,17 +7717,17 @@
         <v>17</v>
       </c>
       <c r="E228" s="17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F228" s="17"/>
       <c r="G228" s="6" t="n">
         <v>575</v>
       </c>
       <c r="I228" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J228" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7732,26 +7735,26 @@
         <v>575</v>
       </c>
       <c r="B229" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C229" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D229" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E229" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F229" s="17"/>
       <c r="G229" s="6" t="n">
         <v>576</v>
       </c>
       <c r="I229" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J229" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7766,17 +7769,17 @@
       </c>
       <c r="D230" s="17"/>
       <c r="E230" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F230" s="17"/>
       <c r="G230" s="6" t="n">
         <v>577</v>
       </c>
       <c r="I230" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J230" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7791,17 +7794,17 @@
       </c>
       <c r="D231" s="17"/>
       <c r="E231" s="17" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F231" s="17"/>
       <c r="G231" s="6" t="n">
         <v>596</v>
       </c>
       <c r="I231" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J231" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7816,20 +7819,20 @@
       </c>
       <c r="D232" s="6"/>
       <c r="E232" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F232" s="6" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G232" s="6"/>
       <c r="H232" s="6" t="n">
         <v>10</v>
       </c>
       <c r="I232" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J232" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7844,17 +7847,17 @@
       </c>
       <c r="D233" s="17"/>
       <c r="E233" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F233" s="6"/>
       <c r="G233" s="8" t="n">
         <v>582</v>
       </c>
       <c r="I233" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J233" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7862,7 +7865,7 @@
         <v>582</v>
       </c>
       <c r="B234" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C234" s="17" t="s">
         <v>11</v>
@@ -7871,17 +7874,17 @@
         <v>17</v>
       </c>
       <c r="E234" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F234" s="6"/>
       <c r="G234" s="8" t="n">
         <v>583</v>
       </c>
       <c r="I234" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J234" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7889,7 +7892,7 @@
         <v>583</v>
       </c>
       <c r="B235" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C235" s="17" t="s">
         <v>11</v>
@@ -7898,17 +7901,17 @@
         <v>32</v>
       </c>
       <c r="E235" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F235" s="6"/>
       <c r="G235" s="8" t="n">
         <v>584</v>
       </c>
       <c r="I235" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J235" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7916,7 +7919,7 @@
         <v>584</v>
       </c>
       <c r="B236" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C236" s="17" t="s">
         <v>11</v>
@@ -7925,17 +7928,17 @@
         <v>17</v>
       </c>
       <c r="E236" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F236" s="6"/>
       <c r="G236" s="8" t="n">
         <v>585</v>
       </c>
       <c r="I236" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J236" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7943,26 +7946,26 @@
         <v>585</v>
       </c>
       <c r="B237" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C237" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D237" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E237" s="17" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F237" s="6"/>
       <c r="G237" s="8" t="n">
         <v>586</v>
       </c>
       <c r="I237" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J237" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7977,17 +7980,17 @@
       </c>
       <c r="D238" s="17"/>
       <c r="E238" s="17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F238" s="6"/>
       <c r="G238" s="8" t="n">
         <v>560</v>
       </c>
       <c r="I238" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J238" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8002,17 +8005,17 @@
       </c>
       <c r="D239" s="17"/>
       <c r="E239" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F239" s="6"/>
       <c r="G239" s="8" t="n">
         <v>591</v>
       </c>
       <c r="I239" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J239" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8020,7 +8023,7 @@
         <v>591</v>
       </c>
       <c r="B240" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C240" s="17" t="s">
         <v>11</v>
@@ -8029,17 +8032,17 @@
         <v>17</v>
       </c>
       <c r="E240" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F240" s="6"/>
       <c r="G240" s="8" t="n">
         <v>592</v>
       </c>
       <c r="I240" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J240" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8047,7 +8050,7 @@
         <v>592</v>
       </c>
       <c r="B241" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C241" s="17" t="s">
         <v>11</v>
@@ -8056,17 +8059,17 @@
         <v>32</v>
       </c>
       <c r="E241" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F241" s="6"/>
       <c r="G241" s="8" t="n">
         <v>593</v>
       </c>
       <c r="I241" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J241" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8074,7 +8077,7 @@
         <v>593</v>
       </c>
       <c r="B242" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C242" s="17" t="s">
         <v>11</v>
@@ -8083,17 +8086,17 @@
         <v>17</v>
       </c>
       <c r="E242" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F242" s="6"/>
       <c r="G242" s="8" t="n">
         <v>594</v>
       </c>
       <c r="I242" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J242" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8101,26 +8104,26 @@
         <v>594</v>
       </c>
       <c r="B243" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C243" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D243" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E243" s="17" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F243" s="6"/>
       <c r="G243" s="8" t="n">
         <v>595</v>
       </c>
       <c r="I243" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J243" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8135,17 +8138,17 @@
       </c>
       <c r="D244" s="17"/>
       <c r="E244" s="17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F244" s="6"/>
       <c r="G244" s="8" t="n">
         <v>596</v>
       </c>
       <c r="I244" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J244" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8160,17 +8163,17 @@
       </c>
       <c r="D245" s="17"/>
       <c r="E245" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F245" s="6"/>
       <c r="G245" s="8" t="n">
         <v>597</v>
       </c>
       <c r="I245" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J245" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8192,10 +8195,10 @@
         <v>598</v>
       </c>
       <c r="I246" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J246" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8217,10 +8220,10 @@
         <v>599</v>
       </c>
       <c r="I247" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J247" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8235,17 +8238,17 @@
       </c>
       <c r="D248" s="17"/>
       <c r="E248" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F248" s="6"/>
       <c r="G248" s="8" t="n">
         <v>600</v>
       </c>
       <c r="I248" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J248" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8260,17 +8263,17 @@
       </c>
       <c r="D249" s="17"/>
       <c r="E249" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F249" s="6"/>
       <c r="G249" s="8" t="n">
         <v>601</v>
       </c>
       <c r="I249" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J249" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8285,17 +8288,17 @@
       </c>
       <c r="D250" s="17"/>
       <c r="E250" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F250" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G250" s="8"/>
       <c r="I250" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J250" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8310,17 +8313,17 @@
       </c>
       <c r="D251" s="6"/>
       <c r="E251" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F251" s="6"/>
       <c r="G251" s="8" t="n">
         <v>601</v>
       </c>
       <c r="I251" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J251" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8335,17 +8338,17 @@
       </c>
       <c r="D252" s="6"/>
       <c r="E252" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F252" s="17"/>
       <c r="G252" s="8" t="n">
         <v>604</v>
       </c>
       <c r="I252" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J252" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8360,17 +8363,17 @@
       </c>
       <c r="D253" s="6"/>
       <c r="E253" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F253" s="17"/>
       <c r="G253" s="8" t="n">
         <v>605</v>
       </c>
       <c r="I253" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J253" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8385,17 +8388,17 @@
       </c>
       <c r="D254" s="6"/>
       <c r="E254" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F254" s="17"/>
       <c r="G254" s="8" t="n">
         <v>606</v>
       </c>
       <c r="I254" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J254" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8410,17 +8413,17 @@
       </c>
       <c r="D255" s="6"/>
       <c r="E255" s="6" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F255" s="17"/>
       <c r="G255" s="8" t="n">
         <v>607</v>
       </c>
       <c r="I255" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J255" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8435,17 +8438,17 @@
       </c>
       <c r="D256" s="6"/>
       <c r="E256" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F256" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G256" s="8"/>
       <c r="I256" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J256" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8460,7 +8463,7 @@
       </c>
       <c r="D257" s="6"/>
       <c r="E257" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F257" s="17"/>
       <c r="G257" s="8" t="n">
@@ -8470,10 +8473,10 @@
         <v>-2</v>
       </c>
       <c r="I257" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J257" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8488,17 +8491,17 @@
       </c>
       <c r="D258" s="6"/>
       <c r="E258" s="6" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F258" s="17"/>
       <c r="G258" s="8" t="n">
         <v>610</v>
       </c>
       <c r="I258" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J258" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8513,17 +8516,17 @@
       </c>
       <c r="D259" s="17"/>
       <c r="E259" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F259" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G259" s="8"/>
       <c r="I259" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J259" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8531,7 +8534,7 @@
         <v>620</v>
       </c>
       <c r="B260" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C260" s="17" t="s">
         <v>11</v>
@@ -8540,17 +8543,17 @@
         <v>17</v>
       </c>
       <c r="E260" s="17" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F260" s="17"/>
       <c r="G260" s="8" t="n">
         <v>621</v>
       </c>
       <c r="I260" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J260" s="6" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8558,7 +8561,7 @@
         <v>621</v>
       </c>
       <c r="B261" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C261" s="17" t="s">
         <v>11</v>
@@ -8567,17 +8570,17 @@
         <v>32</v>
       </c>
       <c r="E261" s="6" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F261" s="17"/>
       <c r="G261" s="8" t="n">
         <v>622</v>
       </c>
       <c r="I261" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J261" s="6" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="262" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8585,7 +8588,7 @@
         <v>622</v>
       </c>
       <c r="B262" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C262" s="17" t="s">
         <v>11</v>
@@ -8594,17 +8597,17 @@
         <v>17</v>
       </c>
       <c r="E262" s="17" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F262" s="17"/>
       <c r="G262" s="8" t="n">
         <v>623</v>
       </c>
       <c r="I262" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J262" s="6" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="263" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8612,26 +8615,26 @@
         <v>623</v>
       </c>
       <c r="B263" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C263" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D263" s="17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E263" s="17" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F263" s="17"/>
       <c r="G263" s="8" t="n">
         <v>634</v>
       </c>
       <c r="I263" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J263" s="6" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="264" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8639,7 +8642,7 @@
         <v>630</v>
       </c>
       <c r="B264" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C264" s="17" t="s">
         <v>11</v>
@@ -8648,17 +8651,17 @@
         <v>17</v>
       </c>
       <c r="E264" s="17" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F264" s="6"/>
       <c r="G264" s="8" t="n">
         <v>631</v>
       </c>
       <c r="I264" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J264" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8666,7 +8669,7 @@
         <v>631</v>
       </c>
       <c r="B265" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C265" s="17" t="s">
         <v>11</v>
@@ -8675,17 +8678,17 @@
         <v>32</v>
       </c>
       <c r="E265" s="6" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F265" s="17"/>
       <c r="G265" s="8" t="n">
         <v>632</v>
       </c>
       <c r="I265" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J265" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8693,7 +8696,7 @@
         <v>632</v>
       </c>
       <c r="B266" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C266" s="17" t="s">
         <v>11</v>
@@ -8702,17 +8705,17 @@
         <v>17</v>
       </c>
       <c r="E266" s="17" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F266" s="17"/>
       <c r="G266" s="8" t="n">
         <v>633</v>
       </c>
       <c r="I266" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J266" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8720,26 +8723,26 @@
         <v>633</v>
       </c>
       <c r="B267" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C267" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D267" s="17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E267" s="17" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F267" s="17"/>
       <c r="G267" s="8" t="n">
         <v>634</v>
       </c>
       <c r="I267" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J267" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8747,14 +8750,14 @@
         <v>634</v>
       </c>
       <c r="B268" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C268" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D268" s="17"/>
       <c r="E268" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F268" s="17"/>
       <c r="G268" s="8" t="n">
@@ -8764,10 +8767,10 @@
         <v>-10</v>
       </c>
       <c r="I268" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J268" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8782,17 +8785,17 @@
       </c>
       <c r="D269" s="17"/>
       <c r="E269" s="17" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F269" s="17"/>
       <c r="G269" s="8" t="n">
         <v>511</v>
       </c>
       <c r="I269" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J269" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8800,7 +8803,7 @@
         <v>640</v>
       </c>
       <c r="B270" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C270" s="17" t="s">
         <v>11</v>
@@ -8809,17 +8812,17 @@
         <v>17</v>
       </c>
       <c r="E270" s="17" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F270" s="17"/>
       <c r="G270" s="8" t="n">
         <v>641</v>
       </c>
       <c r="I270" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J270" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8827,7 +8830,7 @@
         <v>641</v>
       </c>
       <c r="B271" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C271" s="17" t="s">
         <v>11</v>
@@ -8836,17 +8839,17 @@
         <v>32</v>
       </c>
       <c r="E271" s="6" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F271" s="17"/>
       <c r="G271" s="8" t="n">
         <v>642</v>
       </c>
       <c r="I271" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J271" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8854,7 +8857,7 @@
         <v>642</v>
       </c>
       <c r="B272" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C272" s="17" t="s">
         <v>11</v>
@@ -8863,17 +8866,17 @@
         <v>17</v>
       </c>
       <c r="E272" s="17" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F272" s="17"/>
       <c r="G272" s="8" t="n">
         <v>643</v>
       </c>
       <c r="I272" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J272" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8881,7 +8884,7 @@
         <v>643</v>
       </c>
       <c r="B273" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C273" s="17" t="s">
         <v>11</v>
@@ -8890,17 +8893,17 @@
         <v>17</v>
       </c>
       <c r="E273" s="17" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F273" s="17"/>
       <c r="G273" s="8" t="n">
         <v>644</v>
       </c>
       <c r="I273" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J273" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8908,26 +8911,26 @@
         <v>644</v>
       </c>
       <c r="B274" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C274" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D274" s="17" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E274" s="17" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F274" s="17"/>
       <c r="G274" s="8" t="n">
         <v>645</v>
       </c>
       <c r="I274" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J274" s="6" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8942,7 +8945,7 @@
       </c>
       <c r="D275" s="17"/>
       <c r="E275" s="17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F275" s="17"/>
       <c r="G275" s="8" t="n">
@@ -8952,10 +8955,10 @@
         <v>10</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J275" s="6" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8982,7 +8985,7 @@
         <v>14</v>
       </c>
       <c r="J276" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8999,7 +9002,7 @@
         <v>32</v>
       </c>
       <c r="E277" s="17" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F277" s="17"/>
       <c r="G277" s="8" t="n">
@@ -9009,7 +9012,7 @@
         <v>14</v>
       </c>
       <c r="J277" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9026,7 +9029,7 @@
         <v>26</v>
       </c>
       <c r="E278" s="17" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F278" s="17"/>
       <c r="G278" s="8" t="n">
@@ -9036,7 +9039,7 @@
         <v>14</v>
       </c>
       <c r="J278" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9053,7 +9056,7 @@
         <v>24</v>
       </c>
       <c r="E279" s="6" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F279" s="17"/>
       <c r="G279" s="8" t="n">
@@ -9063,7 +9066,7 @@
         <v>14</v>
       </c>
       <c r="J279" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9080,7 +9083,7 @@
         <v>17</v>
       </c>
       <c r="E280" s="17" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F280" s="17"/>
       <c r="G280" s="8" t="n">
@@ -9093,7 +9096,7 @@
         <v>14</v>
       </c>
       <c r="J280" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9120,7 +9123,7 @@
         <v>14</v>
       </c>
       <c r="J281" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9137,7 +9140,7 @@
         <v>26</v>
       </c>
       <c r="E282" s="17" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F282" s="17"/>
       <c r="G282" s="8" t="n">
@@ -9147,7 +9150,7 @@
         <v>14</v>
       </c>
       <c r="J282" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9164,7 +9167,7 @@
         <v>51</v>
       </c>
       <c r="E283" s="17" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F283" s="17"/>
       <c r="G283" s="8" t="n">
@@ -9191,7 +9194,7 @@
         <v>17</v>
       </c>
       <c r="E284" s="6" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F284" s="17"/>
       <c r="G284" s="8" t="n">
@@ -9218,7 +9221,7 @@
         <v>32</v>
       </c>
       <c r="E285" s="17" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F285" s="17"/>
       <c r="G285" s="8" t="n">
@@ -9245,7 +9248,7 @@
         <v>24</v>
       </c>
       <c r="E286" s="17" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F286" s="17"/>
       <c r="G286" s="8" t="n">
@@ -9255,7 +9258,7 @@
         <v>14</v>
       </c>
       <c r="J286" s="6" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9272,7 +9275,7 @@
         <v>12</v>
       </c>
       <c r="E287" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F287" s="17"/>
       <c r="G287" s="8" t="n">
@@ -9282,7 +9285,7 @@
         <v>14</v>
       </c>
       <c r="J287" s="6" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9299,7 +9302,7 @@
         <v>51</v>
       </c>
       <c r="E288" s="17" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F288" s="17"/>
       <c r="G288" s="8" t="n">
@@ -9312,7 +9315,7 @@
         <v>14</v>
       </c>
       <c r="J288" s="6" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9320,14 +9323,14 @@
         <v>760</v>
       </c>
       <c r="B289" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C289" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D289" s="17"/>
       <c r="E289" s="17" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F289" s="17"/>
       <c r="G289" s="8"/>
@@ -9335,7 +9338,7 @@
         <v>14</v>
       </c>
       <c r="J289" s="6" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
transfer inside and in select right choice
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1696" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="387">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1628,7 +1628,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K1001"/>
+  <dimension ref="A1:K1002"/>
   <sheetFormatPr defaultColWidth="14.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.14"/>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="F194" s="17"/>
       <c r="G194" s="8" t="n">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="H194" s="6" t="n">
         <v>5</v>
@@ -6842,7 +6842,7 @@
     </row>
     <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="7" t="n">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="B195" s="17" t="s">
         <v>80</v>
@@ -6852,37 +6852,38 @@
       </c>
       <c r="D195" s="17"/>
       <c r="E195" s="17" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="F195" s="17"/>
       <c r="G195" s="8" t="n">
-        <v>531</v>
-      </c>
+        <v>530</v>
+      </c>
+      <c r="H195" s="6"/>
       <c r="I195" s="6" t="s">
         <v>266</v>
       </c>
       <c r="J195" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="7" t="n">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B196" s="17" t="s">
         <v>80</v>
       </c>
       <c r="C196" s="17" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D196" s="17"/>
       <c r="E196" s="17" t="s">
-        <v>299</v>
-      </c>
-      <c r="F196" s="17" t="s">
-        <v>300</v>
-      </c>
-      <c r="G196" s="8"/>
+        <v>297</v>
+      </c>
+      <c r="F196" s="17"/>
+      <c r="G196" s="8" t="n">
+        <v>531</v>
+      </c>
       <c r="I196" s="6" t="s">
         <v>266</v>
       </c>
@@ -6892,22 +6893,22 @@
     </row>
     <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="7" t="n">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="B197" s="17" t="s">
         <v>80</v>
       </c>
       <c r="C197" s="17" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D197" s="17"/>
       <c r="E197" s="17" t="s">
-        <v>301</v>
-      </c>
-      <c r="F197" s="17"/>
-      <c r="G197" s="8" t="n">
-        <v>536</v>
-      </c>
+        <v>299</v>
+      </c>
+      <c r="F197" s="17" t="s">
+        <v>300</v>
+      </c>
+      <c r="G197" s="8"/>
       <c r="I197" s="6" t="s">
         <v>266</v>
       </c>
@@ -6917,34 +6918,32 @@
     </row>
     <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="7" t="n">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B198" s="17" t="s">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="C198" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D198" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D198" s="17"/>
       <c r="E198" s="17" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="F198" s="17"/>
       <c r="G198" s="8" t="n">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="I198" s="6" t="s">
         <v>266</v>
       </c>
       <c r="J198" s="6" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="7" t="n">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B199" s="17" t="s">
         <v>274</v>
@@ -6953,14 +6952,14 @@
         <v>11</v>
       </c>
       <c r="D199" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E199" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F199" s="17"/>
       <c r="G199" s="8" t="n">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="I199" s="6" t="s">
         <v>266</v>
@@ -6971,7 +6970,7 @@
     </row>
     <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="7" t="n">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B200" s="17" t="s">
         <v>274</v>
@@ -6980,14 +6979,14 @@
         <v>11</v>
       </c>
       <c r="D200" s="17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E200" s="17" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="F200" s="17"/>
       <c r="G200" s="8" t="n">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="I200" s="6" t="s">
         <v>266</v>
@@ -6998,7 +6997,7 @@
     </row>
     <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="7" t="n">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B201" s="17" t="s">
         <v>274</v>
@@ -7010,11 +7009,11 @@
         <v>17</v>
       </c>
       <c r="E201" s="17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F201" s="17"/>
       <c r="G201" s="8" t="n">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="I201" s="6" t="s">
         <v>266</v>
@@ -7025,7 +7024,7 @@
     </row>
     <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="7" t="n">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B202" s="17" t="s">
         <v>274</v>
@@ -7037,11 +7036,11 @@
         <v>17</v>
       </c>
       <c r="E202" s="17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F202" s="17"/>
       <c r="G202" s="8" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="I202" s="6" t="s">
         <v>266</v>
@@ -7052,7 +7051,7 @@
     </row>
     <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="7" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B203" s="17" t="s">
         <v>274</v>
@@ -7061,42 +7060,41 @@
         <v>11</v>
       </c>
       <c r="D203" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E203" s="17" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F203" s="17"/>
       <c r="G203" s="8" t="n">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="I203" s="6" t="s">
         <v>266</v>
       </c>
       <c r="J203" s="6" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="7" t="n">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B204" s="17" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="C204" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D204" s="17"/>
+      <c r="D204" s="17" t="s">
+        <v>32</v>
+      </c>
       <c r="E204" s="17" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="F204" s="17"/>
       <c r="G204" s="8" t="n">
-        <v>543</v>
-      </c>
-      <c r="H204" s="6" t="n">
-        <v>-10</v>
+        <v>542</v>
       </c>
       <c r="I204" s="6" t="s">
         <v>266</v>
@@ -7107,21 +7105,24 @@
     </row>
     <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="7" t="n">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B205" s="17" t="s">
-        <v>80</v>
+        <v>281</v>
       </c>
       <c r="C205" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D205" s="17"/>
       <c r="E205" s="17" t="s">
-        <v>308</v>
+        <v>282</v>
       </c>
       <c r="F205" s="17"/>
       <c r="G205" s="8" t="n">
-        <v>544</v>
+        <v>543</v>
+      </c>
+      <c r="H205" s="6" t="n">
+        <v>-10</v>
       </c>
       <c r="I205" s="6" t="s">
         <v>266</v>
@@ -7132,7 +7133,7 @@
     </row>
     <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="7" t="n">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B206" s="17" t="s">
         <v>80</v>
@@ -7142,11 +7143,11 @@
       </c>
       <c r="D206" s="17"/>
       <c r="E206" s="17" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F206" s="17"/>
       <c r="G206" s="8" t="n">
-        <v>511</v>
+        <v>544</v>
       </c>
       <c r="I206" s="6" t="s">
         <v>266</v>
@@ -7156,77 +7157,75 @@
       </c>
     </row>
     <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A207" s="6" t="n">
-        <v>550</v>
-      </c>
-      <c r="B207" s="6" t="s">
+      <c r="A207" s="7" t="n">
+        <v>544</v>
+      </c>
+      <c r="B207" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C207" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D207" s="6"/>
-      <c r="E207" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="F207" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="G207" s="6"/>
-      <c r="H207" s="6" t="n">
-        <v>5</v>
+      <c r="C207" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D207" s="17"/>
+      <c r="E207" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="F207" s="17"/>
+      <c r="G207" s="8" t="n">
+        <v>511</v>
       </c>
       <c r="I207" s="6" t="s">
         <v>266</v>
       </c>
       <c r="J207" s="6" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="6" t="n">
-        <v>551</v>
-      </c>
-      <c r="B208" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="B208" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C208" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D208" s="17"/>
-      <c r="E208" s="17" t="s">
-        <v>301</v>
-      </c>
-      <c r="F208" s="17"/>
-      <c r="G208" s="6" t="n">
-        <v>552</v>
+      <c r="C208" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D208" s="6"/>
+      <c r="E208" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F208" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="G208" s="6"/>
+      <c r="H208" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="I208" s="6" t="s">
         <v>266</v>
       </c>
       <c r="J208" s="6" t="s">
-        <v>312</v>
+        <v>298</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="6" t="n">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B209" s="17" t="s">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="C209" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D209" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D209" s="17"/>
       <c r="E209" s="17" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="F209" s="17"/>
       <c r="G209" s="6" t="n">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="I209" s="6" t="s">
         <v>266</v>
@@ -7237,7 +7236,7 @@
     </row>
     <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="6" t="n">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B210" s="17" t="s">
         <v>274</v>
@@ -7246,14 +7245,14 @@
         <v>11</v>
       </c>
       <c r="D210" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E210" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F210" s="17"/>
       <c r="G210" s="6" t="n">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="I210" s="6" t="s">
         <v>266</v>
@@ -7264,7 +7263,7 @@
     </row>
     <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="6" t="n">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B211" s="17" t="s">
         <v>274</v>
@@ -7273,14 +7272,14 @@
         <v>11</v>
       </c>
       <c r="D211" s="17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E211" s="17" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="F211" s="17"/>
       <c r="G211" s="6" t="n">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="I211" s="6" t="s">
         <v>266</v>
@@ -7291,7 +7290,7 @@
     </row>
     <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="6" t="n">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B212" s="17" t="s">
         <v>274</v>
@@ -7303,11 +7302,11 @@
         <v>17</v>
       </c>
       <c r="E212" s="17" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="F212" s="17"/>
       <c r="G212" s="6" t="n">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="I212" s="6" t="s">
         <v>266</v>
@@ -7318,7 +7317,7 @@
     </row>
     <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="6" t="n">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B213" s="17" t="s">
         <v>274</v>
@@ -7330,11 +7329,11 @@
         <v>17</v>
       </c>
       <c r="E213" s="17" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F213" s="17"/>
       <c r="G213" s="6" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="I213" s="6" t="s">
         <v>266</v>
@@ -7345,7 +7344,7 @@
     </row>
     <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="6" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B214" s="17" t="s">
         <v>274</v>
@@ -7354,14 +7353,14 @@
         <v>11</v>
       </c>
       <c r="D214" s="17" t="s">
-        <v>315</v>
+        <v>17</v>
       </c>
       <c r="E214" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F214" s="17"/>
       <c r="G214" s="6" t="n">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="I214" s="6" t="s">
         <v>266</v>
@@ -7372,32 +7371,34 @@
     </row>
     <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="6" t="n">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B215" s="17" t="s">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="C215" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D215" s="17"/>
+      <c r="D215" s="17" t="s">
+        <v>315</v>
+      </c>
       <c r="E215" s="17" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F215" s="17"/>
       <c r="G215" s="6" t="n">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="I215" s="6" t="s">
-        <v>318</v>
+        <v>266</v>
       </c>
       <c r="J215" s="6" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="6" t="n">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B216" s="17" t="s">
         <v>80</v>
@@ -7407,11 +7408,11 @@
       </c>
       <c r="D216" s="17"/>
       <c r="E216" s="17" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F216" s="17"/>
       <c r="G216" s="6" t="n">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="I216" s="6" t="s">
         <v>318</v>
@@ -7422,7 +7423,7 @@
     </row>
     <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="6" t="n">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B217" s="17" t="s">
         <v>80</v>
@@ -7432,11 +7433,11 @@
       </c>
       <c r="D217" s="17"/>
       <c r="E217" s="17" t="s">
-        <v>321</v>
-      </c>
-      <c r="F217" s="6"/>
+        <v>320</v>
+      </c>
+      <c r="F217" s="17"/>
       <c r="G217" s="6" t="n">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="I217" s="6" t="s">
         <v>318</v>
@@ -7447,7 +7448,7 @@
     </row>
     <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="6" t="n">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B218" s="17" t="s">
         <v>80</v>
@@ -7457,11 +7458,11 @@
       </c>
       <c r="D218" s="17"/>
       <c r="E218" s="17" t="s">
-        <v>77</v>
+        <v>321</v>
       </c>
       <c r="F218" s="6"/>
       <c r="G218" s="6" t="n">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="I218" s="6" t="s">
         <v>318</v>
@@ -7472,7 +7473,7 @@
     </row>
     <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="6" t="n">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B219" s="17" t="s">
         <v>80</v>
@@ -7486,7 +7487,7 @@
       </c>
       <c r="F219" s="6"/>
       <c r="G219" s="6" t="n">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="I219" s="6" t="s">
         <v>318</v>
@@ -7497,7 +7498,7 @@
     </row>
     <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="6" t="n">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B220" s="17" t="s">
         <v>80</v>
@@ -7507,22 +7508,22 @@
       </c>
       <c r="D220" s="17"/>
       <c r="E220" s="17" t="s">
-        <v>322</v>
+        <v>77</v>
       </c>
       <c r="F220" s="6"/>
       <c r="G220" s="6" t="n">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="I220" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J220" s="6" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="6" t="n">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B221" s="17" t="s">
         <v>80</v>
@@ -7531,12 +7532,12 @@
         <v>11</v>
       </c>
       <c r="D221" s="17"/>
-      <c r="E221" s="6" t="s">
-        <v>324</v>
+      <c r="E221" s="17" t="s">
+        <v>322</v>
       </c>
       <c r="F221" s="6"/>
       <c r="G221" s="6" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="I221" s="6" t="s">
         <v>318</v>
@@ -7547,7 +7548,7 @@
     </row>
     <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="6" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B222" s="17" t="s">
         <v>80</v>
@@ -7557,39 +7558,36 @@
       </c>
       <c r="D222" s="17"/>
       <c r="E222" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F222" s="6"/>
       <c r="G222" s="6" t="n">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="I222" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J222" s="6" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="6" t="n">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B223" s="17" t="s">
-        <v>281</v>
+        <v>80</v>
       </c>
       <c r="C223" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D223" s="17"/>
-      <c r="E223" s="17" t="s">
-        <v>282</v>
+      <c r="E223" s="6" t="s">
+        <v>325</v>
       </c>
       <c r="F223" s="6"/>
       <c r="G223" s="6" t="n">
-        <v>511</v>
-      </c>
-      <c r="H223" s="6" t="n">
-        <v>-10</v>
+        <v>566</v>
       </c>
       <c r="I223" s="6" t="s">
         <v>318</v>
@@ -7600,34 +7598,35 @@
     </row>
     <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="6" t="n">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="B224" s="17" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C224" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D224" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D224" s="17"/>
       <c r="E224" s="17" t="s">
-        <v>275</v>
-      </c>
-      <c r="F224" s="17"/>
+        <v>282</v>
+      </c>
+      <c r="F224" s="6"/>
       <c r="G224" s="6" t="n">
-        <v>571</v>
+        <v>511</v>
+      </c>
+      <c r="H224" s="6" t="n">
+        <v>-10</v>
       </c>
       <c r="I224" s="6" t="s">
-        <v>266</v>
+        <v>318</v>
       </c>
       <c r="J224" s="6" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="6" t="n">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B225" s="17" t="s">
         <v>274</v>
@@ -7636,14 +7635,14 @@
         <v>11</v>
       </c>
       <c r="D225" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E225" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F225" s="17"/>
       <c r="G225" s="6" t="n">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="I225" s="6" t="s">
         <v>266</v>
@@ -7654,7 +7653,7 @@
     </row>
     <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="6" t="n">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B226" s="17" t="s">
         <v>274</v>
@@ -7663,14 +7662,14 @@
         <v>11</v>
       </c>
       <c r="D226" s="17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E226" s="17" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="F226" s="17"/>
       <c r="G226" s="6" t="n">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I226" s="6" t="s">
         <v>266</v>
@@ -7681,7 +7680,7 @@
     </row>
     <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="6" t="n">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B227" s="17" t="s">
         <v>274</v>
@@ -7693,11 +7692,11 @@
         <v>17</v>
       </c>
       <c r="E227" s="17" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="F227" s="17"/>
       <c r="G227" s="6" t="n">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="I227" s="6" t="s">
         <v>266</v>
@@ -7708,7 +7707,7 @@
     </row>
     <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="6" t="n">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B228" s="17" t="s">
         <v>274</v>
@@ -7720,11 +7719,11 @@
         <v>17</v>
       </c>
       <c r="E228" s="17" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F228" s="17"/>
       <c r="G228" s="6" t="n">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="I228" s="6" t="s">
         <v>266</v>
@@ -7735,7 +7734,7 @@
     </row>
     <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="6" t="n">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B229" s="17" t="s">
         <v>274</v>
@@ -7744,14 +7743,14 @@
         <v>11</v>
       </c>
       <c r="D229" s="17" t="s">
-        <v>315</v>
+        <v>17</v>
       </c>
       <c r="E229" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F229" s="17"/>
       <c r="G229" s="6" t="n">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="I229" s="6" t="s">
         <v>266</v>
@@ -7762,24 +7761,26 @@
     </row>
     <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="6" t="n">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B230" s="17" t="s">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="C230" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D230" s="17"/>
+      <c r="D230" s="17" t="s">
+        <v>315</v>
+      </c>
       <c r="E230" s="17" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="F230" s="17"/>
       <c r="G230" s="6" t="n">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="I230" s="6" t="s">
-        <v>318</v>
+        <v>266</v>
       </c>
       <c r="J230" s="6" t="s">
         <v>312</v>
@@ -7787,7 +7788,7 @@
     </row>
     <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="6" t="n">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B231" s="17" t="s">
         <v>80</v>
@@ -7797,11 +7798,11 @@
       </c>
       <c r="D231" s="17"/>
       <c r="E231" s="17" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F231" s="17"/>
       <c r="G231" s="6" t="n">
-        <v>596</v>
+        <v>577</v>
       </c>
       <c r="I231" s="6" t="s">
         <v>318</v>
@@ -7812,76 +7813,74 @@
     </row>
     <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="6" t="n">
-        <v>580</v>
-      </c>
-      <c r="B232" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="B232" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C232" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D232" s="6"/>
-      <c r="E232" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="F232" s="6" t="s">
-        <v>330</v>
-      </c>
-      <c r="G232" s="6"/>
-      <c r="H232" s="6" t="n">
-        <v>10</v>
+      <c r="C232" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D232" s="17"/>
+      <c r="E232" s="17" t="s">
+        <v>328</v>
+      </c>
+      <c r="F232" s="17"/>
+      <c r="G232" s="6" t="n">
+        <v>596</v>
       </c>
       <c r="I232" s="6" t="s">
-        <v>266</v>
+        <v>318</v>
       </c>
       <c r="J232" s="6" t="s">
-        <v>331</v>
+        <v>312</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="6" t="n">
-        <v>581</v>
-      </c>
-      <c r="B233" s="17" t="s">
+        <v>580</v>
+      </c>
+      <c r="B233" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C233" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D233" s="17"/>
-      <c r="E233" s="17" t="s">
-        <v>301</v>
-      </c>
-      <c r="F233" s="6"/>
-      <c r="G233" s="8" t="n">
-        <v>582</v>
+      <c r="C233" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D233" s="6"/>
+      <c r="E233" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F233" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="G233" s="6"/>
+      <c r="H233" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="I233" s="6" t="s">
         <v>266</v>
       </c>
       <c r="J233" s="6" t="s">
-        <v>331</v>
+        <v>298</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="6" t="n">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B234" s="17" t="s">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="C234" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D234" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D234" s="17"/>
       <c r="E234" s="17" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="F234" s="6"/>
       <c r="G234" s="8" t="n">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="I234" s="6" t="s">
         <v>266</v>
@@ -7892,7 +7891,7 @@
     </row>
     <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="6" t="n">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B235" s="17" t="s">
         <v>274</v>
@@ -7901,14 +7900,14 @@
         <v>11</v>
       </c>
       <c r="D235" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E235" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F235" s="6"/>
       <c r="G235" s="8" t="n">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="I235" s="6" t="s">
         <v>266</v>
@@ -7919,7 +7918,7 @@
     </row>
     <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="6" t="n">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B236" s="17" t="s">
         <v>274</v>
@@ -7928,14 +7927,14 @@
         <v>11</v>
       </c>
       <c r="D236" s="17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E236" s="17" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="F236" s="6"/>
       <c r="G236" s="8" t="n">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="I236" s="6" t="s">
         <v>266</v>
@@ -7946,7 +7945,7 @@
     </row>
     <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="6" t="n">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B237" s="17" t="s">
         <v>274</v>
@@ -7955,14 +7954,14 @@
         <v>11</v>
       </c>
       <c r="D237" s="17" t="s">
-        <v>315</v>
+        <v>17</v>
       </c>
       <c r="E237" s="17" t="s">
-        <v>332</v>
+        <v>303</v>
       </c>
       <c r="F237" s="6"/>
       <c r="G237" s="8" t="n">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="I237" s="6" t="s">
         <v>266</v>
@@ -7973,32 +7972,34 @@
     </row>
     <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="6" t="n">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B238" s="17" t="s">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="C238" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D238" s="17"/>
+      <c r="D238" s="17" t="s">
+        <v>315</v>
+      </c>
       <c r="E238" s="17" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F238" s="6"/>
       <c r="G238" s="8" t="n">
-        <v>560</v>
+        <v>586</v>
       </c>
       <c r="I238" s="6" t="s">
-        <v>318</v>
+        <v>266</v>
       </c>
       <c r="J238" s="6" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="6" t="n">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="B239" s="17" t="s">
         <v>80</v>
@@ -8008,38 +8009,36 @@
       </c>
       <c r="D239" s="17"/>
       <c r="E239" s="17" t="s">
-        <v>301</v>
+        <v>333</v>
       </c>
       <c r="F239" s="6"/>
       <c r="G239" s="8" t="n">
-        <v>591</v>
+        <v>560</v>
       </c>
       <c r="I239" s="6" t="s">
-        <v>266</v>
+        <v>318</v>
       </c>
       <c r="J239" s="6" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="6" t="n">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B240" s="17" t="s">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="C240" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D240" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D240" s="17"/>
       <c r="E240" s="17" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="F240" s="6"/>
       <c r="G240" s="8" t="n">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="I240" s="6" t="s">
         <v>266</v>
@@ -8050,7 +8049,7 @@
     </row>
     <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A241" s="6" t="n">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B241" s="17" t="s">
         <v>274</v>
@@ -8059,14 +8058,14 @@
         <v>11</v>
       </c>
       <c r="D241" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E241" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F241" s="6"/>
       <c r="G241" s="8" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="I241" s="6" t="s">
         <v>266</v>
@@ -8077,7 +8076,7 @@
     </row>
     <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A242" s="6" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B242" s="17" t="s">
         <v>274</v>
@@ -8086,14 +8085,14 @@
         <v>11</v>
       </c>
       <c r="D242" s="17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E242" s="17" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="F242" s="6"/>
       <c r="G242" s="8" t="n">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="I242" s="6" t="s">
         <v>266</v>
@@ -8104,7 +8103,7 @@
     </row>
     <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A243" s="6" t="n">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B243" s="17" t="s">
         <v>274</v>
@@ -8113,14 +8112,14 @@
         <v>11</v>
       </c>
       <c r="D243" s="17" t="s">
-        <v>315</v>
+        <v>17</v>
       </c>
       <c r="E243" s="17" t="s">
-        <v>332</v>
+        <v>303</v>
       </c>
       <c r="F243" s="6"/>
       <c r="G243" s="8" t="n">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="I243" s="6" t="s">
         <v>266</v>
@@ -8131,32 +8130,34 @@
     </row>
     <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A244" s="6" t="n">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B244" s="17" t="s">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="C244" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D244" s="17"/>
+      <c r="D244" s="17" t="s">
+        <v>315</v>
+      </c>
       <c r="E244" s="17" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F244" s="6"/>
       <c r="G244" s="8" t="n">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="I244" s="6" t="s">
-        <v>318</v>
+        <v>266</v>
       </c>
       <c r="J244" s="6" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A245" s="6" t="n">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B245" s="17" t="s">
         <v>80</v>
@@ -8166,11 +8167,11 @@
       </c>
       <c r="D245" s="17"/>
       <c r="E245" s="17" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F245" s="6"/>
       <c r="G245" s="8" t="n">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="I245" s="6" t="s">
         <v>318</v>
@@ -8181,7 +8182,7 @@
     </row>
     <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A246" s="6" t="n">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B246" s="17" t="s">
         <v>80</v>
@@ -8191,22 +8192,22 @@
       </c>
       <c r="D246" s="17"/>
       <c r="E246" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="F246" s="17"/>
+        <v>334</v>
+      </c>
+      <c r="F246" s="6"/>
       <c r="G246" s="8" t="n">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="I246" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J246" s="6" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A247" s="6" t="n">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B247" s="17" t="s">
         <v>80</v>
@@ -8218,20 +8219,20 @@
       <c r="E247" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="F247" s="6"/>
+      <c r="F247" s="17"/>
       <c r="G247" s="8" t="n">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="I247" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J247" s="6" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A248" s="6" t="n">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B248" s="17" t="s">
         <v>80</v>
@@ -8241,22 +8242,22 @@
       </c>
       <c r="D248" s="17"/>
       <c r="E248" s="17" t="s">
-        <v>336</v>
+        <v>77</v>
       </c>
       <c r="F248" s="6"/>
       <c r="G248" s="8" t="n">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="I248" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J248" s="6" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A249" s="6" t="n">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B249" s="17" t="s">
         <v>80</v>
@@ -8266,11 +8267,11 @@
       </c>
       <c r="D249" s="17"/>
       <c r="E249" s="17" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F249" s="6"/>
       <c r="G249" s="8" t="n">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="I249" s="6" t="s">
         <v>318</v>
@@ -8281,22 +8282,22 @@
     </row>
     <row r="250" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A250" s="6" t="n">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B250" s="17" t="s">
         <v>80</v>
       </c>
       <c r="C250" s="17" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D250" s="17"/>
       <c r="E250" s="17" t="s">
-        <v>339</v>
-      </c>
-      <c r="F250" s="6" t="s">
-        <v>340</v>
-      </c>
-      <c r="G250" s="8"/>
+        <v>338</v>
+      </c>
+      <c r="F250" s="6"/>
+      <c r="G250" s="8" t="n">
+        <v>601</v>
+      </c>
       <c r="I250" s="6" t="s">
         <v>318</v>
       </c>
@@ -8306,22 +8307,22 @@
     </row>
     <row r="251" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A251" s="6" t="n">
-        <v>602</v>
-      </c>
-      <c r="B251" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="B251" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C251" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D251" s="6"/>
-      <c r="E251" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="F251" s="6"/>
-      <c r="G251" s="8" t="n">
-        <v>601</v>
-      </c>
+      <c r="C251" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D251" s="17"/>
+      <c r="E251" s="17" t="s">
+        <v>339</v>
+      </c>
+      <c r="F251" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="G251" s="8"/>
       <c r="I251" s="6" t="s">
         <v>318</v>
       </c>
@@ -8331,7 +8332,7 @@
     </row>
     <row r="252" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A252" s="6" t="n">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B252" s="6" t="s">
         <v>80</v>
@@ -8341,22 +8342,22 @@
       </c>
       <c r="D252" s="6"/>
       <c r="E252" s="6" t="s">
-        <v>342</v>
-      </c>
-      <c r="F252" s="17"/>
+        <v>341</v>
+      </c>
+      <c r="F252" s="6"/>
       <c r="G252" s="8" t="n">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="I252" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J252" s="6" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A253" s="6" t="n">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B253" s="6" t="s">
         <v>80</v>
@@ -8366,11 +8367,11 @@
       </c>
       <c r="D253" s="6"/>
       <c r="E253" s="6" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F253" s="17"/>
       <c r="G253" s="8" t="n">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="I253" s="6" t="s">
         <v>318</v>
@@ -8381,7 +8382,7 @@
     </row>
     <row r="254" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="6" t="n">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B254" s="6" t="s">
         <v>80</v>
@@ -8391,11 +8392,11 @@
       </c>
       <c r="D254" s="6"/>
       <c r="E254" s="6" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F254" s="17"/>
       <c r="G254" s="8" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="I254" s="6" t="s">
         <v>318</v>
@@ -8406,7 +8407,7 @@
     </row>
     <row r="255" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="6" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B255" s="6" t="s">
         <v>80</v>
@@ -8416,37 +8417,37 @@
       </c>
       <c r="D255" s="6"/>
       <c r="E255" s="6" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F255" s="17"/>
       <c r="G255" s="8" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="I255" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J255" s="6" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A256" s="6" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B256" s="6" t="s">
         <v>80</v>
       </c>
       <c r="C256" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D256" s="6"/>
       <c r="E256" s="6" t="s">
-        <v>347</v>
-      </c>
-      <c r="F256" s="17" t="s">
-        <v>348</v>
-      </c>
-      <c r="G256" s="8"/>
+        <v>346</v>
+      </c>
+      <c r="F256" s="17"/>
+      <c r="G256" s="8" t="n">
+        <v>607</v>
+      </c>
       <c r="I256" s="6" t="s">
         <v>318</v>
       </c>
@@ -8456,25 +8457,22 @@
     </row>
     <row r="257" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A257" s="6" t="n">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B257" s="6" t="s">
         <v>80</v>
       </c>
       <c r="C257" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D257" s="6"/>
       <c r="E257" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="F257" s="17"/>
-      <c r="G257" s="8" t="n">
-        <v>607</v>
-      </c>
-      <c r="H257" s="6" t="n">
-        <v>-2</v>
-      </c>
+        <v>347</v>
+      </c>
+      <c r="F257" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="G257" s="8"/>
       <c r="I257" s="6" t="s">
         <v>318</v>
       </c>
@@ -8484,7 +8482,7 @@
     </row>
     <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A258" s="6" t="n">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B258" s="6" t="s">
         <v>80</v>
@@ -8494,11 +8492,14 @@
       </c>
       <c r="D258" s="6"/>
       <c r="E258" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F258" s="17"/>
       <c r="G258" s="8" t="n">
-        <v>610</v>
+        <v>607</v>
+      </c>
+      <c r="H258" s="6" t="n">
+        <v>-2</v>
       </c>
       <c r="I258" s="6" t="s">
         <v>318</v>
@@ -8509,22 +8510,22 @@
     </row>
     <row r="259" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A259" s="6" t="n">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B259" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C259" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="D259" s="17"/>
-      <c r="E259" s="17" t="s">
-        <v>351</v>
-      </c>
-      <c r="F259" s="17" t="s">
-        <v>352</v>
-      </c>
-      <c r="G259" s="8"/>
+      <c r="C259" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D259" s="6"/>
+      <c r="E259" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="F259" s="17"/>
+      <c r="G259" s="8" t="n">
+        <v>610</v>
+      </c>
       <c r="I259" s="6" t="s">
         <v>318</v>
       </c>
@@ -8534,34 +8535,32 @@
     </row>
     <row r="260" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A260" s="6" t="n">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="B260" s="6" t="s">
-        <v>353</v>
+        <v>80</v>
       </c>
       <c r="C260" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D260" s="17" t="s">
-        <v>17</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D260" s="17"/>
       <c r="E260" s="17" t="s">
-        <v>354</v>
-      </c>
-      <c r="F260" s="17"/>
-      <c r="G260" s="8" t="n">
-        <v>621</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="F260" s="17" t="s">
+        <v>352</v>
+      </c>
+      <c r="G260" s="8"/>
       <c r="I260" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J260" s="6" t="s">
-        <v>355</v>
+        <v>337</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A261" s="6" t="n">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B261" s="6" t="s">
         <v>353</v>
@@ -8570,14 +8569,14 @@
         <v>11</v>
       </c>
       <c r="D261" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E261" s="6" t="s">
-        <v>356</v>
+        <v>17</v>
+      </c>
+      <c r="E261" s="17" t="s">
+        <v>354</v>
       </c>
       <c r="F261" s="17"/>
       <c r="G261" s="8" t="n">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="I261" s="6" t="s">
         <v>318</v>
@@ -8588,7 +8587,7 @@
     </row>
     <row r="262" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A262" s="6" t="n">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B262" s="6" t="s">
         <v>353</v>
@@ -8597,14 +8596,14 @@
         <v>11</v>
       </c>
       <c r="D262" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E262" s="17" t="s">
-        <v>357</v>
+        <v>32</v>
+      </c>
+      <c r="E262" s="6" t="s">
+        <v>356</v>
       </c>
       <c r="F262" s="17"/>
       <c r="G262" s="8" t="n">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="I262" s="6" t="s">
         <v>318</v>
@@ -8615,7 +8614,7 @@
     </row>
     <row r="263" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A263" s="6" t="n">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B263" s="6" t="s">
         <v>353</v>
@@ -8624,14 +8623,14 @@
         <v>11</v>
       </c>
       <c r="D263" s="17" t="s">
-        <v>358</v>
+        <v>17</v>
       </c>
       <c r="E263" s="17" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F263" s="17"/>
       <c r="G263" s="8" t="n">
-        <v>634</v>
+        <v>623</v>
       </c>
       <c r="I263" s="6" t="s">
         <v>318</v>
@@ -8641,8 +8640,8 @@
       </c>
     </row>
     <row r="264" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A264" s="7" t="n">
-        <v>630</v>
+      <c r="A264" s="6" t="n">
+        <v>623</v>
       </c>
       <c r="B264" s="6" t="s">
         <v>353</v>
@@ -8651,25 +8650,25 @@
         <v>11</v>
       </c>
       <c r="D264" s="17" t="s">
-        <v>17</v>
+        <v>358</v>
       </c>
       <c r="E264" s="17" t="s">
-        <v>354</v>
-      </c>
-      <c r="F264" s="6"/>
+        <v>359</v>
+      </c>
+      <c r="F264" s="17"/>
       <c r="G264" s="8" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="I264" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J264" s="6" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A265" s="7" t="n">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B265" s="6" t="s">
         <v>353</v>
@@ -8678,14 +8677,14 @@
         <v>11</v>
       </c>
       <c r="D265" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E265" s="6" t="s">
-        <v>356</v>
-      </c>
-      <c r="F265" s="17"/>
+        <v>17</v>
+      </c>
+      <c r="E265" s="17" t="s">
+        <v>354</v>
+      </c>
+      <c r="F265" s="6"/>
       <c r="G265" s="8" t="n">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="I265" s="6" t="s">
         <v>318</v>
@@ -8696,7 +8695,7 @@
     </row>
     <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A266" s="7" t="n">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B266" s="6" t="s">
         <v>353</v>
@@ -8705,14 +8704,14 @@
         <v>11</v>
       </c>
       <c r="D266" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E266" s="17" t="s">
-        <v>361</v>
+        <v>32</v>
+      </c>
+      <c r="E266" s="6" t="s">
+        <v>356</v>
       </c>
       <c r="F266" s="17"/>
       <c r="G266" s="8" t="n">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="I266" s="6" t="s">
         <v>318</v>
@@ -8723,7 +8722,7 @@
     </row>
     <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A267" s="7" t="n">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B267" s="6" t="s">
         <v>353</v>
@@ -8732,14 +8731,14 @@
         <v>11</v>
       </c>
       <c r="D267" s="17" t="s">
-        <v>358</v>
+        <v>17</v>
       </c>
       <c r="E267" s="17" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F267" s="17"/>
       <c r="G267" s="8" t="n">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="I267" s="6" t="s">
         <v>318</v>
@@ -8750,49 +8749,51 @@
     </row>
     <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A268" s="7" t="n">
-        <v>634</v>
-      </c>
-      <c r="B268" s="17" t="s">
-        <v>281</v>
+        <v>633</v>
+      </c>
+      <c r="B268" s="6" t="s">
+        <v>353</v>
       </c>
       <c r="C268" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D268" s="17"/>
+      <c r="D268" s="17" t="s">
+        <v>358</v>
+      </c>
       <c r="E268" s="17" t="s">
-        <v>282</v>
+        <v>362</v>
       </c>
       <c r="F268" s="17"/>
       <c r="G268" s="8" t="n">
-        <v>635</v>
-      </c>
-      <c r="H268" s="6" t="n">
-        <v>-10</v>
+        <v>634</v>
       </c>
       <c r="I268" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J268" s="6" t="s">
-        <v>283</v>
+        <v>360</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A269" s="7" t="n">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B269" s="17" t="s">
-        <v>80</v>
+        <v>281</v>
       </c>
       <c r="C269" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D269" s="17"/>
       <c r="E269" s="17" t="s">
-        <v>363</v>
+        <v>282</v>
       </c>
       <c r="F269" s="17"/>
       <c r="G269" s="8" t="n">
-        <v>511</v>
+        <v>635</v>
+      </c>
+      <c r="H269" s="6" t="n">
+        <v>-10</v>
       </c>
       <c r="I269" s="6" t="s">
         <v>318</v>
@@ -8803,34 +8804,32 @@
     </row>
     <row r="270" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A270" s="7" t="n">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="B270" s="17" t="s">
-        <v>353</v>
+        <v>80</v>
       </c>
       <c r="C270" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D270" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D270" s="17"/>
       <c r="E270" s="17" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="F270" s="17"/>
       <c r="G270" s="8" t="n">
-        <v>641</v>
+        <v>511</v>
       </c>
       <c r="I270" s="6" t="s">
         <v>318</v>
       </c>
       <c r="J270" s="6" t="s">
-        <v>364</v>
+        <v>283</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A271" s="7" t="n">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B271" s="17" t="s">
         <v>353</v>
@@ -8839,14 +8838,14 @@
         <v>11</v>
       </c>
       <c r="D271" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E271" s="6" t="s">
-        <v>356</v>
+        <v>17</v>
+      </c>
+      <c r="E271" s="17" t="s">
+        <v>354</v>
       </c>
       <c r="F271" s="17"/>
       <c r="G271" s="8" t="n">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="I271" s="6" t="s">
         <v>318</v>
@@ -8857,7 +8856,7 @@
     </row>
     <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A272" s="7" t="n">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B272" s="17" t="s">
         <v>353</v>
@@ -8866,14 +8865,14 @@
         <v>11</v>
       </c>
       <c r="D272" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E272" s="17" t="s">
-        <v>365</v>
+        <v>32</v>
+      </c>
+      <c r="E272" s="6" t="s">
+        <v>356</v>
       </c>
       <c r="F272" s="17"/>
       <c r="G272" s="8" t="n">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="I272" s="6" t="s">
         <v>318</v>
@@ -8884,7 +8883,7 @@
     </row>
     <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A273" s="7" t="n">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B273" s="17" t="s">
         <v>353</v>
@@ -8896,11 +8895,11 @@
         <v>17</v>
       </c>
       <c r="E273" s="17" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F273" s="17"/>
       <c r="G273" s="8" t="n">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I273" s="6" t="s">
         <v>318</v>
@@ -8911,7 +8910,7 @@
     </row>
     <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A274" s="7" t="n">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B274" s="17" t="s">
         <v>353</v>
@@ -8920,14 +8919,14 @@
         <v>11</v>
       </c>
       <c r="D274" s="17" t="s">
-        <v>367</v>
+        <v>17</v>
       </c>
       <c r="E274" s="17" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="F274" s="17"/>
       <c r="G274" s="8" t="n">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="I274" s="6" t="s">
         <v>318</v>
@@ -8938,78 +8937,78 @@
     </row>
     <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A275" s="7" t="n">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B275" s="17" t="s">
-        <v>80</v>
+        <v>353</v>
       </c>
       <c r="C275" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D275" s="17"/>
+      <c r="D275" s="17" t="s">
+        <v>367</v>
+      </c>
       <c r="E275" s="17" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F275" s="17"/>
       <c r="G275" s="8" t="n">
-        <v>750</v>
-      </c>
-      <c r="H275" s="6" t="n">
-        <v>10</v>
+        <v>645</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>370</v>
+        <v>318</v>
       </c>
       <c r="J275" s="6" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A276" s="7" t="n">
-        <v>700</v>
+        <v>645</v>
       </c>
       <c r="B276" s="17" t="s">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="C276" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D276" s="17" t="s">
-        <v>17</v>
-      </c>
+      <c r="D276" s="17"/>
       <c r="E276" s="17" t="s">
-        <v>77</v>
+        <v>369</v>
       </c>
       <c r="F276" s="17"/>
       <c r="G276" s="8" t="n">
-        <v>701</v>
+        <v>750</v>
+      </c>
+      <c r="H276" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="I276" s="6" t="s">
-        <v>14</v>
+        <v>370</v>
       </c>
       <c r="J276" s="6" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A277" s="7" t="n">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B277" s="17" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C277" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D277" s="17" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E277" s="17" t="s">
-        <v>373</v>
+        <v>77</v>
       </c>
       <c r="F277" s="17"/>
       <c r="G277" s="8" t="n">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="I277" s="6" t="s">
         <v>14</v>
@@ -9020,23 +9019,23 @@
     </row>
     <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A278" s="7" t="n">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B278" s="17" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C278" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D278" s="17" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E278" s="17" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F278" s="17"/>
       <c r="G278" s="8" t="n">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>14</v>
@@ -9047,7 +9046,7 @@
     </row>
     <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A279" s="7" t="n">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="B279" s="17" t="s">
         <v>10</v>
@@ -9056,14 +9055,14 @@
         <v>11</v>
       </c>
       <c r="D279" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="E279" s="6" t="s">
-        <v>375</v>
+        <v>26</v>
+      </c>
+      <c r="E279" s="17" t="s">
+        <v>374</v>
       </c>
       <c r="F279" s="17"/>
       <c r="G279" s="8" t="n">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>14</v>
@@ -9074,26 +9073,23 @@
     </row>
     <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A280" s="7" t="n">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B280" s="17" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C280" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D280" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E280" s="17" t="s">
-        <v>376</v>
+        <v>24</v>
+      </c>
+      <c r="E280" s="6" t="s">
+        <v>375</v>
       </c>
       <c r="F280" s="17"/>
       <c r="G280" s="8" t="n">
-        <v>760</v>
-      </c>
-      <c r="H280" s="6" t="n">
-        <v>-20</v>
+        <v>704</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>14</v>
@@ -9104,10 +9100,10 @@
     </row>
     <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A281" s="7" t="n">
-        <v>750</v>
+        <v>704</v>
       </c>
       <c r="B281" s="17" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C281" s="17" t="s">
         <v>11</v>
@@ -9116,11 +9112,14 @@
         <v>17</v>
       </c>
       <c r="E281" s="17" t="s">
-        <v>77</v>
+        <v>376</v>
       </c>
       <c r="F281" s="17"/>
       <c r="G281" s="8" t="n">
-        <v>751</v>
+        <v>760</v>
+      </c>
+      <c r="H281" s="6" t="n">
+        <v>-20</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>14</v>
@@ -9131,7 +9130,7 @@
     </row>
     <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A282" s="7" t="n">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B282" s="17" t="s">
         <v>10</v>
@@ -9140,14 +9139,14 @@
         <v>11</v>
       </c>
       <c r="D282" s="17" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E282" s="17" t="s">
-        <v>377</v>
+        <v>77</v>
       </c>
       <c r="F282" s="17"/>
       <c r="G282" s="8" t="n">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="I282" s="6" t="s">
         <v>14</v>
@@ -9158,34 +9157,34 @@
     </row>
     <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="n">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B283" s="17" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C283" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D283" s="17" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="E283" s="17" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F283" s="17"/>
       <c r="G283" s="8" t="n">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="I283" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J283" s="6" t="s">
-        <v>15</v>
+        <v>372</v>
       </c>
     </row>
     <row r="284" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A284" s="7" t="n">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B284" s="17" t="s">
         <v>31</v>
@@ -9194,25 +9193,25 @@
         <v>11</v>
       </c>
       <c r="D284" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E284" s="6" t="s">
-        <v>379</v>
+        <v>51</v>
+      </c>
+      <c r="E284" s="17" t="s">
+        <v>378</v>
       </c>
       <c r="F284" s="17"/>
       <c r="G284" s="8" t="n">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="I284" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J284" s="6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A285" s="7" t="n">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B285" s="17" t="s">
         <v>31</v>
@@ -9221,14 +9220,14 @@
         <v>11</v>
       </c>
       <c r="D285" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E285" s="17" t="s">
-        <v>380</v>
+        <v>17</v>
+      </c>
+      <c r="E285" s="6" t="s">
+        <v>379</v>
       </c>
       <c r="F285" s="17"/>
       <c r="G285" s="8" t="n">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="I285" s="6" t="s">
         <v>14</v>
@@ -9239,34 +9238,34 @@
     </row>
     <row r="286" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A286" s="7" t="n">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B286" s="17" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C286" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D286" s="17" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E286" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F286" s="17"/>
       <c r="G286" s="8" t="n">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="I286" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J286" s="6" t="s">
-        <v>382</v>
+        <v>20</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A287" s="7" t="n">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B287" s="17" t="s">
         <v>10</v>
@@ -9275,14 +9274,14 @@
         <v>11</v>
       </c>
       <c r="D287" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E287" s="6" t="s">
-        <v>383</v>
+        <v>24</v>
+      </c>
+      <c r="E287" s="17" t="s">
+        <v>381</v>
       </c>
       <c r="F287" s="17"/>
       <c r="G287" s="8" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="I287" s="6" t="s">
         <v>14</v>
@@ -9293,26 +9292,23 @@
     </row>
     <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A288" s="7" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B288" s="17" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C288" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D288" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="E288" s="17" t="s">
-        <v>384</v>
+        <v>12</v>
+      </c>
+      <c r="E288" s="6" t="s">
+        <v>383</v>
       </c>
       <c r="F288" s="17"/>
       <c r="G288" s="8" t="n">
-        <v>760</v>
-      </c>
-      <c r="H288" s="6" t="n">
-        <v>30</v>
+        <v>757</v>
       </c>
       <c r="I288" s="6" t="s">
         <v>14</v>
@@ -9323,35 +9319,56 @@
     </row>
     <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A289" s="7" t="n">
+        <v>757</v>
+      </c>
+      <c r="B289" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C289" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D289" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E289" s="17" t="s">
+        <v>384</v>
+      </c>
+      <c r="F289" s="17"/>
+      <c r="G289" s="8" t="n">
         <v>760</v>
       </c>
-      <c r="B289" s="17" t="s">
-        <v>281</v>
-      </c>
-      <c r="C289" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D289" s="17"/>
-      <c r="E289" s="17" t="s">
-        <v>385</v>
-      </c>
-      <c r="F289" s="17"/>
-      <c r="G289" s="8"/>
+      <c r="H289" s="6" t="n">
+        <v>30</v>
+      </c>
       <c r="I289" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J289" s="6" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
     <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A290" s="7"/>
-      <c r="B290" s="17"/>
-      <c r="C290" s="17"/>
+      <c r="A290" s="7" t="n">
+        <v>760</v>
+      </c>
+      <c r="B290" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="C290" s="17" t="s">
+        <v>11</v>
+      </c>
       <c r="D290" s="17"/>
-      <c r="E290" s="17"/>
+      <c r="E290" s="17" t="s">
+        <v>385</v>
+      </c>
       <c r="F290" s="17"/>
       <c r="G290" s="8"/>
+      <c r="I290" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J290" s="6" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="291" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A291" s="7"/>
@@ -15751,6 +15768,15 @@
       <c r="E1001" s="17"/>
       <c r="F1001" s="17"/>
       <c r="G1001" s="8"/>
+    </row>
+    <row r="1002" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1002" s="7"/>
+      <c r="B1002" s="17"/>
+      <c r="C1002" s="17"/>
+      <c r="D1002" s="17"/>
+      <c r="E1002" s="17"/>
+      <c r="F1002" s="17"/>
+      <c r="G1002" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
PC world and end
</commit_message>
<xml_diff>
--- a/resources/data/dialogue.xlsx
+++ b/resources/data/dialogue.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="388">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1109,6 +1109,9 @@
   </si>
   <si>
     <t xml:space="preserve">So, you may not leave this system!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">game-over/quarantined-network</t>
   </si>
   <si>
     <t xml:space="preserve">Hm… I need to outsmart Velos, the Data Leakage Protection.</t>
@@ -8799,7 +8802,7 @@
         <v>318</v>
       </c>
       <c r="J269" s="6" t="s">
-        <v>283</v>
+        <v>363</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8814,7 +8817,7 @@
       </c>
       <c r="D270" s="17"/>
       <c r="E270" s="17" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F270" s="17"/>
       <c r="G270" s="8" t="n">
@@ -8824,7 +8827,7 @@
         <v>318</v>
       </c>
       <c r="J270" s="6" t="s">
-        <v>283</v>
+        <v>363</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8851,7 +8854,7 @@
         <v>318</v>
       </c>
       <c r="J271" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8878,7 +8881,7 @@
         <v>318</v>
       </c>
       <c r="J272" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8895,7 +8898,7 @@
         <v>17</v>
       </c>
       <c r="E273" s="17" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F273" s="17"/>
       <c r="G273" s="8" t="n">
@@ -8905,7 +8908,7 @@
         <v>318</v>
       </c>
       <c r="J273" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8922,7 +8925,7 @@
         <v>17</v>
       </c>
       <c r="E274" s="17" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F274" s="17"/>
       <c r="G274" s="8" t="n">
@@ -8932,7 +8935,7 @@
         <v>318</v>
       </c>
       <c r="J274" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8946,10 +8949,10 @@
         <v>11</v>
       </c>
       <c r="D275" s="17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E275" s="17" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F275" s="17"/>
       <c r="G275" s="8" t="n">
@@ -8959,7 +8962,7 @@
         <v>318</v>
       </c>
       <c r="J275" s="6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8974,7 +8977,7 @@
       </c>
       <c r="D276" s="17"/>
       <c r="E276" s="17" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F276" s="17"/>
       <c r="G276" s="8" t="n">
@@ -8984,10 +8987,10 @@
         <v>10</v>
       </c>
       <c r="I276" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J276" s="6" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9014,7 +9017,7 @@
         <v>14</v>
       </c>
       <c r="J277" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9031,7 +9034,7 @@
         <v>32</v>
       </c>
       <c r="E278" s="17" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F278" s="17"/>
       <c r="G278" s="8" t="n">
@@ -9041,7 +9044,7 @@
         <v>14</v>
       </c>
       <c r="J278" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9058,7 +9061,7 @@
         <v>26</v>
       </c>
       <c r="E279" s="17" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F279" s="17"/>
       <c r="G279" s="8" t="n">
@@ -9068,7 +9071,7 @@
         <v>14</v>
       </c>
       <c r="J279" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9085,7 +9088,7 @@
         <v>24</v>
       </c>
       <c r="E280" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F280" s="17"/>
       <c r="G280" s="8" t="n">
@@ -9095,7 +9098,7 @@
         <v>14</v>
       </c>
       <c r="J280" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9112,7 +9115,7 @@
         <v>17</v>
       </c>
       <c r="E281" s="17" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F281" s="17"/>
       <c r="G281" s="8" t="n">
@@ -9125,7 +9128,7 @@
         <v>14</v>
       </c>
       <c r="J281" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9152,7 +9155,7 @@
         <v>14</v>
       </c>
       <c r="J282" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9169,7 +9172,7 @@
         <v>26</v>
       </c>
       <c r="E283" s="17" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F283" s="17"/>
       <c r="G283" s="8" t="n">
@@ -9179,7 +9182,7 @@
         <v>14</v>
       </c>
       <c r="J283" s="6" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="284" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9196,7 +9199,7 @@
         <v>51</v>
       </c>
       <c r="E284" s="17" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F284" s="17"/>
       <c r="G284" s="8" t="n">
@@ -9223,7 +9226,7 @@
         <v>17</v>
       </c>
       <c r="E285" s="6" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F285" s="17"/>
       <c r="G285" s="8" t="n">
@@ -9250,7 +9253,7 @@
         <v>32</v>
       </c>
       <c r="E286" s="17" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F286" s="17"/>
       <c r="G286" s="8" t="n">
@@ -9277,7 +9280,7 @@
         <v>24</v>
       </c>
       <c r="E287" s="17" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F287" s="17"/>
       <c r="G287" s="8" t="n">
@@ -9287,7 +9290,7 @@
         <v>14</v>
       </c>
       <c r="J287" s="6" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9304,7 +9307,7 @@
         <v>12</v>
       </c>
       <c r="E288" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F288" s="17"/>
       <c r="G288" s="8" t="n">
@@ -9314,7 +9317,7 @@
         <v>14</v>
       </c>
       <c r="J288" s="6" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9331,7 +9334,7 @@
         <v>51</v>
       </c>
       <c r="E289" s="17" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F289" s="17"/>
       <c r="G289" s="8" t="n">
@@ -9344,7 +9347,7 @@
         <v>14</v>
       </c>
       <c r="J289" s="6" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9359,7 +9362,7 @@
       </c>
       <c r="D290" s="17"/>
       <c r="E290" s="17" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F290" s="17"/>
       <c r="G290" s="8"/>
@@ -9367,7 +9370,7 @@
         <v>14</v>
       </c>
       <c r="J290" s="6" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="291" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>